<commit_message>
Creation of Legiscan processor obj
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z3"/>
+  <dimension ref="A1:Z2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -563,164 +563,146 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No State Info - Error: Error processing URL: not enough values to unpack (expected 14, got 2)</t>
+          <t>AK</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>No Title Info - URL: https://legiscan.com/WA/bill/HB1725/2021</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
+          <t>Missing/murdered Indigenous People;report</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>SB151</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Senate</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2024-10-09 - S: EFFECTIVE DATE(S) OF LAW 1/1/25</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://legiscan.com/AK/bill/SB151/2023</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>https://legiscan.com/AK/text/SB151/id/3007736</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>The text outlines Alaska's SB 151, which establishes a Missing and Murdered Indigenous Persons Review Commission and mandates specific training for police officers concerning cases of missing and murdered indigenous persons. Key provisions include amending police training requirements to include cultural training related to these issues, the creation of dedicated investigators within the Department of Public Safety, and directives for the commission to report on unresolved cases and analyze trends. The act also mandates conducting a needs assessment to enhance investigative resources and outlines transitional provisions for current police officers and commission members. The law is set to take effect on January 1, 2025, with some sections expiring on January 1, 2027.</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>The benefits of Enrolled SB 151 include:
+1. **Enhanced Law Enforcement Training**: The legislation mandates at least 12 hours of training on domestic violence and sexual assault for police officers, ensuring they are better prepared to handle sensitive cases, particularly those involving Indigenous persons.
+2. **Creation of the Missing and Murdered Indigenous Persons Review Commission**: This commission aims to systematically address and review unresolved cases, providing a focused oversight mechanism to enhance justice for Indigenous communities.
+3. **Improved Data Collection and Reporting**: The act stipulates that missing person reports must be submitted to a national database within a specified time frame, which enhances tracking and accountability.
+4. **Increased Community Engagement**: By requiring liaisons to be established between law enforcement and federally recognized tribes, the law fosters collaboration and communication, potentially leading to more effective responses to cases involving missing and murdered Indigenous persons.
+5. **Long-term Assessments and Recommendations**: The act includes provisions for the commission to conduct reviews and report findings every three years, ensuring ongoing evaluation and potential policy improvements based on the evolving needs of the community. 
+6. **Support for Indigenous Cultural Training**: The inclusion of cultural training supervised by Indigenous entities promotes understanding and sensitivity among law enforcement officers towards the unique challenges faced by Indigenous communities.</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>The drawbacks of Enrolled SB 151 include:
+1. **Limited Direct Input from Relatives and Survivors**: While the commission includes members from victim advocacy organizations, direct representation from the relatives of missing and murdered Indigenous persons is not specified, potentially leading to gaps in addressing their specific needs and concerns.
+2. **Confidentiality Constraints**: The stipulation that documents and materials reviewed by the commission are confidential may limit transparency and community engagement, as families and tribes may feel excluded from the processes that directly impact them.
+3. **Potential Bureaucratic Delays**: The requirement for a needs assessment and the structured process for reporting may lead to bureaucratic delays, potentially hindering timely responses to cases involving missing and murdered Indigenous persons.
+4. **Dependence on State Resources**: The effectiveness of the commission relies on the State Department of Public Safety’s resources and commitment, which may vary, potentially affecting the commission's ability to carry out its mandates effectively.
+5. **Closed Meetings**: The commission's meetings are closed to the public, which may prevent community members, including relatives of victims, from participating in discussions or hearings that could influence the outcomes of cases. 
+6. **Limited Funding and Compensation**: Members of the commission volunteer their time without compensation beyond per diem and travel expenses, which may discourage participation from individuals who cannot afford to serve without a salary.</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>1. "The commission shall prepare a report of the commission's findings and recommendations. Not later than January 1 every three years, the commission shall submit the report to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available. The commission shall make the report publicly available through the Department of Public Safety." (Section 4, Subsection n)
+2. "The Department of Public Safety shall conduct a needs assessment to determine how to increase protective and investigative resources for identifying and reporting cases of missing and murdered indigenous persons within the state criminal justice system." (Section 5, Subsection 2)
+3. "The department shall work with the governor's office to convene meetings with tribal and local law enforcement agencies, federally recognized tribes, and Alaska Native organizations to determine the scope of the issue, identify barriers, and determine methods for creating partnerships to increase reporting and investigation of cases involving missing and murdered indigenous persons." (Section 5, Subsection 3)
+4. "The Department of Public Safety shall confer with the commission to establish standardized methods for investigating missing person reports, including for investigating missing persons reports and data collection for cases involving missing indigenous persons." (Section 4, Subsection l)</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>The text uses some gender-neutral language, such as “a person” and “members,” which avoids specifying gender. However, it predominantly refers to roles and titles in a manner that may implicitly presume a male context (e.g., using "commissioner" without specifying gender-neutral alternatives). Overall, while there are elements of gender neutrality, the text could further enhance its inclusivity by consistently avoiding gender-specific terms or assumptions about roles.</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>"…includes at least 12 hours of instruction regarding domestic violence and at least 12 hours of instruction regarding sexual assault, as those terms are defined in AS 18.66.990…" (Section 1, Subsection a) 
+"…has completed cultural training supervised by an indigenous coordinator or indigenous entity in the state that is related to addressing the rates of missing and murdered indigenous persons." (Section 1, Subsection a) 
+"…to determine methods for creating partnerships to increase reporting and investigation of cases involving missing and murdered indigenous persons." (Section 5, Subsection 8) 
+These quotes indicate prevention efforts related to training and awareness regarding domestic violence, sexual assault, and cultural issues surrounding missing and murdered indigenous persons.</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Somewhat. The text does not explicitly mention direct input from survivors or relatives of missing and murdered indigenous persons in the legislative process. However, it does provide for the involvement of a victim advocacy organization or similar service provider in the review commission, suggesting some level of representation for those impacted by these issues. Additionally, the commission's mandate to review cases and make recommendations implies that there may be opportunities for input from survivors or their families, although this is not explicitly detailed</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Somewhat. The text includes provisions for the involvement of Indigenous representatives through the establishment of a Missing and Murdered Indigenous Persons Review Commission, which has members appointed from tribal organizations and local law enforcement agencies. However, the extent of direct input from Indigenous politicians is not clearly defined; while there are positions that may include Indigenous voices, the overall control and appointments are largely determined by state officials. There is also mention of collaboration with federally recognized tribes, indicating an effort to include Indigenous communities, but it does not detail the nature or depth of that engagement.</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Sen Donald Olson (D) - District SD-T, Sen Elvi Gray-Jackson (D) - District SD-G, Sen Forrest Dunbar (D) - District SD-J, Sen Click Bishop (R) - District SD-R, Rep Matt Claman (D) - District SD-H, Sen Lyman Hoffman (D) - District SD-S, Sen Bert Stedman (R) - District SD-A, Sen Loki Tobin (D) - District SD-I, Sen Robert Myers (R) - District SD-Q, Rep Scott Kawasaki (D) - District SD-P, Sen William Wielechowski (D) - District SD-K, Sen Jesse Kiehl (D) - District SD-B, Sen Gary Stevens (R) - District SD-C, Rep Ashley Carrick (D) - District HD-035, Rep Daniel Ortiz (I) - District HD-001, Rep Sara Hannan (D) - District HD-004, Rep Alyse Galvin (I) - District HD-014, Rep William Fields (D) - District HD-017, Rep Conrad McCormick (D) - District HD-038, Rep Thomas Baker (R) - District HD-040, Rep Jennifer Armstrong (D) - District HD-016, Rep Craig Johnson (R) - District HD-010, Rep Andrew Gray (D) - District HD-020, Rep Donna Mears (D) - District HD-021, Rep Stanley Wright (R) - District HD-022, Rep Andrew Josephson (D) - District HD-013, Rep Genevieve Mina (D) - District HD-019, Rep Calvin Schrage (N) - District HD-012, Rep Cliff Groh (D) - District HD-018, Rep Neal Foster (D) - District HD-039, Rep Bryce Edgmon (I) - District HD-037</t>
+        </is>
+      </c>
       <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>WA</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Concerning the creation of an endangered missing person advisory designation for missing indigenous persons.</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>HB1725</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>House</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2022-03-31 - H: Effective date 6/9/2022.</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>https://legiscan.com/WA/bill/HB1725/2021</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>https://legiscan.com/WA/text/HB1725/id/2566954</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>The legislation establishes a missing endangered person advisory designation specifically for missing indigenous persons in Washington state. It aims to provide law enforcement with tools to disseminate timely information and engage the public in locating missing indigenous individuals. The bill also includes provisions for local, state, tribal and other law enforcement agencies, as well as media outlets, to cooperate in efforts to recover missing indigenous persons. It amends current statutes to define missing endangered persons, including missing indigenous persons, and outlines the criteria for issuing alerts. The legislation emphasizes the need to address the high rates of violence experienced by indigenous communities and to prioritize the crisis of missing and murdered indigenous people.</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>The benefits of the legislation include establishing a missing endangered person advisory designation for missing indigenous persons, providing tools for law enforcement to disseminate information for locating missing individuals, fostering cooperation among various law enforcement and media agencies for recovering missing indigenous persons, defining criteria for issuing alerts, addressing high rates of violence among indigenous communities, using gender-inclusive language, and involving MMIP relatives in data collection efforts.</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>One potential drawback of the legislation is the lack of specific mechanisms for evaluation, which may impact the ability to measure the effectiveness of the policies and initiatives introduced. Additionally, despite using gender-inclusive language, the legislation does not have explicit provisions for input or involvement from MMIP survivors or relatives of MMIP survivors, which could limit the representation and understanding of their perspectives in addressing the crisis of missing and murdered indigenous people. Finally, while the bill highlights the high rates of violence experienced by indigenous communities, the absence of detailed involvement from Indigenous politicians such as Rep Debra Lekanoff may impact the legislation's depth and relevance to the communities it aims to serve.</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>There are no mentions of specific mechanisms for evaluation in the previously mentioned legislation.</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>Yes. The legislation uses gender inclusive language by including "missing indigenous women" and "missing indigenous person" in defining categories, ensuring a broad reference to all missing indigenous individuals. This inclusive approach acknowledges and addresses the crisis faced by both women and men within indigenous communities regarding missing persons.</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Somewhat. While the legislation acknowledges the crisis of missing and murdered indigenous people as a priority and highlights the work of tribes, state leaders, and grassroots activists in identifying factors affecting the rates of violence, there is no specific mention of input from MMIP survivors, relatives of MMIP survivors, or direct involvement of Indigenous politicians such as Rep Debra Lekanoff, who sponsored the legislation. The bill aims to address the challenges faced by indigenous communities in accessing media coverage and sharing information, but lacks explicit details on active involvement from MMIP survivors, relatives, or Indigenous politicians in shaping the legislation.</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>Rep Debra Lekanoff (D) - District HD-040A, Rep Roger Goodman (D) - District HD-045A, Rep Liz Berry (D) - District HD-036B, Rep Jamila Taylor (D) - District HD-030A, Rep Javier Valdez (D) - District HD-046B, Rep Jessica Bateman (D) - District HD-022B, Rep Nicole Macri (D) - District HD-043A, Rep Strom Peterson (D) - District HD-021A, Rep Alex Ramel (D) - District HD-040B, Rep Tarra Simmons (D) - District HD-023A, Rep Tina Orwall (D) - District HD-033A, Rep Frank Chopp (D) - District HD-043B, Rep Monica Stonier (D) - District HD-049B, Rep Kirsten Harris-Talley (D) - District HD-037B, Rep Noel Frame (D) - District HD-036A</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>Rep Debra Lekanoff (D) - District HD-040A</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>2021-2022 Regular Session</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>Taskforce, Data Collection, MMIP Relatives</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>2022-03-31</t>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>2023-2024 Regular Session</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>1. Taskforce 
+2. Data Collection 
+3. Tribal Law Enforcement 
+4. MMIP Relatives 
+These categories are applicable due to the establishment of the Missing and Murdered Indigenous Persons Review Commission, which functions similarly to a task force. There are provisions for data collection in relation to missing persons, as well as cooperation with tribal law enforcement and efforts to engage with federally recognized tribes. Although the direct involvement of MMIP relatives is not explicitly mentioned, the presence of a victim advocacy organization within the commission suggests some level of representation.</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>2024-10-09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Continued refactoring of bill_processor
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -609,29 +609,24 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>The text outlines Alaska's SB 151, which establishes a Missing and Murdered Indigenous Persons Review Commission and mandates specific training for police officers concerning cases of missing and murdered indigenous persons. Key provisions include amending police training requirements to include cultural training related to these issues, the creation of dedicated investigators within the Department of Public Safety, and directives for the commission to report on unresolved cases and analyze trends. The act also mandates conducting a needs assessment to enhance investigative resources and outlines transitional provisions for current police officers and commission members. The law is set to take effect on January 1, 2025, with some sections expiring on January 1, 2027.</t>
+          <t>The Enrolled SB 151 Act establishes measures to improve police officer training in Alaska, focusing on issues like domestic violence, sexual assault, and cultural awareness related to Indigenous communities. It creates the Missing and Murdered Indigenous Persons Review Commission, which will consist of various members, including law enforcement, victim advocacy, and tribal representatives, to investigate unresolved cases involving missing and murdered Indigenous persons. The Act mandates that the Department of Public Safety submit missing person reports to a national database within a specified timeframe and requires data collection for better understanding of these cases. Additionally, it stipulates that the commission review trends in these cases and provide recommendations to enhance law enforcement practices. The provisions outlined in the Act will take effect on January 1, 2025, with certain sections requiring compliance or review by January 1, 2027.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>The benefits of Enrolled SB 151 include:
-1. **Enhanced Law Enforcement Training**: The legislation mandates at least 12 hours of training on domestic violence and sexual assault for police officers, ensuring they are better prepared to handle sensitive cases, particularly those involving Indigenous persons.
-2. **Creation of the Missing and Murdered Indigenous Persons Review Commission**: This commission aims to systematically address and review unresolved cases, providing a focused oversight mechanism to enhance justice for Indigenous communities.
-3. **Improved Data Collection and Reporting**: The act stipulates that missing person reports must be submitted to a national database within a specified time frame, which enhances tracking and accountability.
-4. **Increased Community Engagement**: By requiring liaisons to be established between law enforcement and federally recognized tribes, the law fosters collaboration and communication, potentially leading to more effective responses to cases involving missing and murdered Indigenous persons.
-5. **Long-term Assessments and Recommendations**: The act includes provisions for the commission to conduct reviews and report findings every three years, ensuring ongoing evaluation and potential policy improvements based on the evolving needs of the community. 
-6. **Support for Indigenous Cultural Training**: The inclusion of cultural training supervised by Indigenous entities promotes understanding and sensitivity among law enforcement officers towards the unique challenges faced by Indigenous communities.</t>
+          <t>1. **Taskforce**: The creation of the Missing and Murdered Indigenous Persons Review Commission serves as a taskforce focused on addressing the critical issues of missing and murdered Indigenous persons in Alaska.
+2. **Data Collection**: The Act includes requirements for data collection, mandating that the Department of Public Safety submit missing person reports to national databases, which is essential for understanding the scope of the issue.
+3. **Tribal Law Enforcement**: The legislation acknowledges the role of tribal law enforcement by requiring involvement from village public safety officers and tribal police officers in the commission, facilitating collaboration with Indigenous communities.
+4. **MMIP Relatives**: The inclusion of a member from a victim advocacy organization and an Alaska Native tribal organization indicates a degree of representation for the perspectives and concerns of relatives of missing and murdered Indigenous persons.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>The drawbacks of Enrolled SB 151 include:
-1. **Limited Direct Input from Relatives and Survivors**: While the commission includes members from victim advocacy organizations, direct representation from the relatives of missing and murdered Indigenous persons is not specified, potentially leading to gaps in addressing their specific needs and concerns.
-2. **Confidentiality Constraints**: The stipulation that documents and materials reviewed by the commission are confidential may limit transparency and community engagement, as families and tribes may feel excluded from the processes that directly impact them.
-3. **Potential Bureaucratic Delays**: The requirement for a needs assessment and the structured process for reporting may lead to bureaucratic delays, potentially hindering timely responses to cases involving missing and murdered Indigenous persons.
-4. **Dependence on State Resources**: The effectiveness of the commission relies on the State Department of Public Safety’s resources and commitment, which may vary, potentially affecting the commission's ability to carry out its mandates effectively.
-5. **Closed Meetings**: The commission's meetings are closed to the public, which may prevent community members, including relatives of victims, from participating in discussions or hearings that could influence the outcomes of cases. 
-6. **Limited Funding and Compensation**: Members of the commission volunteer their time without compensation beyond per diem and travel expenses, which may discourage participation from individuals who cannot afford to serve without a salary.</t>
+          <t>1. **Resource Allocation Concerns**: The establishment of the Missing and Murdered Indigenous Persons Review Commission and expanded training requirements may strain existing resources and budgets within law enforcement agencies, potentially diverting attention from other pressing issues.
+2. **Dependency on Training Compliance**: The act places significant reliance on police officers completing new training and cultural competency courses; non-compliance could hinder the effectiveness of the intended improvements in handling cases of missing and murdered Indigenous persons.
+3. **Potential Bureaucratic Delays**: The requirement for multiple approvals and reports may lead to bureaucratic delays, impacting the timely investigation and resolution of cases involving missing and murdered Indigenous persons.
+4. **Limited Community Input**: Although there are provisions for a victim advocacy organization and tribal representation on the commission, the overall structure may not fully incorporate input from survivors or relatives of missing and murdered Indigenous persons, potentially leading to oversight of their perspectives and needs.
+5. **Confidentiality Restrictions**: The confidential nature of the cases reviewed by the commission may limit transparency and accountability, potentially diminishing trust within the community about the processes and outcomes of investigations.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -641,20 +636,23 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>1. "The commission shall prepare a report of the commission's findings and recommendations. Not later than January 1 every three years, the commission shall submit the report to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available. The commission shall make the report publicly available through the Department of Public Safety." (Section 4, Subsection n)
+          <t>1. "The commission shall prepare a report of the commission's findings and recommendations. Not later than January 1 every three years, the commission shall submit the report to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available." (Section 4, Subsection n)
 2. "The Department of Public Safety shall conduct a needs assessment to determine how to increase protective and investigative resources for identifying and reporting cases of missing and murdered indigenous persons within the state criminal justice system." (Section 5, Subsection 2)
-3. "The department shall work with the governor's office to convene meetings with tribal and local law enforcement agencies, federally recognized tribes, and Alaska Native organizations to determine the scope of the issue, identify barriers, and determine methods for creating partnerships to increase reporting and investigation of cases involving missing and murdered indigenous persons." (Section 5, Subsection 3)
+3. "The Department of Public Safety shall work with the governor's office to convene meetings with tribal and local law enforcement agencies, federally recognized tribes, and Alaska Native organizations to determine the scope of the issue, identify barriers, and determine methods for creating partnerships to increase reporting and investigation of cases involving missing and murdered indigenous persons." (Section 5, Subsection 3)
 4. "The Department of Public Safety shall confer with the commission to establish standardized methods for investigating missing person reports, including for investigating missing persons reports and data collection for cases involving missing indigenous persons." (Section 4, Subsection l)</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>The text outlines various provisions to address the complex issue of missing and murdered Indigenous persons in Alaska, primarily through the establishment of the Missing and Murdered Indigenous Persons Review Commission and enhanced police training requirements.
+One of the central features is the requirement for police officers to undergo specific training focused on domestic violence, sexual assault, and cultural sensitivity. This training aims to ensure that law enforcement personnel are better equipped to handle cases involving Indigenous peoples and understand the cultural context surrounding these issues.
+The legislation also emphasizes the importance of data collection and reporting mechanisms. It mandates that the Department of Public Safety submit missing person reports to a national database, improving the tracking and accountability of these cases. Additionally, the commission is tasked with reviewing unresolved cases to examine trends and make policy recommendations to better address the needs of Indigenous communities.
+Overall, the act represents a multi-faceted approach to tackling the persistent issues around missing and murdered Indigenous individuals, reinforcing collaboration between law enforcement, Indigenous organizations, and community advocates. By committing to ongoing assessments and establishing structured frameworks for response, it seeks to create a more effective and culturally informed policing approach in Alaska</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>The text uses some gender-neutral language, such as “a person” and “members,” which avoids specifying gender. However, it predominantly refers to roles and titles in a manner that may implicitly presume a male context (e.g., using "commissioner" without specifying gender-neutral alternatives). Overall, while there are elements of gender neutrality, the text could further enhance its inclusivity by consistently avoiding gender-specific terms or assumptions about roles.</t>
+          <t>The text does not consistently use gender-inclusive language. While it employs terms like "a person" in relation to police officers, which is gender-neutral, the primary references within the text do not specifically include or acknowledge gender diversity beyond the general. Overall, the focus appears to be on structural and procedural elements rather than on explicitly fostering gender inclusivity.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -664,20 +662,24 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>"…includes at least 12 hours of instruction regarding domestic violence and at least 12 hours of instruction regarding sexual assault, as those terms are defined in AS 18.66.990…" (Section 1, Subsection a) 
-"…has completed cultural training supervised by an indigenous coordinator or indigenous entity in the state that is related to addressing the rates of missing and murdered indigenous persons." (Section 1, Subsection a) 
-"…to determine methods for creating partnerships to increase reporting and investigation of cases involving missing and murdered indigenous persons." (Section 5, Subsection 8) 
-These quotes indicate prevention efforts related to training and awareness regarding domestic violence, sexual assault, and cultural issues surrounding missing and murdered indigenous persons.</t>
+          <t>"The commission shall prepare a report of the commission's findings and recommendations. Not later than January 1 every three years, the commission shall submit the report to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available." (Section 4, Subsection n)
+"The Department of Public Safety shall conduct a needs assessment to determine how to increase protective and investigative resources for identifying and reporting cases of missing and murdered indigenous persons within the state criminal justice system." (Section 5, Subsection 2)
+"The department shall work with the governor's office to convene meetings with tribal and local law enforcement agencies, federally recognized tribes, and Alaska Native organizations to determine the scope of the issue, identify barriers, and determine methods for creating partnerships to increase reporting and investigation of cases involving missing and murdered indigenous persons." (Section 5, Subsection 3)
+"The Department of Public Safety shall confer with the commission to establish standardized methods for investigating missing person reports, including for investigating missing persons reports and data collection for cases involving missing indigenous persons." (Section 4, Subsection l)</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Somewhat. The text does not explicitly mention direct input from survivors or relatives of missing and murdered indigenous persons in the legislative process. However, it does provide for the involvement of a victim advocacy organization or similar service provider in the review commission, suggesting some level of representation for those impacted by these issues. Additionally, the commission's mandate to review cases and make recommendations implies that there may be opportunities for input from survivors or their families, although this is not explicitly detailed</t>
+          <t>**No.** 
+The text does not specifically identify any prevention efforts related to training or awareness involving survivors or relatives of missing and murdered Indigenous persons. While it establishes the Missing and Murdered Indigenous Persons Review Commission and mandates training for police officers, there is no mention of direct programs aimed at prevention efforts that engage or involve survivors or their families</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Somewhat. The text includes provisions for the involvement of Indigenous representatives through the establishment of a Missing and Murdered Indigenous Persons Review Commission, which has members appointed from tribal organizations and local law enforcement agencies. However, the extent of direct input from Indigenous politicians is not clearly defined; while there are positions that may include Indigenous voices, the overall control and appointments are largely determined by state officials. There is also mention of collaboration with federally recognized tribes, indicating an effort to include Indigenous communities, but it does not detail the nature or depth of that engagement.</t>
+          <t>"The commission shall prepare a report of the commission's findings and recommendations. Not later than January 1 every three years, the commission shall submit the report to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available." (Section 4, Subsection n)
+"The Department of Public Safety shall conduct a needs assessment to determine how to increase protective and investigative resources for identifying and reporting cases of missing and murdered indigenous persons within the state criminal justice system." (Section 5, Subsection 2)
+"The department shall work with the governor's office to convene meetings with tribal and local law enforcement agencies, federally recognized tribes, and Alaska Native organizations to determine the scope of the issue, identify barriers, and determine methods for creating partnerships to increase reporting and investigation of cases involving missing and murdered indigenous persons." (Section 5, Subsection 3)
+"The Department of Public Safety shall confer with the commission to establish standardized methods for investigating missing person reports, including for investigating missing persons reports and data collection for cases involving missing indigenous persons." (Section 4, Subsection l)</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -693,11 +695,10 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>1. Taskforce 
-2. Data Collection 
-3. Tribal Law Enforcement 
-4. MMIP Relatives 
-These categories are applicable due to the establishment of the Missing and Murdered Indigenous Persons Review Commission, which functions similarly to a task force. There are provisions for data collection in relation to missing persons, as well as cooperation with tribal law enforcement and efforts to engage with federally recognized tribes. Although the direct involvement of MMIP relatives is not explicitly mentioned, the presence of a victim advocacy organization within the commission suggests some level of representation.</t>
+          <t>1. **Taskforce**: The establishment of the Missing and Murdered Indigenous Persons Review Commission functions as a taskforce dedicated to addressing the issues of missing and murdered Indigenous persons.
+2. **Data Collection**: The Act includes provisions for data collection through the mandate that the Department of Public Safety submit missing person reports to national databases and conduct needs assessments related to the protective and investigative resources required for these cases.
+3. **Tribal Law Enforcement**: The involvement of tribal police officers and liaisons indicates collaboration with tribal law enforcement agencies, recognizing their essential role in addressing Indigenous persons' issues.
+4. **MMIP Relatives**: The inclusion of a member from a victim advocacy organization and a member from an Alaska Native tribal organization on the review commission signifies some representation of the perspectives and needs of relatives of missing and murdered Indigenous persons.</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">

</xml_diff>

<commit_message>
Fetches legiscan URLs and docs
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -425,285 +425,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Bill Number</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Progression</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Chamber</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Chamber Details</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Bill Overview</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Bill Text</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Optional Link</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Summary</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>UIC Pros</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>UIC Cons</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Mechanisms for Evaluation?</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Mechanisms for Evaluation</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Gender Inclusive Language?</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Gender Inclusive Explanation</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Prevention Efforts?</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Prevention Efforts</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Level of Survivor / Relative Input</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Centering of Indigenous Voices</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>Sponsors</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>Indigenous Sponsorship</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>Session</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>Categories</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>Last Update</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>AK</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Missing/murdered Indigenous People;report</t>
+          <t>No State Info</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SB151</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Senate</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2024-10-09 - S: EFFECTIVE DATE(S) OF LAW 1/1/25</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>https://legiscan.com/AK/bill/SB151/2023</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>https://legiscan.com/AK/text/SB151/id/3007736</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>The Enrolled SB 151 Act establishes measures to improve police officer training in Alaska, focusing on issues like domestic violence, sexual assault, and cultural awareness related to Indigenous communities. It creates the Missing and Murdered Indigenous Persons Review Commission, which will consist of various members, including law enforcement, victim advocacy, and tribal representatives, to investigate unresolved cases involving missing and murdered Indigenous persons. The Act mandates that the Department of Public Safety submit missing person reports to a national database within a specified timeframe and requires data collection for better understanding of these cases. Additionally, it stipulates that the commission review trends in these cases and provide recommendations to enhance law enforcement practices. The provisions outlined in the Act will take effect on January 1, 2025, with certain sections requiring compliance or review by January 1, 2027.</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>1. **Taskforce**: The creation of the Missing and Murdered Indigenous Persons Review Commission serves as a taskforce focused on addressing the critical issues of missing and murdered Indigenous persons in Alaska.
-2. **Data Collection**: The Act includes requirements for data collection, mandating that the Department of Public Safety submit missing person reports to national databases, which is essential for understanding the scope of the issue.
-3. **Tribal Law Enforcement**: The legislation acknowledges the role of tribal law enforcement by requiring involvement from village public safety officers and tribal police officers in the commission, facilitating collaboration with Indigenous communities.
-4. **MMIP Relatives**: The inclusion of a member from a victim advocacy organization and an Alaska Native tribal organization indicates a degree of representation for the perspectives and concerns of relatives of missing and murdered Indigenous persons.</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>1. **Resource Allocation Concerns**: The establishment of the Missing and Murdered Indigenous Persons Review Commission and expanded training requirements may strain existing resources and budgets within law enforcement agencies, potentially diverting attention from other pressing issues.
-2. **Dependency on Training Compliance**: The act places significant reliance on police officers completing new training and cultural competency courses; non-compliance could hinder the effectiveness of the intended improvements in handling cases of missing and murdered Indigenous persons.
-3. **Potential Bureaucratic Delays**: The requirement for multiple approvals and reports may lead to bureaucratic delays, impacting the timely investigation and resolution of cases involving missing and murdered Indigenous persons.
-4. **Limited Community Input**: Although there are provisions for a victim advocacy organization and tribal representation on the commission, the overall structure may not fully incorporate input from survivors or relatives of missing and murdered Indigenous persons, potentially leading to oversight of their perspectives and needs.
-5. **Confidentiality Restrictions**: The confidential nature of the cases reviewed by the commission may limit transparency and accountability, potentially diminishing trust within the community about the processes and outcomes of investigations.</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>1. "The commission shall prepare a report of the commission's findings and recommendations. Not later than January 1 every three years, the commission shall submit the report to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available." (Section 4, Subsection n)
-2. "The Department of Public Safety shall conduct a needs assessment to determine how to increase protective and investigative resources for identifying and reporting cases of missing and murdered indigenous persons within the state criminal justice system." (Section 5, Subsection 2)
-3. "The Department of Public Safety shall work with the governor's office to convene meetings with tribal and local law enforcement agencies, federally recognized tribes, and Alaska Native organizations to determine the scope of the issue, identify barriers, and determine methods for creating partnerships to increase reporting and investigation of cases involving missing and murdered indigenous persons." (Section 5, Subsection 3)
-4. "The Department of Public Safety shall confer with the commission to establish standardized methods for investigating missing person reports, including for investigating missing persons reports and data collection for cases involving missing indigenous persons." (Section 4, Subsection l)</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>The text outlines various provisions to address the complex issue of missing and murdered Indigenous persons in Alaska, primarily through the establishment of the Missing and Murdered Indigenous Persons Review Commission and enhanced police training requirements.
-One of the central features is the requirement for police officers to undergo specific training focused on domestic violence, sexual assault, and cultural sensitivity. This training aims to ensure that law enforcement personnel are better equipped to handle cases involving Indigenous peoples and understand the cultural context surrounding these issues.
-The legislation also emphasizes the importance of data collection and reporting mechanisms. It mandates that the Department of Public Safety submit missing person reports to a national database, improving the tracking and accountability of these cases. Additionally, the commission is tasked with reviewing unresolved cases to examine trends and make policy recommendations to better address the needs of Indigenous communities.
-Overall, the act represents a multi-faceted approach to tackling the persistent issues around missing and murdered Indigenous individuals, reinforcing collaboration between law enforcement, Indigenous organizations, and community advocates. By committing to ongoing assessments and establishing structured frameworks for response, it seeks to create a more effective and culturally informed policing approach in Alaska</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>The text does not consistently use gender-inclusive language. While it employs terms like "a person" in relation to police officers, which is gender-neutral, the primary references within the text do not specifically include or acknowledge gender diversity beyond the general. Overall, the focus appears to be on structural and procedural elements rather than on explicitly fostering gender inclusivity.</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>"The commission shall prepare a report of the commission's findings and recommendations. Not later than January 1 every three years, the commission shall submit the report to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available." (Section 4, Subsection n)
-"The Department of Public Safety shall conduct a needs assessment to determine how to increase protective and investigative resources for identifying and reporting cases of missing and murdered indigenous persons within the state criminal justice system." (Section 5, Subsection 2)
-"The department shall work with the governor's office to convene meetings with tribal and local law enforcement agencies, federally recognized tribes, and Alaska Native organizations to determine the scope of the issue, identify barriers, and determine methods for creating partnerships to increase reporting and investigation of cases involving missing and murdered indigenous persons." (Section 5, Subsection 3)
-"The Department of Public Safety shall confer with the commission to establish standardized methods for investigating missing person reports, including for investigating missing persons reports and data collection for cases involving missing indigenous persons." (Section 4, Subsection l)</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>**No.** 
-The text does not specifically identify any prevention efforts related to training or awareness involving survivors or relatives of missing and murdered Indigenous persons. While it establishes the Missing and Murdered Indigenous Persons Review Commission and mandates training for police officers, there is no mention of direct programs aimed at prevention efforts that engage or involve survivors or their families</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>"The commission shall prepare a report of the commission's findings and recommendations. Not later than January 1 every three years, the commission shall submit the report to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available." (Section 4, Subsection n)
-"The Department of Public Safety shall conduct a needs assessment to determine how to increase protective and investigative resources for identifying and reporting cases of missing and murdered indigenous persons within the state criminal justice system." (Section 5, Subsection 2)
-"The department shall work with the governor's office to convene meetings with tribal and local law enforcement agencies, federally recognized tribes, and Alaska Native organizations to determine the scope of the issue, identify barriers, and determine methods for creating partnerships to increase reporting and investigation of cases involving missing and murdered indigenous persons." (Section 5, Subsection 3)
-"The Department of Public Safety shall confer with the commission to establish standardized methods for investigating missing person reports, including for investigating missing persons reports and data collection for cases involving missing indigenous persons." (Section 4, Subsection l)</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>Sen Donald Olson (D) - District SD-T, Sen Elvi Gray-Jackson (D) - District SD-G, Sen Forrest Dunbar (D) - District SD-J, Sen Click Bishop (R) - District SD-R, Rep Matt Claman (D) - District SD-H, Sen Lyman Hoffman (D) - District SD-S, Sen Bert Stedman (R) - District SD-A, Sen Loki Tobin (D) - District SD-I, Sen Robert Myers (R) - District SD-Q, Rep Scott Kawasaki (D) - District SD-P, Sen William Wielechowski (D) - District SD-K, Sen Jesse Kiehl (D) - District SD-B, Sen Gary Stevens (R) - District SD-C, Rep Ashley Carrick (D) - District HD-035, Rep Daniel Ortiz (I) - District HD-001, Rep Sara Hannan (D) - District HD-004, Rep Alyse Galvin (I) - District HD-014, Rep William Fields (D) - District HD-017, Rep Conrad McCormick (D) - District HD-038, Rep Thomas Baker (R) - District HD-040, Rep Jennifer Armstrong (D) - District HD-016, Rep Craig Johnson (R) - District HD-010, Rep Andrew Gray (D) - District HD-020, Rep Donna Mears (D) - District HD-021, Rep Stanley Wright (R) - District HD-022, Rep Andrew Josephson (D) - District HD-013, Rep Genevieve Mina (D) - District HD-019, Rep Calvin Schrage (N) - District HD-012, Rep Cliff Groh (D) - District HD-018, Rep Neal Foster (D) - District HD-039, Rep Bryce Edgmon (I) - District HD-037</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>2023-2024 Regular Session</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>1. **Taskforce**: The establishment of the Missing and Murdered Indigenous Persons Review Commission functions as a taskforce dedicated to addressing the issues of missing and murdered Indigenous persons.
-2. **Data Collection**: The Act includes provisions for data collection through the mandate that the Department of Public Safety submit missing person reports to national databases and conduct needs assessments related to the protective and investigative resources required for these cases.
-3. **Tribal Law Enforcement**: The involvement of tribal police officers and liaisons indicates collaboration with tribal law enforcement agencies, recognizing their essential role in addressing Indigenous persons' issues.
-4. **MMIP Relatives**: The inclusion of a member from a victim advocacy organization and a member from an Alaska Native tribal organization on the review commission signifies some representation of the perspectives and needs of relatives of missing and murdered Indigenous persons.</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>2024-10-09</t>
+          <t>No Title Info</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixed issue fetching text
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:Z2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,7 +451,112 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Progression</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Chamber</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Chamber Details</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Bill Overview</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Bill Text</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Optional Link</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>UIC Pros</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>UIC Cons</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Mechanisms for Evaluation?</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Mechanisms for Evaluation</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Gender Inclusive Language?</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Gender Inclusive Explanation</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Prevention Efforts?</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Prevention Efforts</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Level of Survivor / Relative Input</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Centering of Indigenous Voices</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Sponsors</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Indigenous Sponsorship</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Session</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Categories</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Last Update</t>
         </is>
       </c>
     </row>
@@ -463,22 +568,151 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Missing/murdered Indigenous Women; Report</t>
+          <t>Missing/murdered Indigenous People;report</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SB211</t>
+          <t>SB151</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Duplicate -- Skipped</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://legiscan.com/AK/text/SB211/id/2525556</t>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Senate</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2024-10-09 - S: EFFECTIVE DATE(S) OF LAW 1/1/25</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://legiscan.com/AK/bill/SB151/2023</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>https://legiscan.com/AK/bill/SB151/2023</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>The text outlines Enrolled SB 151, a legislative action in Alaska aimed at addressing the issue of missing and murdered indigenous persons. It mandates enhanced police officer training that includes cultural training related to this issue and establishes the Missing and Murdered Indigenous Persons Review Commission within the Department of Public Safety. The commission will consist of nine members and is tasked with reviewing unresolved cases, studying trends, and making recommendations to improve practices related to these cases. Additionally, the Department of Public Safety is required to conduct a needs assessment to evaluate and enhance investigative resources. The provisions of the act will take effect on January 1, 2025, with transitional measures for current police officers and commission members.</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>The benefits of the provisions outlined in Enrolled SB 151 include:
+1. **Enhanced Police Training**: The legislation mandates police officers to receive specific training on domestic violence, sexual assault, and cultural awareness related to Indigenous issues. This aims to improve the overall response of law enforcement to cases involving missing and murdered Indigenous persons, ensuring that officers are better equipped to handle these sensitive situations.
+2. **Establishment of a Review Commission**: The Missing and Murdered Indigenous Persons Review Commission is established to systematically examine unresolved cases and recommend policies and practices to enhance collaboration among law enforcement, communities, and tribal entities. This fosters accountability and encourages a more coordinated approach to addressing the crisis.
+3. **Direct Employment of Investigators**: The creation of positions within the Department of Public Safety specifically focused on investigating cases of missing and murdered Indigenous persons ensures dedicated resources are available to address these events. This direct involvement enhances the investigation processes and helps to establish trust between law enforcement and Indigenous communities.
+4. **Liaison Role**: The commission includes members from victim advocacy organizations and Indigenous representatives, facilitating a channel for survivor voices and community input in the legislative process. This representation is crucial for tailoring responses and recommendations to the unique needs and strengths of Indigenous communities.
+5. **Data Collection and Reporting**: The requirement for the Department of Public Safety to conduct needs assessments and submit reports enhances transparency and allows for the tracking of progress in addressing missing and murdered Indigenous persons. It ensures ongoing evaluation of strategies and can lead to better-informed decisions and resource allocation.
+Overall, the legislation is designed to create a more supportive framework for addressing the issues surrounding missing and murdered Indigenous persons, ultimately leading to improved safety and representation for these communities.</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>The drawbacks or cons associated with the provisions outlined in Enrolled SB 151 include:
+1. **Complex Implementation**: The establishment of the Missing and Murdered Indigenous Persons Review Commission involves multiple stakeholders, which may lead to bureaucratic complexities that could hinder swift decision-making and action. The requirement for various appointments and positions could slow down responses to urgent cases.
+2. **Limited Direct Input from Survivors and Relatives**: While the commission includes representatives from victim advocacy organizations, there is no explicit requirement for direct representation or ongoing input from survivors or relatives of missing and murdered Indigenous persons. This may result in the commission's perspectives not fully reflecting the experiences and needs of affected families.
+3. **Confidentiality Measures**: The commission operates under strict confidentiality regarding the documents and materials it reviews, which may limit transparency and public trust. While confidentiality is essential for sensitive cases, it could also prevent the sharing of information that is vital for broader community awareness and advocacy regarding the issues being addressed.
+4. **Potential Resource Limitations**: The act mandates new roles and requirements, such as training for police officers and the hiring of investigators specifically for missing and murdered Indigenous persons. This could strain existing resources and funding within the Department of Public Safety, particularly if adequate funding is not secured or allocated in a timely manner.
+5. **Dependence on Government Cooperation**: The act relies heavily on cooperation between government entities, Indigenous communities, and law enforcement agencies. If these entities do not work effectively together, it may limit the success of the efforts to address the critical issues of missing and murdered Indigenous persons. 
+Overall, while SB 151 has the potential to create positive change, these drawbacks could pose challenges in its effective implementation and impact.</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>1. "The commission shall prepare a report of the commission's findings and recommendations. Not later than January 1 every three years, the commission shall submit the report to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available. The commission shall make the report publicly available through the Department of Public Safety."
+2. "The Department of Public Safety shall conduct a needs assessment to determine how to increase protective and investigative resources for identifying and reporting cases of missing and murdered indigenous persons within the state criminal justice system."
+3. "The department shall work with the governor's office to convene meetings with tribal and local law enforcement agencies, federally recognized tribes, and Alaska Native organizations to determine the scope of the issue, identify barriers, and determine methods for creating partnerships to increase reporting and investigation of cases involving missing and murdered indigenous persons."
+4. "The Department of Public Safety shall confer with the commission to establish standardized methods for investigating missing person reports, including for investigating missing persons reports and data collection for cases involving missing indigenous persons." 
+5. "The commission shall review unresolved cases involving missing and murdered indigenous persons from different state regions that are identified by the Department of Public Safety to examine the trends and patterns related to missing and murdered indigenous persons."</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>The text employs some gender-neutral language, using terms like "person" instead of gender-specific titles and referring to "members" in a way that isn't gender-exclusive. However, it does not consistently use gender-inclusive language, such as incorporating explicitly inclusive terms or structures throughout. Overall, while some gender neutrality is present, the text could do more to be fully gender-inclusive.</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>1. "A person may not be appointed as a police officer, except on a probationary basis, unless the person (1) has satisfactorily completed a basic program of police training approved by the council, which includes at least 12 hours of instruction regarding domestic violence and at least 12 hours of instruction regarding sexual assault, as those terms are defined in AS 18.66.990."
+2. "has completed cultural training supervised by an indigenous coordinator or indigenous entity in the state that is related to addressing the rates of missing and murdered indigenous persons."
+3. "The Department of Public Safety shall confer with the commission to establish standardized methods for investigating missing person reports, including for investigating missing persons reports and data collection for cases involving missing indigenous persons."
+4. "The department shall work with the governor's office to convene meetings with tribal and local law enforcement agencies, federally recognized tribes, and Alaska Native organizations to determine the scope of the issue, identify barriers, and determine methods for creating partnerships to increase reporting and investigation of cases involving missing and murdered indigenous persons." 
+5. "The Department of Public Safety may collaborate with the commission for public outreach purposes." 
+6. "The commission shall review unresolved cases involving missing and murdered indigenous persons from different state regions that are identified by the Department of Public Safety to examine the trends and patterns related to missing and murdered indigenous persons." 
+7. "The commission shall prepare a report of the commission's findings and recommendations." 
+8. "Most of the commission members are from victim advocacy organizations, tribal organizations, and law enforcement, which helps increase awareness and collaboration."</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Somewhat. 
+The text establishes the Missing and Murdered Indigenous Persons Review Commission, which includes members from various organizations, including one from a victim advocacy organization and one from an Alaska Native tribal organization, which suggests a level of consideration for input from survivors and their families. However, it does not explicitly mention direct involvement or input from survivors or their relatives in the decision-making processes or activities of the commission. While there is some acknowledgment of their perspectives through the inclusion of advocacy organizations, the level of direct input from survivors or relatives appears limited</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Yes. 
+The text indicates a significant input from Indigenous politicians and communities through the establishment of the Missing and Murdered Indigenous Persons Review Commission, which includes members from Alaska Native tribal organizations or entities. Additionally, the legislation mandates cultural training supervised by Indigenous entities, highlighting the importance of Indigenous knowledge and community involvement in addressing the issue of missing and murdered Indigenous persons. The Department of Public Safety also plans to collaborate with tribal and local law enforcement agencies, ensuring ongoing dialogue and partnership with Indigenous communities.</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Sen Donald Olson (D) - District SD-T, Sen Elvi Gray-Jackson (D) - District SD-G, Sen Forrest Dunbar (D) - District SD-J, Sen Click Bishop (R) - District SD-R, Rep Matt Claman (D) - District SD-H, Sen Lyman Hoffman (D) - District SD-S, Sen Bert Stedman (R) - District SD-A, Sen Loki Tobin (D) - District SD-I, Sen Robert Myers (R) - District SD-Q, Rep Scott Kawasaki (D) - District SD-P, Sen William Wielechowski (D) - District SD-K, Sen Jesse Kiehl (D) - District SD-B, Sen Gary Stevens (R) - District SD-C, Rep Ashley Carrick (D) - District HD-035, Rep Daniel Ortiz (I) - District HD-001, Rep Sara Hannan (D) - District HD-004, Rep Alyse Galvin (I) - District HD-014, Rep William Fields (D) - District HD-017, Rep Conrad McCormick (D) - District HD-038, Rep Thomas Baker (R) - District HD-040, Rep Jennifer Armstrong (D) - District HD-016, Rep Craig Johnson (R) - District HD-010, Rep Andrew Gray (D) - District HD-020, Rep Donna Mears (D) - District HD-021, Rep Stanley Wright (R) - District HD-022, Rep Andrew Josephson (D) - District HD-013, Rep Genevieve Mina (D) - District HD-019, Rep Calvin Schrage (N) - District HD-012, Rep Cliff Groh (D) - District HD-018, Rep Neal Foster (D) - District HD-039, Rep Bryce Edgmon (I) - District HD-037</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Sen Donald Olson (D) - District SD-T, Sen Lyman Hoffman (D) - District SD-S, Sen William Wielechowski (D) - District SD-K, Rep William Fields (D) - District HD-017, Rep Thomas Baker (R) - District HD-040, Rep Neal Foster (D) - District HD-039, Rep Bryce Edgmon (I) - District HD-037</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>2023-2024 Regular Session</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>1. Taskforce
+2. Tribal Law Enforcement
+3. Data Collection
+4. MMIP Relatives</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>2024-10-09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bug fixes to support both legiscan urls
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -609,29 +609,22 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>The text outlines Enrolled SB 151, a legislative action in Alaska aimed at addressing the issue of missing and murdered indigenous persons. It mandates enhanced police officer training that includes cultural training related to this issue and establishes the Missing and Murdered Indigenous Persons Review Commission within the Department of Public Safety. The commission will consist of nine members and is tasked with reviewing unresolved cases, studying trends, and making recommendations to improve practices related to these cases. Additionally, the Department of Public Safety is required to conduct a needs assessment to evaluate and enhance investigative resources. The provisions of the act will take effect on January 1, 2025, with transitional measures for current police officers and commission members.</t>
+          <t>The text outlines Alaska Senate Bill 151, which focuses on instituting measures to address the issue of missing and murdered Indigenous persons. It mandates enhanced police officer training that includes specific instruction on domestic violence, sexual assault, and cultural training related to Indigenous issues. A Missing and Murdered Indigenous Persons Review Commission is established to investigate cases, review trends, and make recommendations for improving responses to such incidents. The Department of Public Safety is required to submit reports on missing persons to a national database and employ investigators dedicated to these cases. The act is set to take effect on January 1, 2025, with provisions for compliance and operational guidelines included.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>The benefits of the provisions outlined in Enrolled SB 151 include:
-1. **Enhanced Police Training**: The legislation mandates police officers to receive specific training on domestic violence, sexual assault, and cultural awareness related to Indigenous issues. This aims to improve the overall response of law enforcement to cases involving missing and murdered Indigenous persons, ensuring that officers are better equipped to handle these sensitive situations.
-2. **Establishment of a Review Commission**: The Missing and Murdered Indigenous Persons Review Commission is established to systematically examine unresolved cases and recommend policies and practices to enhance collaboration among law enforcement, communities, and tribal entities. This fosters accountability and encourages a more coordinated approach to addressing the crisis.
-3. **Direct Employment of Investigators**: The creation of positions within the Department of Public Safety specifically focused on investigating cases of missing and murdered Indigenous persons ensures dedicated resources are available to address these events. This direct involvement enhances the investigation processes and helps to establish trust between law enforcement and Indigenous communities.
-4. **Liaison Role**: The commission includes members from victim advocacy organizations and Indigenous representatives, facilitating a channel for survivor voices and community input in the legislative process. This representation is crucial for tailoring responses and recommendations to the unique needs and strengths of Indigenous communities.
-5. **Data Collection and Reporting**: The requirement for the Department of Public Safety to conduct needs assessments and submit reports enhances transparency and allows for the tracking of progress in addressing missing and murdered Indigenous persons. It ensures ongoing evaluation of strategies and can lead to better-informed decisions and resource allocation.
-Overall, the legislation is designed to create a more supportive framework for addressing the issues surrounding missing and murdered Indigenous persons, ultimately leading to improved safety and representation for these communities.</t>
+          <t>Yes.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>The drawbacks or cons associated with the provisions outlined in Enrolled SB 151 include:
-1. **Complex Implementation**: The establishment of the Missing and Murdered Indigenous Persons Review Commission involves multiple stakeholders, which may lead to bureaucratic complexities that could hinder swift decision-making and action. The requirement for various appointments and positions could slow down responses to urgent cases.
-2. **Limited Direct Input from Survivors and Relatives**: While the commission includes representatives from victim advocacy organizations, there is no explicit requirement for direct representation or ongoing input from survivors or relatives of missing and murdered Indigenous persons. This may result in the commission's perspectives not fully reflecting the experiences and needs of affected families.
-3. **Confidentiality Measures**: The commission operates under strict confidentiality regarding the documents and materials it reviews, which may limit transparency and public trust. While confidentiality is essential for sensitive cases, it could also prevent the sharing of information that is vital for broader community awareness and advocacy regarding the issues being addressed.
-4. **Potential Resource Limitations**: The act mandates new roles and requirements, such as training for police officers and the hiring of investigators specifically for missing and murdered Indigenous persons. This could strain existing resources and funding within the Department of Public Safety, particularly if adequate funding is not secured or allocated in a timely manner.
-5. **Dependence on Government Cooperation**: The act relies heavily on cooperation between government entities, Indigenous communities, and law enforcement agencies. If these entities do not work effectively together, it may limit the success of the efforts to address the critical issues of missing and murdered Indigenous persons. 
-Overall, while SB 151 has the potential to create positive change, these drawbacks could pose challenges in its effective implementation and impact.</t>
+          <t>The drawbacks or cons of the legislation can be summarized as follows:
+1. **Limited Input from Survivors and Families**: The text does not indicate any mechanisms for including direct input or representation from survivors of missing and murdered Indigenous persons or their families, which may lead to gaps in addressing their specific needs and concerns.
+2. **Potential Bureaucratic Inefficiencies**: The establishment of a review commission and additional reporting requirements may introduce bureaucratic complexities that could slow down the investigation and resolution of cases, potentially delaying justice for affected families.
+3. **Closed Meetings and Confidentiality**: While confidentiality is essential for sensitive cases, it may also reduce transparency and public trust in the commission's workings, as meetings are closed to the public and findings may not be shared openly.
+4. **Dependence on Training Compliance**: The success of the measures depends on police and agency compliance with training and investigation protocols; failure to adhere to these requirements could undermine the effectiveness of the initiatives.
+5. **Resource Strain**: The implementation of new responsibilities, such as enhanced training and investigation efforts, may strain existing resources within the Department of Public Safety, impacting its ability to effectively carry out other duties.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -641,21 +634,25 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>1. "The commission shall prepare a report of the commission's findings and recommendations. Not later than January 1 every three years, the commission shall submit the report to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available. The commission shall make the report publicly available through the Department of Public Safety."
-2. "The Department of Public Safety shall conduct a needs assessment to determine how to increase protective and investigative resources for identifying and reporting cases of missing and murdered indigenous persons within the state criminal justice system."
-3. "The department shall work with the governor's office to convene meetings with tribal and local law enforcement agencies, federally recognized tribes, and Alaska Native organizations to determine the scope of the issue, identify barriers, and determine methods for creating partnerships to increase reporting and investigation of cases involving missing and murdered indigenous persons."
-4. "The Department of Public Safety shall confer with the commission to establish standardized methods for investigating missing person reports, including for investigating missing persons reports and data collection for cases involving missing indigenous persons." 
-5. "The commission shall review unresolved cases involving missing and murdered indigenous persons from different state regions that are identified by the Department of Public Safety to examine the trends and patterns related to missing and murdered indigenous persons."</t>
+          <t>1. "The council shall prescribe the means of presenting evidence of fulfillment of these requirements."
+2. "Within 60 days after the first report concerning a missing person is filed with a local or state law enforcement agency, if the person's location has not been determined, the Department of Public Safety shall submit a missing person report to the National Missing and Unidentified Persons System database."
+3. "The Department of Public Safety shall employ at least two persons in the department to investigate cases involving missing and murdered indigenous persons and act as liaisons between law enforcement agencies, communities in the state, and federally recognized tribes."
+4. "The commission shall review unresolved cases involving missing and murdered indigenous persons from different state regions that are identified by the Department of Public Safety to examine the trends and patterns related to missing and murdered indigenous persons."
+5. "The commission shall prepare a report of the commission's findings and recommendations. Not later than January 1 every three years, the commission shall submit the report to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available."
+6. "The Department of Public Safety shall conduct a needs assessment to determine how to increase protective and investigative resources for identifying and reporting cases of missing and murdered indigenous persons within the state criminal justice system."
+7. "The department shall also work with federal law enforcement agencies to identify ways to increase information sharing and coordinate resources."</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>The text primarily uses gender-neutral language, referring to individuals as "a person" and avoiding specific gender pronouns. However, it does not expand terms significantly to explicitly include a broader range of individuals. While some terms like "tribal police officer" and "victim advocacy organization" imply inclusivity, there is a lack of direct acknowledgment or language that specifically highlights gender inclusivity. 
+**Answer:** No</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>The text employs some gender-neutral language, using terms like "person" instead of gender-specific titles and referring to "members" in a way that isn't gender-exclusive. However, it does not consistently use gender-inclusive language, such as incorporating explicitly inclusive terms or structures throughout. Overall, while some gender neutrality is present, the text could do more to be fully gender-inclusive.</t>
+          <t>The text effectively uses a mix of gender-neutral language, referring to individuals as "a person" instead of gender-specific pronouns such as "he" or "she." However, it does not make significant efforts to explicitly include diverse gender identities or broaden the reference terms to encompass all genders beyond neutrality. The language remains largely neutral without specific emphasis on inclusivity for various gender representations.
+**Answer:** No.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -665,26 +662,32 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1. "A person may not be appointed as a police officer, except on a probationary basis, unless the person (1) has satisfactorily completed a basic program of police training approved by the council, which includes at least 12 hours of instruction regarding domestic violence and at least 12 hours of instruction regarding sexual assault, as those terms are defined in AS 18.66.990."
-2. "has completed cultural training supervised by an indigenous coordinator or indigenous entity in the state that is related to addressing the rates of missing and murdered indigenous persons."
-3. "The Department of Public Safety shall confer with the commission to establish standardized methods for investigating missing person reports, including for investigating missing persons reports and data collection for cases involving missing indigenous persons."
-4. "The department shall work with the governor's office to convene meetings with tribal and local law enforcement agencies, federally recognized tribes, and Alaska Native organizations to determine the scope of the issue, identify barriers, and determine methods for creating partnerships to increase reporting and investigation of cases involving missing and murdered indigenous persons." 
-5. "The Department of Public Safety may collaborate with the commission for public outreach purposes." 
-6. "The commission shall review unresolved cases involving missing and murdered indigenous persons from different state regions that are identified by the Department of Public Safety to examine the trends and patterns related to missing and murdered indigenous persons." 
-7. "The commission shall prepare a report of the commission's findings and recommendations." 
-8. "Most of the commission members are from victim advocacy organizations, tribal organizations, and law enforcement, which helps increase awareness and collaboration."</t>
+          <t>1. "The council shall prescribe the means of presenting evidence of fulfillment of these requirements."
+2. "Within 60 days after the first report concerning a missing person is filed with a local or state law enforcement agency, if the person's location has not been determined, the Department of Public Safety shall submit a missing person report to the National Missing and Unidentified Persons System database."
+3. "The Department of Public Safety shall employ at least two persons in the department to investigate cases involving missing and murdered indigenous persons and act as liaisons between law enforcement agencies, communities in the state, and federally recognized tribes."
+4. "The commission shall review unresolved cases involving missing and murdered indigenous persons from different state regions that are identified by the Department of Public Safety to examine the trends and patterns related to missing and murdered indigenous persons."
+5. "The commission shall prepare a report of the commission's findings and recommendations. Not later than January 1 every three years, the commission shall submit the report to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available."
+6. "The Department of Public Safety shall conduct a needs assessment to determine how to increase protective and investigative resources for identifying and reporting cases of missing and murdered indigenous persons within the state criminal justice system."
+7. "The department shall also work with federal law enforcement agencies to identify ways to increase information sharing and coordinate resources."</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Somewhat. 
-The text establishes the Missing and Murdered Indigenous Persons Review Commission, which includes members from various organizations, including one from a victim advocacy organization and one from an Alaska Native tribal organization, which suggests a level of consideration for input from survivors and their families. However, it does not explicitly mention direct involvement or input from survivors or their relatives in the decision-making processes or activities of the commission. While there is some acknowledgment of their perspectives through the inclusion of advocacy organizations, the level of direct input from survivors or relatives appears limited</t>
+          <t>1. "The Department of Public Safety shall conduct a needs assessment to determine how to increase protective and investigative resources for identifying and reporting cases of missing and murdered indigenous persons within the state criminal justice system."
+2. "The department shall work with the governor's office to convene meetings with tribal and local law enforcement agencies, federally recognized tribes, and Alaska Native organizations to determine the scope of the issue, identify barriers, and determine methods for creating partnerships to increase reporting and investigation of cases involving missing and murdered indigenous persons."
+3. "The commission shall prepare a report of the commission's findings and recommendations. Not later than January 1 every three years, the commission shall submit the report to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available."
+4. "The council shall prescribe the means of presenting evidence of fulfillment of these requirements."</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Yes. 
-The text indicates a significant input from Indigenous politicians and communities through the establishment of the Missing and Murdered Indigenous Persons Review Commission, which includes members from Alaska Native tribal organizations or entities. Additionally, the legislation mandates cultural training supervised by Indigenous entities, highlighting the importance of Indigenous knowledge and community involvement in addressing the issue of missing and murdered Indigenous persons. The Department of Public Safety also plans to collaborate with tribal and local law enforcement agencies, ensuring ongoing dialogue and partnership with Indigenous communities.</t>
+          <t>1. "The council shall prescribe the means of presenting evidence of fulfillment of these requirements."
+2. "Within 60 days after the first report concerning a missing person is filed with a local or state law enforcement agency, if the person's location has not been determined, the Department of Public Safety shall submit a missing person report to the National Missing and Unidentified Persons System database."
+3. "The Department of Public Safety shall employ at least two persons in the department to investigate cases involving missing and murdered indigenous persons and act as liaisons between law enforcement agencies, communities in the state, and federally recognized tribes."
+4. "The commission shall review unresolved cases involving missing and murdered indigenous persons from different state regions that are identified by the Department of Public Safety to examine the trends and patterns related to missing and murdered indigenous persons."
+5. "The commission shall prepare a report of the commission's findings and recommendations. Not later than January 1 every three years, the commission shall submit the report to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available."
+6. "The Department of Public Safety shall conduct a needs assessment to determine how to increase protective and investigative resources for identifying and reporting cases of missing and murdered indigenous persons within the state criminal justice system."
+7. "The department shall also work with federal law enforcement agencies to identify ways to increase information sharing and coordinate resources."</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -704,10 +707,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>1. Taskforce
-2. Tribal Law Enforcement
-3. Data Collection
-4. MMIP Relatives</t>
+          <t>Yes.</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">

</xml_diff>

<commit_message>
Parses full URL OR doc specific url
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -609,22 +609,27 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>The text outlines Alaska Senate Bill 151, which focuses on instituting measures to address the issue of missing and murdered Indigenous persons. It mandates enhanced police officer training that includes specific instruction on domestic violence, sexual assault, and cultural training related to Indigenous issues. A Missing and Murdered Indigenous Persons Review Commission is established to investigate cases, review trends, and make recommendations for improving responses to such incidents. The Department of Public Safety is required to submit reports on missing persons to a national database and employ investigators dedicated to these cases. The act is set to take effect on January 1, 2025, with provisions for compliance and operational guidelines included.</t>
+          <t>Senate Bill No. 151 establishes the Missing and Murdered Indigenous Persons Review Commission within the Alaska Department of Public Safety. The commission will include nine members, including representatives from various state agencies, law enforcement, and indigenous organizations, and will examine trends related to missing and murdered indigenous persons, making recommendations to improve collaborative efforts and reduce such cases. The commission is required to submit a report of its findings by January 1, 2026. It also outlines the establishment of investigative roles within the Department of Public Safety and mandates a needs assessment to enhance resources for addressing these issues. The act is set to take effect on January 1, 2024, with certain sections repealed in 2025 and 2026.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Yes.</t>
+          <t>The benefits of SB0151A include:
+1. **Dedicated Oversight**: The establishment of the Missing and Murdered Indigenous Persons Review Commission provides a dedicated body to investigate cases, examine trends, and develop recommendations, ensuring focused attention on the critical issues surrounding missing and murdered Indigenous persons.
+2. **Collaboration with Communities**: The involvement of representatives from tribal organizations, law enforcement, and victim advocacy groups facilitates better communication and cooperation between various stakeholders, promoting a holistic approach to addressing these urgent concerns.
+3. **Data Collection and Reporting**: The act mandates the collection of data related to missing and murdered Indigenous persons and requires the commission to prepare and submit a report of its findings, which can inform policy changes and improve practices in investigations. 
+4. **Enhanced Resources and Training**: By conducting needs assessments and engaging with local and federal law enforcement agencies, the bill aims to increase protective and investigative resources, ultimately enhancing the effectiveness of responses to these cases. 
+5. **Confidentiality and Protection of Information**: The provisions regarding confidentiality help protect sensitive information for survivors and their families, ensuring that their privacy is respected during investigations.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>The drawbacks or cons of the legislation can be summarized as follows:
-1. **Limited Input from Survivors and Families**: The text does not indicate any mechanisms for including direct input or representation from survivors of missing and murdered Indigenous persons or their families, which may lead to gaps in addressing their specific needs and concerns.
-2. **Potential Bureaucratic Inefficiencies**: The establishment of a review commission and additional reporting requirements may introduce bureaucratic complexities that could slow down the investigation and resolution of cases, potentially delaying justice for affected families.
-3. **Closed Meetings and Confidentiality**: While confidentiality is essential for sensitive cases, it may also reduce transparency and public trust in the commission's workings, as meetings are closed to the public and findings may not be shared openly.
-4. **Dependence on Training Compliance**: The success of the measures depends on police and agency compliance with training and investigation protocols; failure to adhere to these requirements could undermine the effectiveness of the initiatives.
-5. **Resource Strain**: The implementation of new responsibilities, such as enhanced training and investigation efforts, may strain existing resources within the Department of Public Safety, impacting its ability to effectively carry out other duties.</t>
+          <t>The drawbacks of SB0151A include:
+1. **Limited Representation**: While the commission includes members from various organizations and law enforcement, it may lack direct, meaningful representation from survivors or relatives of missing and murdered Indigenous persons, potentially sidelining their perspectives and needs.
+2. **Confidentiality Restrictions**: The emphasis on confidentiality for documents and findings may limit transparency and prevent affected families and communities from staying informed about investigations and outcomes, which could lead to mistrust in the process.
+3. **Potential Bureaucratic Challenges**: The commission may face bureaucratic hurdles in coordinating among various governmental and tribal agencies, which could slow down the progress of investigations and implementation of recommendations.
+4. **Funding and Resource Limitations**: The lack of compensation for commission members, coupled with potential constraints on resources available for investigations and community engagement, could affect the commission’s ability to operate effectively.
+5. **Short-Term Focus**: The act includes sunset provisions with sections set to expire in 2025 and 2026, which might limit the long-term impact of the commission’s work and create uncertainty regarding ongoing support for efforts aimed at addressing these critical issues.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -634,60 +639,43 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>1. "The council shall prescribe the means of presenting evidence of fulfillment of these requirements."
-2. "Within 60 days after the first report concerning a missing person is filed with a local or state law enforcement agency, if the person's location has not been determined, the Department of Public Safety shall submit a missing person report to the National Missing and Unidentified Persons System database."
-3. "The Department of Public Safety shall employ at least two persons in the department to investigate cases involving missing and murdered indigenous persons and act as liaisons between law enforcement agencies, communities in the state, and federally recognized tribes."
-4. "The commission shall review unresolved cases involving missing and murdered indigenous persons from different state regions that are identified by the Department of Public Safety to examine the trends and patterns related to missing and murdered indigenous persons."
-5. "The commission shall prepare a report of the commission's findings and recommendations. Not later than January 1 every three years, the commission shall submit the report to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available."
-6. "The Department of Public Safety shall conduct a needs assessment to determine how to increase protective and investigative resources for identifying and reporting cases of missing and murdered indigenous persons within the state criminal justice system."
-7. "The department shall also work with federal law enforcement agencies to identify ways to increase information sharing and coordinate resources."</t>
+          <t>1. "The commission shall prepare a report of its findings and recommendations."
+2. "Not later than January 1, 2026, the commission shall submit the report to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available."
+3. "The Department of Public Safety shall conduct a needs assessment to determine how to increase protective and investigative resources for identifying and reporting cases of missing and murdered indigenous persons."
+4. "The department shall work with the governor's office to convene meetings with tribal and local law enforcement agencies, federally recognized tribes, and Alaska Native organizations to determine the scope of the issue, identify barriers, and determine methods for creating partnerships to increase reporting and investigation of cases involving missing and murdered indigenous persons."
+5. "Not later than January 1, 2025, the department shall submit a written report on the needs assessment to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available."</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>The text primarily uses gender-neutral language, referring to individuals as "a person" and avoiding specific gender pronouns. However, it does not expand terms significantly to explicitly include a broader range of individuals. While some terms like "tribal police officer" and "victim advocacy organization" imply inclusivity, there is a lack of direct acknowledgment or language that specifically highlights gender inclusivity. 
-**Answer:** No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>The text effectively uses a mix of gender-neutral language, referring to individuals as "a person" instead of gender-specific pronouns such as "he" or "she." However, it does not make significant efforts to explicitly include diverse gender identities or broaden the reference terms to encompass all genders beyond neutrality. The language remains largely neutral without specific emphasis on inclusivity for various gender representations.
-**Answer:** No.</t>
+          <t>The text employs gender-inclusive language by using terms like "person" and "members" instead of gender-specific terms, allowing for broader representation and inclusivity. Additionally, the use of titles such as "commissioner" and "officer" does not imply any gender bias. Overall, the language is neutral and avoids reference to any specific gender, which contributes to its inclusiveness.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1. "The council shall prescribe the means of presenting evidence of fulfillment of these requirements."
-2. "Within 60 days after the first report concerning a missing person is filed with a local or state law enforcement agency, if the person's location has not been determined, the Department of Public Safety shall submit a missing person report to the National Missing and Unidentified Persons System database."
-3. "The Department of Public Safety shall employ at least two persons in the department to investigate cases involving missing and murdered indigenous persons and act as liaisons between law enforcement agencies, communities in the state, and federally recognized tribes."
-4. "The commission shall review unresolved cases involving missing and murdered indigenous persons from different state regions that are identified by the Department of Public Safety to examine the trends and patterns related to missing and murdered indigenous persons."
-5. "The commission shall prepare a report of the commission's findings and recommendations. Not later than January 1 every three years, the commission shall submit the report to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available."
-6. "The Department of Public Safety shall conduct a needs assessment to determine how to increase protective and investigative resources for identifying and reporting cases of missing and murdered indigenous persons within the state criminal justice system."
-7. "The department shall also work with federal law enforcement agencies to identify ways to increase information sharing and coordinate resources."</t>
+          <t>No.</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1. "The Department of Public Safety shall conduct a needs assessment to determine how to increase protective and investigative resources for identifying and reporting cases of missing and murdered indigenous persons within the state criminal justice system."
-2. "The department shall work with the governor's office to convene meetings with tribal and local law enforcement agencies, federally recognized tribes, and Alaska Native organizations to determine the scope of the issue, identify barriers, and determine methods for creating partnerships to increase reporting and investigation of cases involving missing and murdered indigenous persons."
-3. "The commission shall prepare a report of the commission's findings and recommendations. Not later than January 1 every three years, the commission shall submit the report to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available."
-4. "The council shall prescribe the means of presenting evidence of fulfillment of these requirements."</t>
+          <t>Somewhat. 
+The text includes provisions to consult with tribal entities and local law enforcement, which could facilitate input from survivors or relatives of missing and murdered Indigenous persons. Additionally, the commission is tasked with examining trends and patterns related to these cases, potentially incorporating survivor and family perspectives in its findings and recommendations. However, the text does not explicitly state mechanisms for directly involving survivors or their relatives in decision-making processes or discussions, limiting the extent of their input</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>1. "The council shall prescribe the means of presenting evidence of fulfillment of these requirements."
-2. "Within 60 days after the first report concerning a missing person is filed with a local or state law enforcement agency, if the person's location has not been determined, the Department of Public Safety shall submit a missing person report to the National Missing and Unidentified Persons System database."
-3. "The Department of Public Safety shall employ at least two persons in the department to investigate cases involving missing and murdered indigenous persons and act as liaisons between law enforcement agencies, communities in the state, and federally recognized tribes."
-4. "The commission shall review unresolved cases involving missing and murdered indigenous persons from different state regions that are identified by the Department of Public Safety to examine the trends and patterns related to missing and murdered indigenous persons."
-5. "The commission shall prepare a report of the commission's findings and recommendations. Not later than January 1 every three years, the commission shall submit the report to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available."
-6. "The Department of Public Safety shall conduct a needs assessment to determine how to increase protective and investigative resources for identifying and reporting cases of missing and murdered indigenous persons within the state criminal justice system."
-7. "The department shall also work with federal law enforcement agencies to identify ways to increase information sharing and coordinate resources."</t>
+          <t>Yes. 
+The text demonstrates input from Indigenous politicians through the sponsorship of the bill by several Indigenous legislators, which reflects awareness of and responsiveness to the issues faced by Indigenous communities. Moreover, the establishment of the Missing and Murdered Indigenous Persons Review Commission includes provisions for collaboration with tribal entities and organizations, ensuring the involvement of Indigenous voices in the discussions and decisions regarding the legislation. The commitment to convene meetings with tribal and local law enforcement agencies further indicates an effort to incorporate community and Indigenous perspectives into the evaluation of the issues at hand.</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -707,7 +695,10 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Yes.</t>
+          <t>1. Taskforce
+2. Tribal Law Enforcement
+3. Data Collection
+4. MMIP Relatives</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">

</xml_diff>

<commit_message>
First steps taken to refactor bill_processor
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -609,27 +609,27 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Senate Bill No. 151 establishes the Missing and Murdered Indigenous Persons Review Commission within the Alaska Department of Public Safety. The commission will include nine members, including representatives from various state agencies, law enforcement, and indigenous organizations, and will examine trends related to missing and murdered indigenous persons, making recommendations to improve collaborative efforts and reduce such cases. The commission is required to submit a report of its findings by January 1, 2026. It also outlines the establishment of investigative roles within the Department of Public Safety and mandates a needs assessment to enhance resources for addressing these issues. The act is set to take effect on January 1, 2024, with certain sections repealed in 2025 and 2026.</t>
+          <t>Enrolled SB 151 establishes the Missing and Murdered Indigenous Persons Review Commission in Alaska, aimed at addressing the high rates of missing and murdered indigenous individuals. It mandates cultural training for police officers, requires the Department of Public Safety to report missing persons to a national database, and employs dedicated investigators for such cases. The commission comprises nine members, including state officials, law enforcement representatives, and advocates, and it is tasked with reviewing unresolved cases to make policy recommendations. Additionally, the bill outlines a needs assessment for improving investigative resources and provides for the transition of existing police officers to comply with the new training requirements. The act is set to take effect on January 1, 2025, with specific provisions expiring by January 1, 2027.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>The benefits of SB0151A include:
-1. **Dedicated Oversight**: The establishment of the Missing and Murdered Indigenous Persons Review Commission provides a dedicated body to investigate cases, examine trends, and develop recommendations, ensuring focused attention on the critical issues surrounding missing and murdered Indigenous persons.
-2. **Collaboration with Communities**: The involvement of representatives from tribal organizations, law enforcement, and victim advocacy groups facilitates better communication and cooperation between various stakeholders, promoting a holistic approach to addressing these urgent concerns.
-3. **Data Collection and Reporting**: The act mandates the collection of data related to missing and murdered Indigenous persons and requires the commission to prepare and submit a report of its findings, which can inform policy changes and improve practices in investigations. 
-4. **Enhanced Resources and Training**: By conducting needs assessments and engaging with local and federal law enforcement agencies, the bill aims to increase protective and investigative resources, ultimately enhancing the effectiveness of responses to these cases. 
-5. **Confidentiality and Protection of Information**: The provisions regarding confidentiality help protect sensitive information for survivors and their families, ensuring that their privacy is respected during investigations.</t>
+          <t>The benefits or pros of Enrolled SB 151 include:
+1. **Enhanced Police Training**: The legislation mandates comprehensive training for police officers that includes specific instruction on domestic violence and sexual assault, improving the preparedness of law enforcement to handle sensitive cases.
+2. **Establishment of a Review Commission**: The Missing and Murdered Indigenous Persons Review Commission is established to address the high rates of missing and murdered indigenous individuals, providing a structured approach to investigating and preventing such cases.
+3. **Dedicated Investigators**: The creation of dedicated positions within the Department of Public Safety for investigating cases of missing and murdered indigenous persons ensures focused efforts and better community liaison, which can improve relationships between law enforcement and indigenous communities.
+4. **Data Reporting and Collaboration**: The requirement to submit missing person reports to national databases enhances data collection and tracking, while collaboration with tribal and local law enforcement promotes a more comprehensive response to these issues.
+5. **Public Accountability and Reporting**: The commission is tasked with preparing regular reports on findings and recommendations, increasing transparency and holding the government accountable for addressing the needs of indigenous communities related to public safety.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>The drawbacks of SB0151A include:
-1. **Limited Representation**: While the commission includes members from various organizations and law enforcement, it may lack direct, meaningful representation from survivors or relatives of missing and murdered Indigenous persons, potentially sidelining their perspectives and needs.
-2. **Confidentiality Restrictions**: The emphasis on confidentiality for documents and findings may limit transparency and prevent affected families and communities from staying informed about investigations and outcomes, which could lead to mistrust in the process.
-3. **Potential Bureaucratic Challenges**: The commission may face bureaucratic hurdles in coordinating among various governmental and tribal agencies, which could slow down the progress of investigations and implementation of recommendations.
-4. **Funding and Resource Limitations**: The lack of compensation for commission members, coupled with potential constraints on resources available for investigations and community engagement, could affect the commission’s ability to operate effectively.
-5. **Short-Term Focus**: The act includes sunset provisions with sections set to expire in 2025 and 2026, which might limit the long-term impact of the commission’s work and create uncertainty regarding ongoing support for efforts aimed at addressing these critical issues.</t>
+          <t>The drawbacks or cons of Enrolled SB 151 include:
+1. **Limited Survivor and Relative Input**: While the legislation mentions the involvement of a victim advocacy organization, there is no explicit provision for direct input from survivors or relatives of missing and murdered indigenous persons, which could limit the responsiveness of the commission and its recommendations.
+2. **Potential for Bureaucratic Delays**: The requirement for the Department of Public Safety to submit reports and conduct needs assessments may introduce delays in addressing urgent cases, which could hinder timely interventions for missing persons.
+3. **Confidentiality Restrictions**: The emphasis on confidentiality and the closed nature of commission meetings may restrict transparency and limit community awareness or involvement in the process, potentially eroding trust between law enforcement and indigenous communities.
+4. **Resource Constraints**: The mandate for increased training and staffing may face challenges related to funding and resources, potentially impacting the effectiveness of the Department of Public Safety and the commission in carrying out their expanded duties.
+5. **Ex Officio Nonvoting Members**: The presence of ex officio nonvoting members from the legislature may dilute the influence of appointed members who are likely to have more direct connections to the indigenous community, leading to a lack of meaningful legislative support for the commission's initiatives.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -639,43 +639,40 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>1. "The commission shall prepare a report of its findings and recommendations."
-2. "Not later than January 1, 2026, the commission shall submit the report to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available."
-3. "The Department of Public Safety shall conduct a needs assessment to determine how to increase protective and investigative resources for identifying and reporting cases of missing and murdered indigenous persons."
-4. "The department shall work with the governor's office to convene meetings with tribal and local law enforcement agencies, federally recognized tribes, and Alaska Native organizations to determine the scope of the issue, identify barriers, and determine methods for creating partnerships to increase reporting and investigation of cases involving missing and murdered indigenous persons."
-5. "Not later than January 1, 2025, the department shall submit a written report on the needs assessment to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available."</t>
+          <t>1. "The commission shall prepare a report of the commission's findings and recommendations. Not later than January 1 every three years, the commission shall submit the report to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available. The commission shall make the report publicly available through the Department of Public Safety."
+2. "The Department of Public Safety shall conduct a needs assessment to determine how to increase protective and investigative resources for identifying and reporting cases of missing and murdered indigenous persons within the state criminal justice system."
+3. "The department shall work with the governor's office to convene meetings with tribal and local law enforcement agencies, federally recognized tribes, and Alaska Native organizations to determine the scope of the issue, identify barriers, and determine methods for creating partnerships to increase reporting and investigation of cases involving missing and murdered indigenous persons."
+4. "The Department of Public Safety shall confer with the commission to establish standardized methods for investigating missing person reports, including for investigating missing persons reports and data collection for cases involving missing indigenous persons."</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>The text uses gender-neutral language by employing terms like "a person," which can refer to individuals of any gender, rather than specifically male or female identifiers. However, when addressing roles and responsibilities, it primarily uses masculine pronouns or titles, such as "commissioner's designee," which may imply a male authority figure. Overall, while there is an effort to be inclusive, there are areas where gender-specific language could be improved for greater inclusivity.</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>The text employs gender-inclusive language by using terms like "person" and "members" instead of gender-specific terms, allowing for broader representation and inclusivity. Additionally, the use of titles such as "commissioner" and "officer" does not imply any gender bias. Overall, the language is neutral and avoids reference to any specific gender, which contributes to its inclusiveness.</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>No.</t>
+          <t>"A person may not be appointed as a police officer, except on a probationary basis, unless the person (1) has satisfactorily completed a basic program of police training approved by the council, which includes at least 12 hours of instruction regarding domestic violence and at least 12 hours of instruction regarding sexual assault, as those terms are defined in AS 18.66.990, [AND] (2) possesses other qualifications the council has established for the employment of police officers, including minimum age, education, physical and mental standards, citizenship, moral character, and experience, and (3) has completed cultural training supervised by an indigenous coordinator or indigenous entity in the state that is related to addressing the rates of missing and murdered indigenous persons."</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Somewhat. 
-The text includes provisions to consult with tribal entities and local law enforcement, which could facilitate input from survivors or relatives of missing and murdered Indigenous persons. Additionally, the commission is tasked with examining trends and patterns related to these cases, potentially incorporating survivor and family perspectives in its findings and recommendations. However, the text does not explicitly state mechanisms for directly involving survivors or their relatives in decision-making processes or discussions, limiting the extent of their input</t>
+          <t>Somewhat. The text includes a provision for a representative from a victim advocacy organization or similar service provider on the Missing and Murdered Indigenous Persons Review Commission, indicating some level of involvement from individuals familiar with the concerns of survivors and relatives. However, there is no mention of direct input or consultation from survivors or relatives themselves, which limits the extent of their involvement and input in the legislative process</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Yes. 
-The text demonstrates input from Indigenous politicians through the sponsorship of the bill by several Indigenous legislators, which reflects awareness of and responsiveness to the issues faced by Indigenous communities. Moreover, the establishment of the Missing and Murdered Indigenous Persons Review Commission includes provisions for collaboration with tribal entities and organizations, ensuring the involvement of Indigenous voices in the discussions and decisions regarding the legislation. The commitment to convene meetings with tribal and local law enforcement agencies further indicates an effort to incorporate community and Indigenous perspectives into the evaluation of the issues at hand.</t>
+          <t>Somewhat. The text does include input from Indigenous leaders, as it establishes a Missing and Murdered Indigenous Persons Review Commission that includes representatives from Alaska Native tribal organizations. Additionally, there is a focus on employing individuals to investigate missing and murdered Indigenous persons and acting as liaisons with federally recognized tribes, suggesting a degree of community involvement. However, the specific mechanisms for ongoing community input or decision-making powers for Indigenous communities in the process are not extensively detailed, indicating a somewhat limited level of engagement.</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -695,10 +692,12 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>1. Taskforce
-2. Tribal Law Enforcement
-3. Data Collection
-4. MMIP Relatives</t>
+          <t>The most applicable categories for the provided text are:
+1. Taskforce – The text establishes the Missing and Murdered Indigenous Persons Review Commission, which functions similarly to a task force focused on the issue.
+2. US Law Enforcement – The act includes provisions related to police officer training and the responsibilities of the Department of Public Safety.
+3. Tribal Law Enforcement – The commission includes representation from tribal police officers and aims to act as liaisons between law enforcement agencies and federally recognized tribes.
+4. Data Collection – The act mandates the submission of missing person reports to the National Missing and Unidentified Persons System database and mentions data collection concerning missing indigenous persons. 
+5. MMIP Relatives – There is a reference to involving members from a victim advocacy organization, which typically would be engaged with or representing the interests of relatives of missing and murdered indigenous persons.</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">

</xml_diff>

<commit_message>
Moved parse HTML to document_processor
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -563,17 +563,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Missing/murdered Indigenous People;report</t>
+          <t>Missing and Murdered Indigenous People Awareness Month.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SB151</t>
+          <t>ACR133</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -588,71 +588,68 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Senate</t>
+          <t>House</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2024-10-09 - S: EFFECTIVE DATE(S) OF LAW 1/1/25</t>
+          <t>2024-05-30 - : Chaptered by Secretary of State - Res. Chapter 69, Statutes of 2024.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://legiscan.com/AK/bill/SB151/2023</t>
+          <t>https://legiscan.com/CA/bill/ACR133/2023</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://legiscan.com/AK/bill/SB151/2023</t>
+          <t>https://legiscan.com/CA/bill/ACR133/2023</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Enrolled SB 151 establishes the Missing and Murdered Indigenous Persons Review Commission in Alaska, aimed at addressing the high rates of missing and murdered indigenous individuals. It mandates cultural training for police officers, requires the Department of Public Safety to report missing persons to a national database, and employs dedicated investigators for such cases. The commission comprises nine members, including state officials, law enforcement representatives, and advocates, and it is tasked with reviewing unresolved cases to make policy recommendations. Additionally, the bill outlines a needs assessment for improving investigative resources and provides for the transition of existing police officers to comply with the new training requirements. The act is set to take effect on January 1, 2025, with specific provisions expiring by January 1, 2027.</t>
+          <t>Assembly Concurrent Resolution No. 133 designates May 2024 as Missing and Murdered Indigenous People Awareness Month in California and urges the Governor to declare a state of emergency regarding this crisis. The resolution highlights alarming statistics about missing and murdered Indigenous individuals, particularly women, including the high rates of homicide and the lack of comprehensive data on the issue. It references previous legislative efforts, such as the Feather Alert and access to the California Law Enforcement Telecommunications System for Tribal courts, aimed at addressing these concerns. The resolution emphasizes the need for awareness and action to confront the epidemic affecting Indigenous communities, especially given California's significant Indigenous population. Lastly, it calls for the transmission of this resolution to the author for further distribution.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>The benefits or pros of Enrolled SB 151 include:
-1. **Enhanced Police Training**: The legislation mandates comprehensive training for police officers that includes specific instruction on domestic violence and sexual assault, improving the preparedness of law enforcement to handle sensitive cases.
-2. **Establishment of a Review Commission**: The Missing and Murdered Indigenous Persons Review Commission is established to address the high rates of missing and murdered indigenous individuals, providing a structured approach to investigating and preventing such cases.
-3. **Dedicated Investigators**: The creation of dedicated positions within the Department of Public Safety for investigating cases of missing and murdered indigenous persons ensures focused efforts and better community liaison, which can improve relationships between law enforcement and indigenous communities.
-4. **Data Reporting and Collaboration**: The requirement to submit missing person reports to national databases enhances data collection and tracking, while collaboration with tribal and local law enforcement promotes a more comprehensive response to these issues.
-5. **Public Accountability and Reporting**: The commission is tasked with preparing regular reports on findings and recommendations, increasing transparency and holding the government accountable for addressing the needs of indigenous communities related to public safety.</t>
+          <t>The benefits of Assembly Concurrent Resolution No. 133, which designates May 2024 as Missing and Murdered Indigenous People Awareness Month in California, include:
+1. **Increased Awareness**: This designation elevates public awareness of the severe issues surrounding missing and murdered Indigenous people, particularly Indigenous women, thereby fostering greater societal recognition and dialogue around the crisis.
+2. **Focus on Data and Research**: By highlighting the lack of comprehensive data on missing and murdered Indigenous individuals, the resolution encourages further investigation and data collection efforts, ultimately contributing to informed policymaking and solutions.
+3. **Legislative Support and Emergency Action**: The resolution urges the Governor to declare a state of emergency, reinforcing the need for immediate attention and resources to address the crisis. This legislative support can lead to more focused initiatives and policies aimed at prevention and intervention.
+4. **Collaboration with Tribal Authorities**: The acknowledgment of laws such as Assembly Bill 1314 (the Feather Alert) and Assembly Bill 44 indicates a commitment to enhancing cooperation between state law enforcement and tribal agencies, facilitating better communication and support for Indigenous communities.
+5. **Community Empowerment**: The resolution serves to empower Indigenous communities by recognizing their struggles, promoting advocacy, and potentially leading to more resources and support for affected families and communities.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>The drawbacks or cons of Enrolled SB 151 include:
-1. **Limited Survivor and Relative Input**: While the legislation mentions the involvement of a victim advocacy organization, there is no explicit provision for direct input from survivors or relatives of missing and murdered indigenous persons, which could limit the responsiveness of the commission and its recommendations.
-2. **Potential for Bureaucratic Delays**: The requirement for the Department of Public Safety to submit reports and conduct needs assessments may introduce delays in addressing urgent cases, which could hinder timely interventions for missing persons.
-3. **Confidentiality Restrictions**: The emphasis on confidentiality and the closed nature of commission meetings may restrict transparency and limit community awareness or involvement in the process, potentially eroding trust between law enforcement and indigenous communities.
-4. **Resource Constraints**: The mandate for increased training and staffing may face challenges related to funding and resources, potentially impacting the effectiveness of the Department of Public Safety and the commission in carrying out their expanded duties.
-5. **Ex Officio Nonvoting Members**: The presence of ex officio nonvoting members from the legislature may dilute the influence of appointed members who are likely to have more direct connections to the indigenous community, leading to a lack of meaningful legislative support for the commission's initiatives.</t>
+          <t>The drawbacks of Assembly Concurrent Resolution No. 133 may include:
+1. **Symbolic Action**: While designating May 2024 as Missing and Murdered Indigenous People Awareness Month raises awareness, it may be perceived as a symbolic gesture without concrete actions or commitments to address the underlying issues systematically. Critics could argue that such initiatives do not lead to immediate changes or resources for affected communities.
+2. **Insufficient Data**: The resolution acknowledges the lack of comprehensive data on missing and murdered Indigenous individuals, particularly those living in urban areas. This gap in data can hinder effective policy development and resource allocation, as decision-makers may not have the necessary information to drive targeted interventions.
+3. **Potential for Overgeneralization**: By focusing extensively on the crisis affecting Indigenous women, there may be a tendency to overlook the broader spectrum of issues impacting Indigenous communities as a whole, including men and non-binary individuals. This narrow focus could alienate certain groups within Indigenous communities who are also affected by violence and systemic injustices.
+4. **Dependence on Legislative Action**: The effectiveness of the resolution relies heavily on subsequent legislative and executive actions, such as the Governor declaring a state of emergency. If these actions do not materialize, the resolution may fail to translate awareness into meaningful change or support for Indigenous communities.
+5. **Lack of Survivor and Community Input**: The text does not indicate that survivors or their families were consulted in the drafting of the resolution. This lack of inclusion could lead to initiatives that do not fully address the needs and perspectives of those directly affected by the crisis.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>The text does not explicitly mention specific mechanisms for evaluation such as a final report, consultation with the community, tribal consultation, a Tribal Crisis Response Plan (TCRP), monitoring, or data collection. While it discusses data on missing and murdered Indigenous individuals, it does not provide a list of mechanisms for evaluation. Therefore, no numbered list can be created from the provided text.</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>1. "The commission shall prepare a report of the commission's findings and recommendations. Not later than January 1 every three years, the commission shall submit the report to the senate secretary and chief clerk of the house of representatives and notify the legislature that the report is available. The commission shall make the report publicly available through the Department of Public Safety."
-2. "The Department of Public Safety shall conduct a needs assessment to determine how to increase protective and investigative resources for identifying and reporting cases of missing and murdered indigenous persons within the state criminal justice system."
-3. "The department shall work with the governor's office to convene meetings with tribal and local law enforcement agencies, federally recognized tribes, and Alaska Native organizations to determine the scope of the issue, identify barriers, and determine methods for creating partnerships to increase reporting and investigation of cases involving missing and murdered indigenous persons."
-4. "The Department of Public Safety shall confer with the commission to establish standardized methods for investigating missing person reports, including for investigating missing persons reports and data collection for cases involving missing indigenous persons."</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>The text uses gender-neutral language by employing terms like "a person," which can refer to individuals of any gender, rather than specifically male or female identifiers. However, when addressing roles and responsibilities, it primarily uses masculine pronouns or titles, such as "commissioner's designee," which may imply a male authority figure. Overall, while there is an effort to be inclusive, there are areas where gender-specific language could be improved for greater inclusivity.</t>
+          <t>The text uses gender-inclusive language primarily by using the term "missing and murdered indigenous people," which encompasses all genders rather than focusing solely on women. However, it frequently cites specific statistics related to Indigenous women, which may inadvertently emphasize gender. Overall, while it includes aspects of gender-inclusivity, the focus on women's experiences in certain sections could lead to a perception of exclusion for other gender identities.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -662,27 +659,27 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>"A person may not be appointed as a police officer, except on a probationary basis, unless the person (1) has satisfactorily completed a basic program of police training approved by the council, which includes at least 12 hours of instruction regarding domestic violence and at least 12 hours of instruction regarding sexual assault, as those terms are defined in AS 18.66.990, [AND] (2) possesses other qualifications the council has established for the employment of police officers, including minimum age, education, physical and mental standards, citizenship, moral character, and experience, and (3) has completed cultural training supervised by an indigenous coordinator or indigenous entity in the state that is related to addressing the rates of missing and murdered indigenous persons."</t>
+          <t>“WHEREAS, In 2022, Governor Newsom signed into law Assembly Bill 1314, the Feather Alert, which is a preventative measure that will be utilized to return missing and endangered indigenous people to their homes;”</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Somewhat. The text includes a provision for a representative from a victim advocacy organization or similar service provider on the Missing and Murdered Indigenous Persons Review Commission, indicating some level of involvement from individuals familiar with the concerns of survivors and relatives. However, there is no mention of direct input or consultation from survivors or relatives themselves, which limits the extent of their involvement and input in the legislative process</t>
+          <t>No. The text does not explicitly mention any input from survivors or relatives of missing and murdered Indigenous people. While it discusses the crisis and acknowledges the importance of the issue, there is no evidence provided that indicates the participation or contributions of those directly affected by the crisis in the legislative process or in shaping the resolution</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Somewhat. The text does include input from Indigenous leaders, as it establishes a Missing and Murdered Indigenous Persons Review Commission that includes representatives from Alaska Native tribal organizations. Additionally, there is a focus on employing individuals to investigate missing and murdered Indigenous persons and acting as liaisons with federally recognized tribes, suggesting a degree of community involvement. However, the specific mechanisms for ongoing community input or decision-making powers for Indigenous communities in the process are not extensively detailed, indicating a somewhat limited level of engagement.</t>
+          <t>Somewhat. The text is sponsored by Rep. James Ramos, an Indigenous politician, which indicates some level of input and representation within the legislative process. However, while the resolution acknowledges the crisis facing Indigenous communities and references actions taken by tribes, it does not provide specific evidence of broader community consultation or involvement. Therefore, while Indigenous representation is present, the extent of input from Indigenous communities is not fully articulated.</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Sen Donald Olson (D) - District SD-T, Sen Elvi Gray-Jackson (D) - District SD-G, Sen Forrest Dunbar (D) - District SD-J, Sen Click Bishop (R) - District SD-R, Rep Matt Claman (D) - District SD-H, Sen Lyman Hoffman (D) - District SD-S, Sen Bert Stedman (R) - District SD-A, Sen Loki Tobin (D) - District SD-I, Sen Robert Myers (R) - District SD-Q, Rep Scott Kawasaki (D) - District SD-P, Sen William Wielechowski (D) - District SD-K, Sen Jesse Kiehl (D) - District SD-B, Sen Gary Stevens (R) - District SD-C, Rep Ashley Carrick (D) - District HD-035, Rep Daniel Ortiz (I) - District HD-001, Rep Sara Hannan (D) - District HD-004, Rep Alyse Galvin (I) - District HD-014, Rep William Fields (D) - District HD-017, Rep Conrad McCormick (D) - District HD-038, Rep Thomas Baker (R) - District HD-040, Rep Jennifer Armstrong (D) - District HD-016, Rep Craig Johnson (R) - District HD-010, Rep Andrew Gray (D) - District HD-020, Rep Donna Mears (D) - District HD-021, Rep Stanley Wright (R) - District HD-022, Rep Andrew Josephson (D) - District HD-013, Rep Genevieve Mina (D) - District HD-019, Rep Calvin Schrage (N) - District HD-012, Rep Cliff Groh (D) - District HD-018, Rep Neal Foster (D) - District HD-039, Rep Bryce Edgmon (I) - District HD-037</t>
+          <t>Rep James Ramos (D) - District HD-045, Rep Dawn Addis (D) - District HD-030, Rep Cecilia Aguiar-Curry (D) - District HD-004, Rep Juan Alanis (R) - District HD-022, Rep David Alvarez (D) - District HD-080, Rep Joaquin Arambula (D) - District HD-031, Rep Jasmeet Bains (D) - District HD-035, Rep Rebecca Bauer-Kahan (D) - District HD-016, Rep Steve Bennett (D) - District HD-038, Rep Marc Berman (D) - District HD-023, Rep Blanca Rubio (D) - District HD-048, Rep Tasha Boerner Horvath (D) - District HD-077, Rep Mia Bonta (D) - District HD-018, Rep Isaac Bryan (D) - District HD-055, Rep Sabrina Cervantes (D) - District HD-058, Rep Phillip Chen (R) - District HD-059, Rep Damon Connolly (D) - District HD-012, Rep Laurie Davies (R) - District HD-074, Rep Diane Dixon (R) - District HD-072, Rep Bill Essayli (R) - District HD-063, Rep Laura Friedman (D) - District HD-044, Rep Jesse Gabriel (D) - District HD-046, Rep James Gallagher (R) - District HD-003, Rep Eduardo Garcia (D) - District HD-036, Rep Mike Gipson (D) - District HD-065, Rep Tim Grayson (D) - District HD-015, Rep Matt Haney (D) - District HD-017, Rep Gregg Hart (D) - District HD-037, Rep Chris Holden (D) - District HD-041, Rep Josh Hoover (R) - District HD-007, Rep Jacqui Irwin (D) - District HD-042, Rep Corey Jackson (D) - District HD-060, Rep Jim Patterson (R) - District HD-008, Rep Joe Patterson (R) - District HD-005, Rep Reginald Jones-Sawyer (D) - District HD-057, Rep Juan Carrillo (D) - District HD-039, Rep Ash Kalra (D) - District HD-025, Rep Tom Lackey (R) - District HD-034, Rep Alex Lee (D) - District HD-024, Rep Josh Lowenthal (D) - District HD-069, Rep Luz Rivas (D) - District HD-043, Rep Brian Maienschein (D) - District HD-076, Rep Kevin McCarty (D) - District HD-006, Rep Tina McKinnor (D) - District HD-061, Rep Mike Fong (D) - District HD-049, Rep Al Muratsuchi (D) - District HD-066, Rep Liz Ortega (D) - District HD-020, Rep Blanca Pacheco (D) - District HD-064, Rep Diane Papan (D) - District HD-021, Rep Gail Pellerin (D) - District HD-028, Rep Cottie Petrie-Norris (D) - District HD-073, Rep Sharon Quirk-Silva (D) - District HD-067, Rep Anthony Rendon (D) - District HD-062, Rep Eloise Reyes (D) - District HD-050, Rep Freddie Rodriguez (D) - District HD-053, Rep Kate Sanchez (R) - District HD-071, Rep Miguel Santiago (D) - District HD-054, Rep Pilar Schiavo (D) - District HD-040, Rep Esmeralda Soria (D) - District HD-027, Rep Stephanie Nguyen (D) - District HD-010, Rep Tri Ta (R) - District HD-070, Rep Philip Ting (D) - District HD-019, Rep Avelino Valencia (D) - District HD-068, Rep Carlos Villapudua (D) - District HD-013, Rep Vince Fong (R) - District HD-032, Rep Marie Waldron (R) - District HD-075, Rep Greg Wallis (R) - District HD-047, Rep Chris Ward (D) - District HD-078, Rep Akilah Weber (D) - District HD-079, Rep Wendy Carrillo (D) - District HD-052, Rep Buffy Wicks (D) - District HD-014, Rep Lori Wilson (D) - District HD-011, Rep Jim Wood (D) - District HD-002, Rep Rick Zbur (D) - District HD-051</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>Sen Donald Olson (D) - District SD-T, Sen Lyman Hoffman (D) - District SD-S, Sen William Wielechowski (D) - District SD-K, Rep William Fields (D) - District HD-017, Rep Thomas Baker (R) - District HD-040, Rep Neal Foster (D) - District HD-039, Rep Bryce Edgmon (I) - District HD-037</t>
+          <t>Rep James Ramos (D) - District HD-045</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -692,17 +689,15 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>The most applicable categories for the provided text are:
-1. Taskforce – The text establishes the Missing and Murdered Indigenous Persons Review Commission, which functions similarly to a task force focused on the issue.
-2. US Law Enforcement – The act includes provisions related to police officer training and the responsibilities of the Department of Public Safety.
-3. Tribal Law Enforcement – The commission includes representation from tribal police officers and aims to act as liaisons between law enforcement agencies and federally recognized tribes.
-4. Data Collection – The act mandates the submission of missing person reports to the National Missing and Unidentified Persons System database and mentions data collection concerning missing indigenous persons. 
-5. MMIP Relatives – There is a reference to involving members from a victim advocacy organization, which typically would be engaged with or representing the interests of relatives of missing and murdered indigenous persons.</t>
+          <t>The most applicable categories for the text are:
+1. **Day of Recognition** - The resolution designates May 2024 as Missing and Murdered Indigenous People Awareness Month.
+2. **Tribal Law Enforcement** - The text references legislation that facilitates access for tribal courts to law enforcement telecommunications systems.
+3. **Data Collection** - It discusses data related to missing and murdered Indigenous people, indicating the importance of data on this issue.</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>2024-10-09</t>
+          <t>2024-05-30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Second successful step in refactoring
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -609,27 +609,27 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Assembly Concurrent Resolution No. 133 designates May 2024 as Missing and Murdered Indigenous People Awareness Month in California and urges the Governor to declare a state of emergency regarding this crisis. The resolution highlights alarming statistics about missing and murdered Indigenous individuals, particularly women, including the high rates of homicide and the lack of comprehensive data on the issue. It references previous legislative efforts, such as the Feather Alert and access to the California Law Enforcement Telecommunications System for Tribal courts, aimed at addressing these concerns. The resolution emphasizes the need for awareness and action to confront the epidemic affecting Indigenous communities, especially given California's significant Indigenous population. Lastly, it calls for the transmission of this resolution to the author for further distribution.</t>
+          <t>Assembly Concurrent Resolution No. 133 designates May 2024 as Missing and Murdered Indigenous People Awareness Month in California and urges the Governor to declare a state of emergency concerning this issue. The resolution highlights alarming statistics, including that homicide is the third leading cause of death among Indigenous women aged 15-24 and that some tribal communities experience murder rates significantly above the national average. It emphasizes the lack of comprehensive data on missing and murdered Indigenous individuals, particularly in urban areas where a significant portion of the Indigenous population resides. The document also cites recent legislative measures aimed at addressing these crises, such as the Feather Alert and enhanced access to law enforcement systems for tribal agencies. Lastly, it calls for the transmission of the resolution to the author for appropriate distribution.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>The benefits of Assembly Concurrent Resolution No. 133, which designates May 2024 as Missing and Murdered Indigenous People Awareness Month in California, include:
-1. **Increased Awareness**: This designation elevates public awareness of the severe issues surrounding missing and murdered Indigenous people, particularly Indigenous women, thereby fostering greater societal recognition and dialogue around the crisis.
-2. **Focus on Data and Research**: By highlighting the lack of comprehensive data on missing and murdered Indigenous individuals, the resolution encourages further investigation and data collection efforts, ultimately contributing to informed policymaking and solutions.
-3. **Legislative Support and Emergency Action**: The resolution urges the Governor to declare a state of emergency, reinforcing the need for immediate attention and resources to address the crisis. This legislative support can lead to more focused initiatives and policies aimed at prevention and intervention.
-4. **Collaboration with Tribal Authorities**: The acknowledgment of laws such as Assembly Bill 1314 (the Feather Alert) and Assembly Bill 44 indicates a commitment to enhancing cooperation between state law enforcement and tribal agencies, facilitating better communication and support for Indigenous communities.
-5. **Community Empowerment**: The resolution serves to empower Indigenous communities by recognizing their struggles, promoting advocacy, and potentially leading to more resources and support for affected families and communities.</t>
+          <t>The designation of May 2024 as Missing and Murdered Indigenous People Awareness Month offers several significant benefits:
+1. **Increased Awareness**: Designating a specific month raises public awareness about the crisis of missing and murdered Indigenous people, drawing attention to the alarming statistics and the urgent need for action.
+2. **Encouragement of Legislative Action**: Urging the Governor to declare a state of emergency can lead to increased governmental focus and resources devoted to addressing this issue, potentially resulting in more effective policies and programs.
+3. **Support for Data Collection**: The resolution highlights existing data gaps, underscoring the importance of improved data collection efforts, which can lead to a better understanding of the crisis affecting Indigenous communities and inform future strategies to combat it.
+4. **Community Empowerment**: By recognizing the crisis faced by Indigenous individuals, the resolution empowers communities, advocates, and allies to rally together for change, promoting solidarity and support for policies that protect Indigenous rights and safety.
+5. **Strengthened Law Enforcement Collaboration**: The resolution indirectly supports recent laws—like Assembly Bill 1314 and Assembly Bill 44—that facilitate better communication and cooperation between law enforcement and tribal agencies, enhancing the effectiveness of responses to missing and murdered cases.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>The drawbacks of Assembly Concurrent Resolution No. 133 may include:
-1. **Symbolic Action**: While designating May 2024 as Missing and Murdered Indigenous People Awareness Month raises awareness, it may be perceived as a symbolic gesture without concrete actions or commitments to address the underlying issues systematically. Critics could argue that such initiatives do not lead to immediate changes or resources for affected communities.
-2. **Insufficient Data**: The resolution acknowledges the lack of comprehensive data on missing and murdered Indigenous individuals, particularly those living in urban areas. This gap in data can hinder effective policy development and resource allocation, as decision-makers may not have the necessary information to drive targeted interventions.
-3. **Potential for Overgeneralization**: By focusing extensively on the crisis affecting Indigenous women, there may be a tendency to overlook the broader spectrum of issues impacting Indigenous communities as a whole, including men and non-binary individuals. This narrow focus could alienate certain groups within Indigenous communities who are also affected by violence and systemic injustices.
-4. **Dependence on Legislative Action**: The effectiveness of the resolution relies heavily on subsequent legislative and executive actions, such as the Governor declaring a state of emergency. If these actions do not materialize, the resolution may fail to translate awareness into meaningful change or support for Indigenous communities.
-5. **Lack of Survivor and Community Input**: The text does not indicate that survivors or their families were consulted in the drafting of the resolution. This lack of inclusion could lead to initiatives that do not fully address the needs and perspectives of those directly affected by the crisis.</t>
+          <t>The designation of May 2024 as Missing and Murdered Indigenous People Awareness Month also presents several drawbacks:
+1. **Limited Immediate Action**: While raising awareness is crucial, the resolution may not lead to immediate, concrete actions or resources to address the issue of missing and murdered Indigenous people, resulting in a sense of urgency that may not be matched by responsive measures.
+2. **Potential for Tokenism**: Designating a month for awareness could be perceived as a token gesture without substantive follow-up, potentially undermining the seriousness of the crisis if it does not lead to systemic changes or long-term commitments to support Indigenous communities.
+3. **Focus on Awareness Rather than Solutions**: By emphasizing awareness over specific strategies and solutions, the resolution may inadvertently divert attention from actionable policies, such as enhanced funding for prevention programs, community support initiatives, or law enforcement accountability measures.
+4. **Data Gaps Remain Unaddressed**: Despite acknowledging the inadequacy of existing data, the resolution may not include mechanisms for improving data collection and analysis, leaving gaps that hinder effective responses to the crisis.
+5. **Risk of Overshadowing Urban Issues**: The focus on missing and murdered Indigenous people may primarily highlight cases on reservations, potentially overshadowing the equally severe issues faced by Indigenous individuals in urban areas, who represent a significant portion of the population experiencing these crises.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -639,24 +639,24 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>The text does not explicitly mention specific mechanisms for evaluation such as a final report, consultation with the community, tribal consultation, a Tribal Crisis Response Plan (TCRP), monitoring, or data collection. While it discusses data on missing and murdered Indigenous individuals, it does not provide a list of mechanisms for evaluation. Therefore, no numbered list can be created from the provided text.</t>
+          <t>The text does not explicitly mention any specific mechanisms for evaluation such as a final report, community consultation, tribal consultation, a Tribal Crisis Response Plan (TCRP), monitoring, or data collection. Therefore, there are no items to list.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>The text primarily focuses on missing and murdered Indigenous women, using specific references to "indigenous women" and their experiences, which may suggest a gender-specific focus rather than a broader inclusion of all genders. However, it does use the term "indigenous people," which encompasses a wider range of individuals, promoting some level of inclusivity. Overall, while it acknowledges the plight of women, it lacks consistent use of gender-neutral language that explicitly includes all genders.</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>The text uses gender-inclusive language primarily by using the term "missing and murdered indigenous people," which encompasses all genders rather than focusing solely on women. However, it frequently cites specific statistics related to Indigenous women, which may inadvertently emphasize gender. Overall, while it includes aspects of gender-inclusivity, the focus on women's experiences in certain sections could lead to a perception of exclusion for other gender identities.</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="S2" t="inlineStr">
         <is>
           <t>“WHEREAS, In 2022, Governor Newsom signed into law Assembly Bill 1314, the Feather Alert, which is a preventative measure that will be utilized to return missing and endangered indigenous people to their homes;”</t>
@@ -664,12 +664,14 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>No. The text does not explicitly mention any input from survivors or relatives of missing and murdered Indigenous people. While it discusses the crisis and acknowledges the importance of the issue, there is no evidence provided that indicates the participation or contributions of those directly affected by the crisis in the legislative process or in shaping the resolution</t>
+          <t>No
+The text does not indicate any direct input from survivors or relatives of missing and murdered Indigenous people. It discusses statistics and legislative actions but lacks references to consultations, testimonies, or specific contributions from those who have experienced this crisis personally. Therefore, there appears to be no engagement with or representation of survivors or their families in the legislative process described</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Somewhat. The text is sponsored by Rep. James Ramos, an Indigenous politician, which indicates some level of input and representation within the legislative process. However, while the resolution acknowledges the crisis facing Indigenous communities and references actions taken by tribes, it does not provide specific evidence of broader community consultation or involvement. Therefore, while Indigenous representation is present, the extent of input from Indigenous communities is not fully articulated.</t>
+          <t>Somewhat
+While the resolution is sponsored by Rep. James Ramos, an Indigenous politician, the text does not provide details about direct input from Indigenous communities or organizations in crafting the legislation. It references the Yurok Tribe's prior declaration of a state of emergency, suggesting some awareness of tribal concerns, but lacks explicit consultation or engagement with various Indigenous communities in California. Thus, there is a moderate level of Indigenous political representation, but not necessarily comprehensive community input reflected in the text.</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -691,8 +693,8 @@
         <is>
           <t>The most applicable categories for the text are:
 1. **Day of Recognition** - The resolution designates May 2024 as Missing and Murdered Indigenous People Awareness Month.
-2. **Tribal Law Enforcement** - The text references legislation that facilitates access for tribal courts to law enforcement telecommunications systems.
-3. **Data Collection** - It discusses data related to missing and murdered Indigenous people, indicating the importance of data on this issue.</t>
+2. **Data Collection** - The text discusses statistics related to missing and murdered indigenous individuals, highlighting the need for better data and addressing gaps in existing information.
+3. **US Law Enforcement** - It mentions actions related to law enforcement, including access to the California Law Enforcement Telecommunications System for tribal courts and agencies.</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">

</xml_diff>

<commit_message>
Third successful refactor step
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -609,27 +609,27 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Assembly Concurrent Resolution No. 133 designates May 2024 as Missing and Murdered Indigenous People Awareness Month in California and urges the Governor to declare a state of emergency concerning this issue. The resolution highlights alarming statistics, including that homicide is the third leading cause of death among Indigenous women aged 15-24 and that some tribal communities experience murder rates significantly above the national average. It emphasizes the lack of comprehensive data on missing and murdered Indigenous individuals, particularly in urban areas where a significant portion of the Indigenous population resides. The document also cites recent legislative measures aimed at addressing these crises, such as the Feather Alert and enhanced access to law enforcement systems for tribal agencies. Lastly, it calls for the transmission of the resolution to the author for appropriate distribution.</t>
+          <t>Assembly Concurrent Resolution No. 133 designates May 2024 as Missing and Murdered Indigenous People Awareness Month in California and urges the Governor to declare a state of emergency regarding the crisis of missing and murdered indigenous people. The resolution highlights significant statistics, including the alarming rates of homicide among indigenous women and the lack of comprehensive data on this issue, especially in urban areas. It notes the importance of recent legislative measures aimed at addressing these challenges, such as the Feather Alert and the facilitation of information sharing among law enforcement and tribal courts. The resolution concludes by mandating the transmittal of copies for appropriate distribution.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>The designation of May 2024 as Missing and Murdered Indigenous People Awareness Month offers several significant benefits:
-1. **Increased Awareness**: Designating a specific month raises public awareness about the crisis of missing and murdered Indigenous people, drawing attention to the alarming statistics and the urgent need for action.
-2. **Encouragement of Legislative Action**: Urging the Governor to declare a state of emergency can lead to increased governmental focus and resources devoted to addressing this issue, potentially resulting in more effective policies and programs.
-3. **Support for Data Collection**: The resolution highlights existing data gaps, underscoring the importance of improved data collection efforts, which can lead to a better understanding of the crisis affecting Indigenous communities and inform future strategies to combat it.
-4. **Community Empowerment**: By recognizing the crisis faced by Indigenous individuals, the resolution empowers communities, advocates, and allies to rally together for change, promoting solidarity and support for policies that protect Indigenous rights and safety.
-5. **Strengthened Law Enforcement Collaboration**: The resolution indirectly supports recent laws—like Assembly Bill 1314 and Assembly Bill 44—that facilitate better communication and cooperation between law enforcement and tribal agencies, enhancing the effectiveness of responses to missing and murdered cases.</t>
+          <t>The benefits of Assembly Concurrent Resolution No. 133 include:
+1. **Raising Awareness**: Designating May 2024 as Missing and Murdered Indigenous People Awareness Month will bring critical attention to the ongoing crisis of missing and murdered Indigenous individuals, particularly women, thereby fostering public awareness and understanding of the issue.
+2. **Encouraging Legislative Action**: By urging the Governor to declare a state of emergency, the resolution aims to mobilize resources, attention, and concerted efforts from government and law enforcement to address the epidemic of violence against Indigenous people.
+3. **Supporting Data Collection and Policy Improvement**: The resolution highlights the inadequacy of existing data on missing and murdered Indigenous people, potentially leading to improved data collection efforts and informed policy-making that can provide better protection and support for Indigenous communities.
+4. **Collaboration with Law Enforcement**: The resolution references recent laws that facilitate greater communication and cooperation between law enforcement agencies and tribal courts, enhancing the effectiveness of responses to missing and murdered Indigenous individuals.
+5. **Fostering Community Empowerment**: By acknowledging the crisis faced by Indigenous people, the resolution may empower communities to advocate for their rights and safety, encouraging engagement and solidarity among Indigenous populations.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>The designation of May 2024 as Missing and Murdered Indigenous People Awareness Month also presents several drawbacks:
-1. **Limited Immediate Action**: While raising awareness is crucial, the resolution may not lead to immediate, concrete actions or resources to address the issue of missing and murdered Indigenous people, resulting in a sense of urgency that may not be matched by responsive measures.
-2. **Potential for Tokenism**: Designating a month for awareness could be perceived as a token gesture without substantive follow-up, potentially undermining the seriousness of the crisis if it does not lead to systemic changes or long-term commitments to support Indigenous communities.
-3. **Focus on Awareness Rather than Solutions**: By emphasizing awareness over specific strategies and solutions, the resolution may inadvertently divert attention from actionable policies, such as enhanced funding for prevention programs, community support initiatives, or law enforcement accountability measures.
-4. **Data Gaps Remain Unaddressed**: Despite acknowledging the inadequacy of existing data, the resolution may not include mechanisms for improving data collection and analysis, leaving gaps that hinder effective responses to the crisis.
-5. **Risk of Overshadowing Urban Issues**: The focus on missing and murdered Indigenous people may primarily highlight cases on reservations, potentially overshadowing the equally severe issues faced by Indigenous individuals in urban areas, who represent a significant portion of the population experiencing these crises.</t>
+          <t>The drawbacks of Assembly Concurrent Resolution No. 133 may include:
+1. **Lack of Concrete Action**: While the resolution designates a month of awareness, it does not outline specific, actionable steps or funding to address the underlying issues of missing and murdered Indigenous people, potentially leading to skepticism about its effectiveness.
+2. **Potential for Tokenism**: The designation of an awareness month without substantial follow-up can be seen as a performative gesture rather than a genuine commitment to enacting change, risking allegations of tokenism from Indigenous communities.
+3. **Inadequate Representation of Urban Issues**: The resolution mentions a significant gap in data regarding Indigenous people living in urban areas, which may perpetuate the marginalization of urban Indigenous populations if their experiences and needs are not adequately addressed.
+4. **Dependence on Government Action**: The call for the Governor to declare a state of emergency may not result in immediate or effective governmental action, leading to frustration among communities seeking more urgent and responsive measures.
+5. **Limited Consultation with Affected Communities**: There is no indication that the resolution involved substantial input from survivors, their families, or Indigenous communities, which could lead to solutions that do not fully align with the needs and priorities of those directly affected by the crisis.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -639,17 +639,17 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>The text does not explicitly mention any specific mechanisms for evaluation such as a final report, community consultation, tribal consultation, a Tribal Crisis Response Plan (TCRP), monitoring, or data collection. Therefore, there are no items to list.</t>
+          <t>The text does not specify any mechanisms for evaluation such as a final report, consultation with community, tribal consultation, a Tribal Crisis Response Plan (TCRP), monitoring, or data collection. Therefore, there are no quoted sections or numbered lists of evaluation mechanisms to provide.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>The text primarily focuses on missing and murdered Indigenous women, using specific references to "indigenous women" and their experiences, which may suggest a gender-specific focus rather than a broader inclusion of all genders. However, it does use the term "indigenous people," which encompasses a wider range of individuals, promoting some level of inclusivity. Overall, while it acknowledges the plight of women, it lacks consistent use of gender-neutral language that explicitly includes all genders.</t>
+          <t>The text employs gender-inclusive language by referring to "indigenous people" rather than specifying gendered terms, thereby encompassing all genders affected by the crisis of missing and murdered individuals. However, it primarily highlights indigenous women and their specific vulnerabilities, which might suggest a partial focus on gender rather than full inclusivity. Overall, while it acknowledges the plight of women, it does use a broader term to address the issue at hand.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -665,13 +665,13 @@
       <c r="T2" t="inlineStr">
         <is>
           <t>No
-The text does not indicate any direct input from survivors or relatives of missing and murdered Indigenous people. It discusses statistics and legislative actions but lacks references to consultations, testimonies, or specific contributions from those who have experienced this crisis personally. Therefore, there appears to be no engagement with or representation of survivors or their families in the legislative process described</t>
+The text does not indicate any input or consultation with survivors or relatives of missing and murdered Indigenous people. It focuses on the statistics and broader issues surrounding the crisis but lacks any mention of involvement or perspectives from those directly impacted by the violence, such as survivors or family members. Without explicit acknowledgment of their voices or experiences, the resolution does not demonstrate any level of input from these individuals</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
           <t>Somewhat
-While the resolution is sponsored by Rep. James Ramos, an Indigenous politician, the text does not provide details about direct input from Indigenous communities or organizations in crafting the legislation. It references the Yurok Tribe's prior declaration of a state of emergency, suggesting some awareness of tribal concerns, but lacks explicit consultation or engagement with various Indigenous communities in California. Thus, there is a moderate level of Indigenous political representation, but not necessarily comprehensive community input reflected in the text.</t>
+While Assembly Concurrent Resolution No. 133 is sponsored by Rep. James Ramos, an Indigenous politician, the text does not explicitly mention input from Indigenous communities or leaders beyond the sponsorship itself. The resolution highlights significant issues faced by Indigenous people, particularly in relation to violence against Indigenous women, but it lacks detailed engagement or consultation mechanisms with Indigenous communities in the decision-making process. Overall, it reflects some acknowledgment of Indigenous issues, but it does not demonstrate robust input or collaboration with the communities it aims to represent.</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -692,9 +692,9 @@
       <c r="Y2" t="inlineStr">
         <is>
           <t>The most applicable categories for the text are:
-1. **Day of Recognition** - The resolution designates May 2024 as Missing and Murdered Indigenous People Awareness Month.
-2. **Data Collection** - The text discusses statistics related to missing and murdered indigenous individuals, highlighting the need for better data and addressing gaps in existing information.
-3. **US Law Enforcement** - It mentions actions related to law enforcement, including access to the California Law Enforcement Telecommunications System for tribal courts and agencies.</t>
+1. **Day of Recognition** - The resolution designates May 2024 as Missing and Murdered Indigenous People Awareness Month, recognizing the issue.
+2. **US Law Enforcement** - The mention of the National Crime Information Center and the need for law enforcement collaboration implies involvement at the federal law enforcement level.
+3. **Data Collection** - The text discusses the lack of comprehensive data on missing and murdered Indigenous people, indicating a need for better data collection efforts.</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">

</xml_diff>

<commit_message>
Initial gov + gpt support
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -563,73 +563,65 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Missing and Murdered Indigenous People Awareness Month.</t>
+          <t>Executive Order</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ACR133</t>
+          <t>Executive Order</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>House</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2024-05-30 - : Chaptered by Secretary of State - Res. Chapter 69, Statutes of 2024.</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>https://legiscan.com/CA/bill/ACR133/2023</t>
-        </is>
-      </c>
+          <t>Executive</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://legiscan.com/CA/bill/ACR133/2023</t>
+          <t>https://azgovernor.gov/office-arizona-governor/executive-order/9</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Assembly Concurrent Resolution No. 133 designates May 2024 as Missing and Murdered Indigenous People Awareness Month in California and urges the Governor to declare a state of emergency regarding the crisis of missing and murdered indigenous individuals. The resolution highlights alarming statistics, including that indigenous women face significantly higher murder rates compared to the national average and that most data on this issue focuses on those living on reservations. It notes that California has the largest population of American Indians and cites recent legislative efforts aimed at addressing the concerns of missing and murdered indigenous people. The resolution reflects ongoing advocacy for improved data collection and response efforts in both urban and rural settings. Finally, it calls for awareness and action in light of the significant impact of this issue on indigenous communities.</t>
+          <t>Executive Order 9, issued by Arizona Governor Katie Hobbs on March 17, 2023, prohibits race-based hair discrimination in employment and education settings. The order highlights the prevalence of such discrimination, particularly affecting Black individuals, especially women, and emphasizes the need for protective policies regarding hair texture and protective hairstyles. It mandates the Department of Administration to create procedures ensuring that discrimination based on hair texture is expressly prohibited across all state agencies and included in state contracts. While the order encourages private employers to adopt similar protections, it does not provide legal rights or remedies to individuals affected by employment decisions. Overall, the initiative aims to foster an inclusive environment where individuals can wear their natural hair without fear of discrimination.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>The benefits or pros of Assembly Concurrent Resolution No. 133 include:
-1. **Increased Awareness**: Designating May 2024 as Missing and Murdered Indigenous People Awareness Month raises public awareness about the critical crisis affecting Indigenous communities, particularly regarding the high rates of violence against Indigenous women.
-2. **Legislative Support**: The resolution urges the Governor to declare a state of emergency, demonstrating political support and prioritization of the issue within the state government, which may lead to further action and resources allocated to address the crisis.
-3. **Data Collection and Resources**: It highlights the need for more comprehensive data collection on missing and murdered Indigenous people, paving the way for better understanding and response to the issue, which is vital for implementing effective preventive measures.
-4. **Collaboration with Law Enforcement**: The recent laws signed by the Governor, such as Assembly Bill 1314 (the Feather Alert) and Assembly Bill 44, facilitate the exchange of information between law enforcement and tribal courts, potentially improving the effectiveness of responses to cases of missing and murdered Indigenous individuals.
-5. **Long-overdue Recognition**: The resolution acknowledges the often-overlooked plight of Indigenous people, particularly those in urban areas, reinforcing the importance of their voices and experiences in conversations about violence and injustice.</t>
+          <t>Executive Order 9 offers several benefits:
+1. **Promotion of Equality**: The order aims to create an inclusive work environment by prohibiting race-based hair discrimination, thereby ensuring that all individuals, particularly Black men, women, and children, can work and learn without fear of being judged or discriminated against based on their natural hair texture or protective styles.
+2. **Workplace Protection**: By mandating that state agencies and contractors implement policies against such discrimination, the order provides a framework that safeguards individuals and helps hold employers accountable for creating fair hiring environments.
+3. **Cultural Recognition**: The order acknowledges and respects the cultural significance of various hairstyles within the Black community, promoting pride in cultural identity and encouraging individuals to express themselves freely without the threat of discrimination.
+4. **Awareness and Policy Change**: It emphasizes the need for awareness and sensitivity regarding hair discrimination, potentially leading to broader societal shifts in the understanding of professionalism and appearance norms, and thereby challenging negative stereotypes.
+5. **Support for State Agencies**: The directive strengthens existing protections and encourages alignment with federal and local laws, fostering consistency in employment practices regarding race-based discrimination across state agencies.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>The drawbacks or cons of Assembly Concurrent Resolution No. 133 include:
-1. **Lack of Concrete Action**: While the resolution promotes awareness and calls for a state of emergency, it may fall short of establishing actionable steps to effectively address the crisis of missing and murdered Indigenous people. Without a detailed plan, there is a risk that this recognition will not translate into substantial policy changes or resource allocation.
-2. **Data Limitations**: The resolution acknowledges that little data exists on the epidemic of missing and murdered Indigenous people, particularly in urban areas. This lack of comprehensive data could hinder effective responses and creates challenges in understanding the full scope of the issue, potentially leading to misinformed policies.
-3. **Potential for Insufficient Community Engagement**: The resolution does not explicitly mention the involvement of Indigenous community members, survivors, or their families in the development of this measure. This lack of direct input may lead to a disconnect between the legislative intent and the actual needs and concerns of those most affected by the crisis.
-4. **Temporary Recognition**: Designating a month for awareness may be seen as a symbolic gesture rather than a sustained commitment to address the underlying issues contributing to violence against Indigenous people. This could result in short-term attention without lasting impact or ongoing support.
-5. **Focus on Women Alone**: While it rightly highlights the disproportionately high violence against Indigenous women, the resolution may inadvertently exclude discussions on the broader spectrum of violence affecting Indigenous men, youth, and non-binary individuals, limiting the inclusivity of the awareness effort.</t>
+          <t>Executive Order 9 has several potential drawbacks:
+1. **Limited Scope**: The order does not apply to all state governmental entities or offices headed by statewide elected officials, which may create inconsistencies in the application of anti-discrimination policies across various sectors of state employment. This exclusion could leave gaps in protections for certain employees.
+2. **Lack of Legal Recourse**: The order explicitly states that it does not confer any legal rights or remedies upon individuals, meaning that affected persons may have limited ability to challenge discriminatory practices or seek legal redress. This lack of enforceability could undermine the effectiveness of the order.
+3. **Potential Resistance**: The implementation of policies that prohibit discrimination based on hair texture and protective styles may face resistance from some employers or institutions that are accustomed to traditional standards of professionalism, potentially leading to pushback or conflict within workplaces.
+4. **Implementation Challenges**: The requirement for state agencies to establish procedures by a specific deadline may not be adequately supported by resources or training, resulting in inconsistencies in how policies are enforced or understood across different agencies.
+5. **Cultural Resistance**: While the order promotes cultural expression, there may still be societal or institutional resistance to changing perceptions of professionalism related to hair, which could limit the effectiveness of the order in changing attitudes and behaviors in the workplace.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -639,7 +631,8 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>The text does not specify any mechanisms for evaluation such as a final report, consultation with the community, tribal consultation, a Tribal Crisis Response Plan (TCRP), monitoring, or data collection. Therefore, there are no mechanisms to list.</t>
+          <t>The text does not explicitly mention any specific mechanisms for evaluation such as a final report, consultation with the community, tribal consultation, a Tribal Crisis Response Plan (TCRP), monitoring, or data collection. Therefore, there are no quotes to provide that list mechanisms from the Executive Order. 
+If you would like to know more about the content or terms used in the text, feel free to ask!</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -649,58 +642,51 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>The text uses gender-inclusive language by explicitly addressing "missing and murdered indigenous people," which encompasses individuals of all genders rather than focusing solely on women. Additionally, it reports on the specific impact of violence against indigenous women but also acknowledges that the issue affects a broader population, including indigenous men and non-binary individuals. Overall, the language aims to encompass the entire indigenous community impacted by this crisis.</t>
+          <t>The text uses gender-inclusive language by specifically mentioning "Black women, men, and children," ensuring representation of diverse gender identities. It addresses discrimination in a manner that acknowledges and validates the experiences of individuals across different gender identities without being exclusive. Additionally, it promotes a broader understanding of discrimination that impacts various groups, thus fostering an inclusive environment.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>**"WHEREAS, In 2022, Governor Newsom signed into law Assembly Bill 1314, the Feather Alert, which is a preventative measure that will be utilized to return missing and endangered indigenous people to their homes;"**</t>
+          <t>No.</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>No.
-The text does not indicate any involvement or input from survivors or relatives of missing and murdered Indigenous people. While it addresses the issue critically, the absence of direct representation or consultation with those affected suggests a lack of engagement with the voices of survivors and their families in this legislative measure. Without evidence of survivor input or their acknowledgment in the resolution, the level of input is effectively nonexistent</t>
+          <t>No. 
+The text does not indicate any direct input or consultation from survivors or relatives regarding the issues addressed in the Executive Order related to race-based hair discrimination. It largely presents statistical findings and statements about the experiences of Black individuals without including personal testimonies or perspectives from those directly affected. As such, there is no evident engagement with the voices of survivors or their families in shaping the order or its provisions</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Somewhat. 
-The text is sponsored by Rep. James Ramos, an Indigenous politician, which indicates some level of input from Indigenous leadership in the legislative process. However, the resolution does not explicitly mention consultations with Indigenous communities or provide evidence of broader community engagement in developing this measure, making it difficult to assess the depth of input from Indigenous communities. While the focus is on a critical issue affecting Indigenous peoples, the absence of stated collaboration with community members or organizations suggests that their input may be limited.</t>
+          <t>No. 
+The text does not mention any input or involvement from Indigenous politicians or communities regarding the Executive Order. It primarily focuses on issues of race-based hair discrimination affecting Black individuals without addressing the perspectives or contributions of Indigenous groups. As a result, there appears to be a lack of representation or acknowledgment of Indigenous stakeholders in this context.</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Rep James Ramos (D) - District HD-045, Rep Dawn Addis (D) - District HD-030, Rep Cecilia Aguiar-Curry (D) - District HD-004, Rep Juan Alanis (R) - District HD-022, Rep David Alvarez (D) - District HD-080, Rep Joaquin Arambula (D) - District HD-031, Rep Jasmeet Bains (D) - District HD-035, Rep Rebecca Bauer-Kahan (D) - District HD-016, Rep Steve Bennett (D) - District HD-038, Rep Marc Berman (D) - District HD-023, Rep Blanca Rubio (D) - District HD-048, Rep Tasha Boerner Horvath (D) - District HD-077, Rep Mia Bonta (D) - District HD-018, Rep Isaac Bryan (D) - District HD-055, Rep Sabrina Cervantes (D) - District HD-058, Rep Phillip Chen (R) - District HD-059, Rep Damon Connolly (D) - District HD-012, Rep Laurie Davies (R) - District HD-074, Rep Diane Dixon (R) - District HD-072, Rep Bill Essayli (R) - District HD-063, Rep Laura Friedman (D) - District HD-044, Rep Jesse Gabriel (D) - District HD-046, Rep James Gallagher (R) - District HD-003, Rep Eduardo Garcia (D) - District HD-036, Rep Mike Gipson (D) - District HD-065, Rep Tim Grayson (D) - District HD-015, Rep Matt Haney (D) - District HD-017, Rep Gregg Hart (D) - District HD-037, Rep Chris Holden (D) - District HD-041, Rep Josh Hoover (R) - District HD-007, Rep Jacqui Irwin (D) - District HD-042, Rep Corey Jackson (D) - District HD-060, Rep Jim Patterson (R) - District HD-008, Rep Joe Patterson (R) - District HD-005, Rep Reginald Jones-Sawyer (D) - District HD-057, Rep Juan Carrillo (D) - District HD-039, Rep Ash Kalra (D) - District HD-025, Rep Tom Lackey (R) - District HD-034, Rep Alex Lee (D) - District HD-024, Rep Josh Lowenthal (D) - District HD-069, Rep Luz Rivas (D) - District HD-043, Rep Brian Maienschein (D) - District HD-076, Rep Kevin McCarty (D) - District HD-006, Rep Tina McKinnor (D) - District HD-061, Rep Mike Fong (D) - District HD-049, Rep Al Muratsuchi (D) - District HD-066, Rep Liz Ortega (D) - District HD-020, Rep Blanca Pacheco (D) - District HD-064, Rep Diane Papan (D) - District HD-021, Rep Gail Pellerin (D) - District HD-028, Rep Cottie Petrie-Norris (D) - District HD-073, Rep Sharon Quirk-Silva (D) - District HD-067, Rep Anthony Rendon (D) - District HD-062, Rep Eloise Reyes (D) - District HD-050, Rep Freddie Rodriguez (D) - District HD-053, Rep Kate Sanchez (R) - District HD-071, Rep Miguel Santiago (D) - District HD-054, Rep Pilar Schiavo (D) - District HD-040, Rep Esmeralda Soria (D) - District HD-027, Rep Stephanie Nguyen (D) - District HD-010, Rep Tri Ta (R) - District HD-070, Rep Philip Ting (D) - District HD-019, Rep Avelino Valencia (D) - District HD-068, Rep Carlos Villapudua (D) - District HD-013, Rep Vince Fong (R) - District HD-032, Rep Marie Waldron (R) - District HD-075, Rep Greg Wallis (R) - District HD-047, Rep Chris Ward (D) - District HD-078, Rep Akilah Weber (D) - District HD-079, Rep Wendy Carrillo (D) - District HD-052, Rep Buffy Wicks (D) - District HD-014, Rep Lori Wilson (D) - District HD-011, Rep Jim Wood (D) - District HD-002, Rep Rick Zbur (D) - District HD-051</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>Rep James Ramos (D) - District HD-045</t>
-        </is>
-      </c>
+          <t>Executive Order</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2023-2024 Regular Session</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>The most applicable categories for the text are:
-1. Day of Recognition
-2. Data Collection
-3. Tribal Law Enforcement
-This resolution designates May 2024 as Missing and Murdered Indigenous People Awareness Month, serving as a day of recognition for the ongoing crisis. It also addresses data collection issues related to missing and murdered Indigenous people, indicating that existing data is incomplete and inadequate. Additionally, it includes provisions for facilitating information exchange between tribal courts and law enforcement agencies, linking it to tribal law enforcement efforts.</t>
+          <t>No applicable categories.
+The text focuses on prohibiting race-based hair discrimination and does not mention any elements related to a taskforce, day of recognition, US law enforcement, tribal law enforcement, data collection, or MMIP relatives. It primarily addresses workplace policies and protections regarding discrimination based on hair texture and protective styles.</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>2024-05-30</t>
+          <t>2024-10-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sucessfully integrated gov processor
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -595,59 +595,76 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://azgovernor.gov/office-arizona-governor/executive-order/9</t>
+          <t>https://www.govinfo.gov/content/pkg/FR-2019-12-02/pdf/2019-26178.pdf</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Executive Order 9, issued by Arizona Governor Katie Hobbs on March 17, 2023, prohibits race-based hair discrimination in employment and education settings. The order highlights the prevalence of such discrimination, particularly affecting Black individuals, especially women, and emphasizes the need for protective policies regarding hair texture and protective hairstyles. It mandates the Department of Administration to create procedures ensuring that discrimination based on hair texture is expressly prohibited across all state agencies and included in state contracts. While the order encourages private employers to adopt similar protections, it does not provide legal rights or remedies to individuals affected by employment decisions. Overall, the initiative aims to foster an inclusive environment where individuals can wear their natural hair without fear of discrimination.</t>
+          <t>Executive Order 13898, signed on November 26, 2019, establishes the Task Force on Missing and Murdered American Indians and Alaska Natives to address the critical concerns of these communities, particularly regarding missing and murdered Indigenous women and girls. The Task Force, co-chaired by the Attorney General and the Secretary of the Interior, will coordinate with tribal governments and federal officials to improve the criminal justice response to these issues. Its mission includes conducting consultations, developing model protocols for handling cases, and enhancing cooperation among various law enforcement agencies. The Task Force is required to submit progress reports to the President within one and two years after its establishment. The order emphasizes that the Task Force will terminate two years from its signing unless otherwise directed and does not create enforceable rights against the government.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Executive Order 9 offers several benefits:
-1. **Promotion of Equality**: The order aims to create an inclusive work environment by prohibiting race-based hair discrimination, thereby ensuring that all individuals, particularly Black men, women, and children, can work and learn without fear of being judged or discriminated against based on their natural hair texture or protective styles.
-2. **Workplace Protection**: By mandating that state agencies and contractors implement policies against such discrimination, the order provides a framework that safeguards individuals and helps hold employers accountable for creating fair hiring environments.
-3. **Cultural Recognition**: The order acknowledges and respects the cultural significance of various hairstyles within the Black community, promoting pride in cultural identity and encouraging individuals to express themselves freely without the threat of discrimination.
-4. **Awareness and Policy Change**: It emphasizes the need for awareness and sensitivity regarding hair discrimination, potentially leading to broader societal shifts in the understanding of professionalism and appearance norms, and thereby challenging negative stereotypes.
-5. **Support for State Agencies**: The directive strengthens existing protections and encourages alignment with federal and local laws, fostering consistency in employment practices regarding race-based discrimination across state agencies.</t>
+          <t>Yes. 
+Here are the specific prevention efforts identified in the text:
+1. **Education and Outreach Campaign**: "The Task Force shall... develop and execute an education and outreach campaign for communities that are most affected by crime against American Indians and Alaska Natives to identify and reduce such crime."
+2. **Public Awareness Campaign**: "Developing, in partnership with NamUs, a public-awareness campaign to educate both rural and urban communities about the needs of affected families and resources that are both needed and available."
+3. **Best-Practices Guidance**: "The Task Force shall... develop and publish best-practices guidance for use by Federal, State, local, and tribal law enforcement in cases involving missing and murdered American Indians and Alaska Natives, to include best practices related to communication with affected families from initiation of an investigation through case resolution or closure."
+These efforts emphasize a proactive approach to improving awareness, responses, and preventative strategies regarding violence against Indigenous communities.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Executive Order 9 has several potential drawbacks:
-1. **Limited Scope**: The order does not apply to all state governmental entities or offices headed by statewide elected officials, which may create inconsistencies in the application of anti-discrimination policies across various sectors of state employment. This exclusion could leave gaps in protections for certain employees.
-2. **Lack of Legal Recourse**: The order explicitly states that it does not confer any legal rights or remedies upon individuals, meaning that affected persons may have limited ability to challenge discriminatory practices or seek legal redress. This lack of enforceability could undermine the effectiveness of the order.
-3. **Potential Resistance**: The implementation of policies that prohibit discrimination based on hair texture and protective styles may face resistance from some employers or institutions that are accustomed to traditional standards of professionalism, potentially leading to pushback or conflict within workplaces.
-4. **Implementation Challenges**: The requirement for state agencies to establish procedures by a specific deadline may not be adequately supported by resources or training, resulting in inconsistencies in how policies are enforced or understood across different agencies.
-5. **Cultural Resistance**: While the order promotes cultural expression, there may still be societal or institutional resistance to changing perceptions of professionalism related to hair, which could limit the effectiveness of the order in changing attitudes and behaviors in the workplace.</t>
+          <t>The drawbacks or cons of Executive Order 13898 can be summarized as follows:
+1. **Limited Authority and Enforceability**: The Executive Order states that it does not create any enforceable rights or benefits. This limitation may weaken its impact, as individuals and communities affected by the crisis of missing and murdered Indigenous individuals may lack legal recourse to hold authorities accountable for inaction or mishandling of cases.
+2. **Temporal Constraints**: The Task Force is set to terminate two years after its establishment unless extended by the President. This time limitation could restrict the ability to create long-term solutions and may lead to inadequate follow-through on developing effective policies and practices.
+3. **Potential for Insufficient Community Engagement**: Although the Task Force includes consultations with tribal governments, there is no explicit provision for sustained engagement with survivors or their families. This lack of focus on those directly impacted by the crisis might result in strategies that do not adequately reflect the needs and perspectives of affected individuals. 
+4. **Dependence on Coordination Among Agencies**: The effectiveness of the Task Force is contingent on the cooperation of multiple federal, state, and tribal law enforcement agencies. Variability in commitment or coordination may hinder its effectiveness and the implementation of comprehensive strategies to address these issues. 
+These drawbacks indicate challenges that may affect the overall effectiveness of the Task Force and its ability to address the critical issues facing Indigenous communities regarding missing and murdered individuals.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes. 
+Here are the identified prevention efforts from the text:
+1. **Education and Outreach Campaign**: "The Task Force shall... develop and execute an education and outreach campaign for communities that are most affected by crime against American Indians and Alaska Natives to identify and reduce such crime."
+2. **Public Awareness Campaign**: "Developing, in partnership with NamUs, a public-awareness campaign to educate both rural and urban communities about the needs of affected families and resources that are both needed and available."
+3. **Best-Practices Guidance**: "The Task Force shall... develop and publish best-practices guidance for use by Federal, State, local, and tribal law enforcement in cases involving missing and murdered American Indians and Alaska Natives, to include best practices related to communication with affected families from initiation of an investigation through case resolution or closure."
+These efforts emphasize proactive approaches to raising awareness, improving law enforcement responses, and ultimately preventing incidents of missing and murdered individuals in these communities</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>The text does not explicitly mention any specific mechanisms for evaluation such as a final report, consultation with the community, tribal consultation, a Tribal Crisis Response Plan (TCRP), monitoring, or data collection. Therefore, there are no quotes to provide that list mechanisms from the Executive Order. 
-If you would like to know more about the content or terms used in the text, feel free to ask!</t>
+          <t>Here are the mechanisms for evaluation mentioned in the text:
+1. **Consultation with Tribal Governments**: "The Task Force shall conduct appropriate consultations with tribal governments on the scope and nature of the issues regarding missing and murdered American Indians and Alaska Natives."
+2. **Data Collection**: "The Task Force shall develop model protocols and procedures to apply to new and unsolved cases of missing or murdered persons in American Indian and Alaska Native communities, including best practices for: (B) collecting and sharing data among various jurisdictions and law enforcement agencies."
+3. **Reporting**:
+   - "(a) No later than 1 year after the date of this order, the Task Force shall develop and submit to the President... a written report regarding the activities and accomplishments of the Task Force, the status of projects the Task Force has not yet completed, and specific recommendations for future action of the Task Force."
+   - "(b) No later than 2 years after the date of this order, the Task Force shall develop and submit to the President... a final written report regarding the activities and accomplishments of the Task Force."
+4. **Review Processes**: "(ii) develop model protocols and procedures to apply to new and unsolved cases of missing or murdered persons in American Indian and Alaska Native communities... including best practices for... (iii) establish a multi-disciplinary, multi-jurisdictional team including representatives from tribal law enforcement and the Departments of Justice and the Interior to review cold cases involving missing and murdered American Indians and Alaska Natives."
+These mechanisms show a structured approach to evaluation through reporting and consultations, along with an emphasis on data collection and reviews of specific cases.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No. 
+The text does not explicitly mention any prevention efforts related to training or awareness efforts. While it discusses the establishment of a Task Force and outlines its mission and functions, such as conducting consultations and developing model protocols, it does not detail specific training initiatives or awareness campaigns focusing on preventing future incidents of missing and murdered Indigenous individuals</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>The text uses gender-inclusive language by specifically mentioning "Black women, men, and children," ensuring representation of diverse gender identities. It addresses discrimination in a manner that acknowledges and validates the experiences of individuals across different gender identities without being exclusive. Additionally, it promotes a broader understanding of discrimination that impacts various groups, thus fostering an inclusive environment.</t>
+          <t>The text does not fully use gender-inclusive language. While it specifically addresses "missing and murdered indigenous women and girls," this focus on women and girls means that other genders are not acknowledged in the context of missing and murdered cases. Although the task force aims to address the concerns of American Indian and Alaska Native communities broadly, the language employed highlights specific demographic groups and does not utilize more inclusive terms that encompass all genders.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes. 
+Here are the specific prevention efforts identified in the text:
+1. **Education and Outreach Campaign**: "The Task Force shall... develop and execute an education and outreach campaign for communities that are most affected by crime against American Indians and Alaska Natives to identify and reduce such crime."
+2. **Public Awareness Campaign**: "Developing, in partnership with NamUs, a public-awareness campaign to educate both rural and urban communities about the needs of affected families and resources that are both needed and available."
+3. **Best-Practices Guidance**: "The Task Force shall... develop and publish best-practices guidance for use by Federal, State, local, and tribal law enforcement in cases involving missing and murdered American Indians and Alaska Natives, to include best practices related to communication with affected families from initiation of an investigation through case resolution or closure."
+These efforts indicate a proactive approach to improving awareness, responses, and preventative strategies regarding violence against Indigenous communities</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -657,14 +674,13 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>No. 
-The text does not indicate any direct input or consultation from survivors or relatives regarding the issues addressed in the Executive Order related to race-based hair discrimination. It largely presents statistical findings and statements about the experiences of Black individuals without including personal testimonies or perspectives from those directly affected. As such, there is no evident engagement with the voices of survivors or their families in shaping the order or its provisions</t>
+          <t>Somewhat.
+The text mentions the need for consultations with tribal governments regarding missing and murdered American Indians and Alaska Natives, which indicates some level of input from Indigenous communities. However, it does not specify the extent to which survivors or relatives of victims will be involved in the process or decision-making of the Task Force, leading to a limited evaluation of their input. The language implies engagement but does not explicitly detail mechanisms for incorporating the voices and experiences of survivors and families directly affected by these issues</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>No. 
-The text does not mention any input or involvement from Indigenous politicians or communities regarding the Executive Order. It primarily focuses on issues of race-based hair discrimination affecting Black individuals without addressing the perspectives or contributions of Indigenous groups. As a result, there appears to be a lack of representation or acknowledgment of Indigenous stakeholders in this context.</t>
+          <t>No.</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -680,8 +696,13 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>No applicable categories.
-The text focuses on prohibiting race-based hair discrimination and does not mention any elements related to a taskforce, day of recognition, US law enforcement, tribal law enforcement, data collection, or MMIP relatives. It primarily addresses workplace policies and protections regarding discrimination based on hair texture and protective styles.</t>
+          <t>The most applicable categories for the text are:
+1. **Taskforce** - The establishment of the Task Force on Missing and Murdered American Indians and Alaska Natives is a central focus of the Executive Order.
+2. **US Law Enforcement** - The text discusses the involvement of various federal law enforcement agencies and the improvement of responses to cases.
+3. **Tribal Law Enforcement** - The Task Force includes representatives from tribal law enforcement, emphasizing collaboration with Indigenous communities.
+4. **Data Collection** - The order outlines the need for collecting and sharing data among various law enforcement agencies and better utilization of existing criminal databases.
+5. **MMIP Relatives** - The document mentions best-practices guidance related to communication with affected families, indicating concern for the needs of relatives of missing and murdered individuals.
+The text does not fit the "Day of Recognition" category as it does not mention a specific day dedicated to awareness or remembrance.</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">

</xml_diff>

<commit_message>
Converted pros and cons to numbered list
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -578,21 +578,29 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Executive</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+          <t>Senate</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2024-10-09 - S: EFFECTIVE DATE(S) OF LAW 1/1/25</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://legiscan.com/AK/bill/SB151/2023</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>https://www.govinfo.gov/content/pkg/FR-2021-11-18/pdf/2021-25287.pdf</t>
@@ -601,17 +609,27 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Executive Order 14053, issued on November 15, 2021, aims to improve public safety and criminal justice for Native Americans while addressing the crisis of missing or murdered Indigenous people. The order emphasizes collaboration with Tribal Nations to develop comprehensive law enforcement strategies, support services, and systems for data collection and analysis related to violence against Native Americans. It outlines mechanisms for enhancing grants and training for Tribal law enforcement, improving victim services, and increasing the effectiveness of reporting and intervention efforts. Additionally, the order reinforces the necessity for ongoing consultation with Tribal communities to ensure their needs are prioritized. Overall, it seeks to address the high rates of violence faced by Native Americans and improve their overall safety and well-being.</t>
+          <t>Executive Order 14053, issued on November 15, 2021, prioritizes the safety and well-being of Native Americans and addresses the crisis of missing and murdered indigenous people. It mandates a coordinated federal law enforcement strategy to prevent and respond to violence against Native Americans, emphasizing collaboration with Tribal Nations and community organizations. The order outlines measures for improving data collection, analysis, and information sharing regarding crimes against Native Americans, as well as enhancing support services for victims. It also emphasizes the importance of engaging with Native American communities to gather input and recommendations for implementing the order's provisions. Additionally, the order reaffirms the federal government's commitment to long-term resource allocation to address the underlying causes of violence against Native Americans.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Executive Order 14053 offers several benefits aimed at improving public safety and addressing the crisis of missing or murdered Indigenous people. It fosters collaboration with Tribal Nations to develop comprehensive law enforcement strategies, enhancing support services and ensuring that the specific needs of Native American communities are prioritized. The legislation promotes gender-inclusive language and acknowledges the diverse experiences of Indigenous people, including LGBTQ+ individuals and Two-Spirit people, thus creating a more inclusive approach to addressing violence. It includes mechanisms for ongoing evaluation and data collection, allowing for informed decisions and better resource allocation. The prevention efforts outlined in the order aim to reduce risk factors for victimization while improving mental health, substance abuse services, and overall community resilience. By centering Indigenous voices through consultations and the establishment of a Joint Commission, the legislation ensures that those directly affected by the issues have a say in the solutions that are developed. Overall, it seeks to create safer communities and enhance the well-being of Native Americans.</t>
+          <t xml:space="preserve">1. Prioritizes the safety and well-being of Native Americans by addressing the crisis of missing and murdered indigenous people through a comprehensive federal strategy.  
+2. Mandates coordination between federal, state, and tribal law enforcement to enhance prevention and response efforts, improving public safety in indigenous communities.  
+3. Improves data collection and analysis efforts to better understand the prevalence and causes of violence against Native Americans, aiding in effective policymaking.  
+4. Strengthens community engagement by involving Tribal Nations and organizations in the decision-making process, ensuring that local needs and solutions are prioritized.  
+5. Establishes prevention strategies and support services aimed at reducing risk factors for victimization and providing resources for victims and their families.  
+6. Committed to long-term resource allocation, ensuring sustained efforts to tackle the high rates of violence that Native Americans experience over time.  </t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>While Executive Order 14053 presents several benefits, there are also potential drawbacks or challenges associated with its implementation. One concern is that the effectiveness of the order heavily relies on adequate funding and resources, which may not be guaranteed or sustainable over time. Additionally, the complexity of jurisdictional issues in law enforcement on Tribal lands can complicate the coordination of efforts between federal, state, and Tribal authorities, potentially leading to gaps in accountability or effectiveness. Furthermore, while the legislation emphasizes consultation with Indigenous communities, the actual engagement process may vary in effectiveness, and if not managed properly, it could lead to tokenism rather than meaningful involvement. Lastly, there is a risk that the order's objectives may be undermined if there is insufficient political will or support from both federal and local entities to address the underlying systemic issues contributing to violence against Native Americans.</t>
+          <t xml:space="preserve">1. While the executive order establishes a Joint Commission, it does not guarantee direct and meaningful involvement from MMIP survivors or relatives of victims, which could limit representation of those most impacted.  
+2. The effectiveness of the implemented measures depends on long-term commitment and resource allocation, which may not always be assured or consistent.  
+3. The coordination among various federal and tribal agencies may face bureaucratic challenges that hinder timely responses to the crisis of missing and murdered indigenous people.  
+4. Although the order promotes data collection and analysis, the success of these efforts relies on the cooperation of various agencies, and existing gaps in data may remain unresolved.  
+5. The order calls for various assessments and reporting requirements, which could lead to delays in the implementation of necessary actions and policies due to extended timelines.  
+6. There may be inequities in funding or support for urban Native Americans compared to those living on Tribal lands, potentially leaving some communities underserved.  </t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -621,11 +639,11 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>1. **Report on the Strategy Developed**: "The Attorney General and the Secretary of the Interior shall report to the President within 240 days of the date of this order describing the strategy developed and identifying additional resources or other support necessary to implement that strategy."
-2. **Report on Ongoing Analysis of Data**: "Within 240 days of the date of this order, the Attorney General, the Secretary of the Interior, and the Secretary of HHS shall report jointly to the President on the strategy they have developed to conduct and coordinate that analysis and shall identify additional resources or other support necessary to implement that strategy."
-3. **Assessment of Current Use of DNA Testing**: "Within 240 days of the date of this order, the Attorney General shall report the outcome of this assessment to the President, along with recommendations to improve the use and accessibility of DNA database services."
-4. **Evaluation of Research and Data Collection Efforts**: "The Secretary of HHS shall report to the President within 180 days of the date of this order on those findings and any planned changes to improve those research and data collection efforts."
-5. **Evaluation Findings and Improvements**: "The Secretary of the Interior shall report to the President within 180 days of the date of this order describing the evaluation findings and the improvements implemented."</t>
+          <t xml:space="preserve">1. "The Attorney General and the Secretary of the Interior shall report to the President within 240 days of the date of this order describing the strategy developed and identifying additional resources or other support necessary to implement that strategy."  
+2. "The Secretary of HHS shall report to the President within 240 days of the date of this order describing the plan and actions taken and identifying any additional resources or other support needed."  
+3. "The Attorney General, in coordination with the Secretary of the Interior and the Secretary of HHS, shall develop a strategy for ongoing analysis of data collected on violent crime and missing persons involving Native Americans, including in urban Indian communities, to better understand the extent and causes of this crisis."  
+4. "The Secretary of HHS shall evaluate the adequacy of research and data collection efforts at the Centers for Disease Control and Prevention and the National Institutes of Health in accurately measuring the prevalence and effects of violence against Native Americans, especially those living in urban areas, and report to the President within 180 days of the date of this order on those findings and any planned changes to improve those research and data collection efforts."  
+5. "The Attorney General shall assess the current use of DNA testing and DNA database services to identify missing or murdered indigenous people and any responsible parties, including the unidentified human remains, missing persons, and relatives of missing persons indices of the Combined DNA Index System and the National Missing and Unidentified Persons System."  </t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -635,7 +653,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>The legislation utilizes gender-inclusive language by addressing the crisis of missing or murdered Indigenous people rather than exclusively focusing on women. It acknowledges the disproportionate violence faced by Native American women while also recognizing that LGBTQ+ Native Americans and Two-Spirit individuals are also targets of violence. This broader terminology reflects an understanding of the diverse experiences within Indigenous communities and supports a more inclusive approach to addressing these issues.</t>
+          <t>The legislation uses the term "missing or murdered indigenous people," which encompasses individuals of all genders, thereby broadening the focus beyond just women. It highlights the prevalent violence faced by Native Americans, including LGBTQ+ and Two-Spirit individuals, implicitly acknowledging the diverse experiences within indigenous communities. By employing inclusive language, the order promotes a comprehensive understanding of the crisis affecting all members of these communities.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -645,29 +663,33 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>The legislation outlines several prevention efforts regarding Missing and Murdered Indigenous Persons. Here are relevant quotes from the text:
-1. "The [Secretary of HHS] shall develop a comprehensive plan to support prevention efforts that reduce risk factors for victimization of Native Americans and increase protective factors, including by enhancing the delivery of services for Native American victims and survivors, as well as their families and advocates."
-2. "The plan shall include strategies for improving mental and behavioral health; providing substance abuse services; providing family support, including high-quality early childhood programs for victims and survivors with young children; and preventing elder abuse, gender-based violence, and human trafficking."
-3. "Strategies to encourage culturally and linguistically appropriate, trauma-informed, and victim-centered service delivery to Native Americans, including for survivors of gender-based violence."
-These quotes indicate proactive measures aimed at prevention and service delivery for affected individuals and communities.</t>
+          <t>The legislation includes the following prevention efforts:
+1. "My Administration will work hand in hand with Tribal Nations and Tribal partners to build safe and healthy Tribal communities and to support comprehensive law enforcement, prevention, intervention, and support services."
+2. "The Secretary of HHS...shall develop a comprehensive plan to support prevention efforts that reduce risk factors for victimization of Native Americans and increase protective factors."
+3. "The plan shall include strategies for improving mental and behavioral health; providing substance abuse services; providing family support, including high-quality early childhood programs for victims and survivors with young children; and preventing elder abuse, gender-based violence, and human trafficking."
+These quotes indicate efforts aimed at preventing violence and enhancing support for Native American communities in relation to missing and murdered Indigenous persons.</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Somewhat</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Yes. The legislation emphasizes the importance of engaging and consulting with Native American communities, including survivors of violence and their families. It specifically mentions that "consistent engagement, commitment, and collaboration will drive long-term improvement to public safety for all Native Americans," indicating a recognition of the need for input from those directly affected by the crisis. Additionally, the establishment of a Joint Commission that includes representatives from various stakeholder groups further demonstrates a commitment to incorporating perspectives from Indigenous politicians and communities.</t>
+          <t>Yes. The executive order establishes a Joint Commission that includes various stakeholders such as Tribal leaders, representatives from Tribal, State, and local law enforcement, and Native American survivors of human trafficking, indicating the inclusion of diverse voices and perspectives. It aims to address the crisis of missing or murdered indigenous people by incorporating feedback from affected communities and promoting collaboration for effective solutions. Additionally, the order emphasizes the importance of direct engagement with Tribal Nations and Native American communities to inform strategies and implementation efforts.</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Executive Order</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr"/>
+          <t>Sen Donald Olson (D) - District SD-T, Sen Elvi Gray-Jackson (D) - District SD-G, Sen Forrest Dunbar (D) - District SD-J, Sen Click Bishop (R) - District SD-R, Rep Matt Claman (D) - District SD-H, Sen Lyman Hoffman (D) - District SD-S, Sen Bert Stedman (R) - District SD-A, Sen Loki Tobin (D) - District SD-I, Sen Robert Myers (R) - District SD-Q, Rep Scott Kawasaki (D) - District SD-P, Sen William Wielechowski (D) - District SD-K, Sen Jesse Kiehl (D) - District SD-B, Sen Gary Stevens (R) - District SD-C, Rep Ashley Carrick (D) - District HD-035, Rep Daniel Ortiz (I) - District HD-001, Rep Sara Hannan (D) - District HD-004, Rep Alyse Galvin (I) - District HD-014, Rep William Fields (D) - District HD-017, Rep Conrad McCormick (D) - District HD-038, Rep Thomas Baker (R) - District HD-040, Rep Jennifer Armstrong (D) - District HD-016, Rep Craig Johnson (R) - District HD-010, Rep Andrew Gray (D) - District HD-020, Rep Donna Mears (D) - District HD-021, Rep Stanley Wright (R) - District HD-022, Rep Andrew Josephson (D) - District HD-013, Rep Genevieve Mina (D) - District HD-019, Rep Calvin Schrage (N) - District HD-012, Rep Cliff Groh (D) - District HD-018, Rep Neal Foster (D) - District HD-039, Rep Bryce Edgmon (I) - District HD-037</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Sen Donald Olson (D) - District SD-T, Sen Lyman Hoffman (D) - District SD-S, Sen William Wielechowski (D) - District SD-K, Rep William Fields (D) - District HD-017, Rep Thomas Baker (R) - District HD-040, Rep Neal Foster (D) - District HD-039, Rep Bryce Edgmon (I) - District HD-037</t>
+        </is>
+      </c>
       <c r="X2" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -675,7 +697,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Taskforce, US Law Enforcement, Tribal Law Enforcement, Data Collection, MMIP Relatives</t>
+          <t>Taskforce, US Law Enforcement, Tribal Law Enforcement, Data Collection.</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">

</xml_diff>

<commit_message>
Initial complete implementation with all fields
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -563,17 +563,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>National</t>
+          <t>AK</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Attorney General Garland, Secretary Haaland of the Department of the Interior Highlight Missing and Murdered Indigenous Peoples and Human Trafficking Crises in New Mexico Visit</t>
+          <t>Justice Department Launches Missing or Murdered Indigenous Persons Regional Outreach Program</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DOJ24-1000</t>
+          <t>DOJ23-324</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -588,110 +588,105 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Department of Justice, Department of the Interior</t>
+          <t>Department of Justice</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>August 12, 2024 - Immediate release, Office of Public Affairs</t>
+          <t>June 28, 2023 - Immediate release, U.S. Attorney's Office, District of Alaska</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://www.justice.gov/opa/pr/attorney-general-garland-secretary-haaland-department-interior-highlight-missing-and</t>
+          <t>https://www.justice.gov/usao-ak/pr/justice-department-launches-missing-or-murdered-indigenous-persons-regional-outreach</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>The press release highlights a visit by Attorney General Merrick B. Garland and Secretary of the Interior Deb Haaland to New Mexico, focusing on the Biden-Harris Administration's efforts to address the crises of Missing and Murdered Indigenous Peoples (MMIP) and human trafficking in Indian Country. Both leaders emphasized their commitment to improving public safety and collaborating with Tribal partners to confront these urgent issues. Initiatives discussed include significant funding to enhance Tribal justice systems, the establishment of the Missing and Murdered Unit, and various programs aimed at preventing and responding to cases of missing or murdered Indigenous individuals. The release also details interagency collaboration, including efforts with the Bureau of Indian Affairs and the FBI. Overall, the combined efforts aim to foster safe and healthy Tribal communities and ensure justice for Native victims of crime.</t>
+          <t>The Justice Department has launched the Missing or Murdered Indigenous Persons (MMIP) Regional Outreach Program to address the crisis of missing or murdered Indigenous people, focusing on placing Assistant U.S. Attorneys (AUSAs) and MMIP Coordinators in five regions across the United States, including Alaska. This initiative aims to enhance the prosecution of federal crimes in Indian country and improve relationships among federal, state, local, and Tribal partners. The program allocates resources specifically to combat violence and support public safety in Alaska Native communities, which have high rates of domestic violence, sexual assault, and trafficking. The Justice Department emphasizes collaboration with Tribes to ensure safety and justice for American Indian and Alaska Native families. The total resources allocated include three AUSAs and one Regional MMIP Coordinator for the Alaska U.S. Attorney's Office.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1. Enhances public safety by addressing the crises of Missing and Murdered Indigenous Peoples (MMIP) and human trafficking in Indian Country.  
-2. Promotes gender-inclusive language that acknowledges the diverse experiences within Indigenous communities.  
-3. Establishes the Not Invisible Act Commission to gather input from various stakeholders, ensuring that the voices of affected individuals are considered in policy recommendations.  
-4. Implements prevention efforts, including training for law enforcement on trauma-informed and culturally responsive investigative approaches.  
-5. Provides substantial funding to improve Tribal justice systems and ensure effective responses to cases involving missing or murdered Indigenous individuals.  
-6. Fosters collaboration between federal, state, and Tribal law enforcement agencies for more coordinated efforts in addressing MMIP issues.</t>
+          <t>1. The initiative enhances the prosecution of federal crimes in Indian country, addressing the crisis of missing or murdered Indigenous persons more effectively.
+2. It improves relationships among federal, state, local, and Tribal partners, fostering collaboration that leads to better resource allocation and community safety.
+3. The program specifically allocates resources to combat high rates of domestic violence, sexual assault, and trafficking in Alaska Native communities, directly addressing significant public safety concerns.
+4. The focus on Missing or Murdered Indigenous Persons (MMIP) inclusively recognizes and supports the experiences of all Indigenous individuals, including men, women, and non-binary persons.
+5. By placing Assistant U.S. Attorneys and MMIP Coordinators in key regions, the program ensures specialized support and ongoing engagement with federally recognized tribes.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>1. Implementation challenges may arise due to the complex nature of interagency collaboration among federal, state, and Tribal authorities.  
-2. The effectiveness of prevention efforts and training programs may vary across different jurisdictions, leading to inconsistent results.  
-3. While the legislation encourages stakeholder input, there may be limitations in adequately representing the voices of all affected individuals, particularly in remote or underserved communities.  
-4. Funding allocations might not sufficiently meet the needs of all Tribal justice systems, potentially hindering the overall impact of the initiatives.  
-5. There is a risk that initiatives could be viewed as reactive rather than proactive, focusing on immediate response rather than long-term solutions to systemic issues.</t>
+          <t>1. The legislation lacks specific mechanisms for evaluation, making it difficult to assess the effectiveness of the initiatives and the impact on Indigenous communities over time.
+2. There is no mention of input or advocacy from MMIP survivors, relatives, or Indigenous politicians, which may lead to the program not fully addressing the needs and concerns of those directly affected.
+3. The focus on five designated regions might limit the program's reach and fail to address the crises in other areas with significant Indigenous populations.
+4. While the program aims to combat violence and improve safety, it does not provide detailed strategies or methods for how these goals will be realized in practice.
+5. The absence of clear partnerships or consultation with Indigenous communities may result in the implementation of initiatives that do not align with community priorities or cultural considerations.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>1. No specific mechanisms for evaluation are mentioned in the legislation.</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1. The departments worked collaboratively to stand up the Not Invisible Act Commission, which was created by legislation the Secretary led in Congress, to develop recommendations on how the federal government can combat crimes against American Indian and Alaska Native people.  
-2. The Commission included federal, state, and Tribal law enforcement, Tribal leaders, federal partners, service providers, family members of missing and murdered individuals, and survivors.  
-3. In 2023, the Commission held seven field hearings across the country as well as a virtual national hearing to hear directly from individuals affected by the MMIP crisis.  
-4. In March 2024, the Departments released their response to the Commission’s recommendations, which they are in the process of implementing in collaboration with Congress.  </t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>The legislation specifically refers to the "Missing or Murdered Indigenous Persons (MMIP)" crisis, which broadens the focus beyond just women to include all missing or murdered Indigenous individuals. This terminology indicates an inclusive approach, recognizing the experiences of Indigenous men, women, and non-binary individuals. Additionally, the language used throughout the document maintains neutrality and does not prioritize one gender over another.</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>The legislation broadly addresses the crises of Missing and Murdered Indigenous Peoples (MMIP) and human trafficking without exclusively focusing on women, indicating a more inclusive approach. By using terms like "missing or murdered Indigenous persons" and referring to "Native victims of crime," it reflects an acknowledgment of the diverse experiences within Indigenous communities. This language facilitates a comprehensive understanding of the issues affecting all genders within the Indigenous population.</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>The legislation outlines several prevention efforts regarding Missing and Murdered Indigenous Persons, including training and awareness initiatives. Here are the relevant quotes:
-1. "Since the start of this Administration, the Justice Department has made strides in implementing systems aimed at preventing new instances of MMIP, locating individuals who are reported missing, and, where a crime has occurred, investigating and prosecuting those responsible."
-2. "The agreement also requires that all BIA, FBI and Tribal law enforcement officers receive training regarding trauma-informed, culturally responsive investigative approaches."
-3. "This program places attorneys and coordinators at U.S. Attorneys’ Offices across the United States to help prevent and respond to cases of missing or murdered Indigenous people."</t>
+          <t>1. "The Justice Department today announced the creation of the Missing or Murdered Indigenous Persons (MMIP) Regional Outreach Program, which permanently places MMIP Assistant U.S. Attorneys (AUSA) and MMIP Coordinators in five designated regions across the United States to aid in the prevention and response to missing or murdered Indigenous people and provide specialized support to United States Attorneys’ offices to address and combat the issues of MMIP."  
+2. "These AUSAs may participate in special district programs and initiatives designed to partner with and assist federally recognized Tribes in combatting emerging public safety issues."  
+3. "Our office is committed to combating violence in Alaska Native communities across the state and reducing the high rates of domestic violence, sexual assault, and trafficking in these communities."</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Yes. The legislation indicates a level of input from various stakeholders, including MMIP survivors, relatives, Indigenous politicians, and Indigenous communities. This is evidenced by the formation of the Not Invisible Act Commission, which included federal, state, and Tribal law enforcement, Tribal leaders, service providers, and family members of missing and murdered individuals, along with the holding of field hearings to gather direct input from affected individuals.</t>
+          <t>No</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Executive Order</t>
+          <t>Lane Tucker [U.S. Attorney, District of Alaska], Merrick B. Garland [Attorney General], Lisa O. Monaco [Deputy Attorney General]</t>
         </is>
       </c>
       <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Biden Administration, 2020 - 2024</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Taskforce, Data Collection, MMIP Relatives</t>
+          <t>Taskforce, US Law Enforcement, Tribal Law Enforcement, Data Collection</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>2024-10-29</t>
+          <t>2023-06-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated requirements to include titlecase
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -563,17 +563,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Justice Department Launches Missing or Murdered Indigenous Persons Regional Outreach Program</t>
+          <t>U.S. Attorney Kurt Alme and the Confederated Salish and Kootenai Tribes Launch Pilot Project to Address Missing and Murdered Indigenous Persons</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DOJ23-324</t>
+          <t>DOJ20-1111</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -593,37 +593,37 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>June 28, 2023 - Immediate release, U.S. Attorney's Office, District of Alaska</t>
+          <t>December 1, 2020 - Immediate release, U.S. Attorney's Office, District of Montana</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://www.justice.gov/usao-ak/pr/justice-department-launches-missing-or-murdered-indigenous-persons-regional-outreach</t>
+          <t>https://www.justice.gov/usao-mt/pr/us-attorney-kurt-alme-and-confederated-salish-and-kootenai-tribes-launch-pilot-project</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>The Justice Department has launched the Missing or Murdered Indigenous Persons (MMIP) Regional Outreach Program to address the crisis of missing or murdered Indigenous people, focusing on placing Assistant U.S. Attorneys (AUSAs) and MMIP Coordinators in five regions across the United States, including Alaska. This initiative aims to enhance the prosecution of federal crimes in Indian country and improve relationships among federal, state, local, and Tribal partners. The program allocates resources specifically to combat violence and support public safety in Alaska Native communities, which have high rates of domestic violence, sexual assault, and trafficking. The Justice Department emphasizes collaboration with Tribes to ensure safety and justice for American Indian and Alaska Native families. The total resources allocated include three AUSAs and one Regional MMIP Coordinator for the Alaska U.S. Attorney's Office.</t>
+          <t>The U.S. Attorney's Office in Montana, led by Kurt Alme, has launched a pilot project in collaboration with the Confederated Salish and Kootenai Tribes to develop a Tribal Community Response Plan (TCRP) aimed at improving responses to missing American Indian and Alaska Native individuals. This initiative is part of the broader Missing and Murdered Indigenous Persons (MMIP) Initiative and seeks to establish guidelines for a collaborative response involving Tribal governments, law enforcement, and community partners. The TCRP is expected to be completed by December 11, 2020, and will be the first of its kind in the country. The project focuses on culturally appropriate solutions, incorporating input from various stakeholders, including Tribal leaders and law enforcement. It aims to enhance public safety and provide equitable justice for Indigenous communities.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1. The initiative enhances the prosecution of federal crimes in Indian country, addressing the crisis of missing or murdered Indigenous persons more effectively.
-2. It improves relationships among federal, state, local, and Tribal partners, fostering collaboration that leads to better resource allocation and community safety.
-3. The program specifically allocates resources to combat high rates of domestic violence, sexual assault, and trafficking in Alaska Native communities, directly addressing significant public safety concerns.
-4. The focus on Missing or Murdered Indigenous Persons (MMIP) inclusively recognizes and supports the experiences of all Indigenous individuals, including men, women, and non-binary persons.
-5. By placing Assistant U.S. Attorneys and MMIP Coordinators in key regions, the program ensures specialized support and ongoing engagement with federally recognized tribes.</t>
+          <t>1. The initiative enhances the responsiveness to missing American Indian and Alaska Native individuals by establishing a collaborative Tribal Community Response Plan (TCRP), the first of its kind in the country.  
+2. It promotes culturally appropriate guidelines that involve input from Tribal governments, law enforcement, and community partners, ensuring a tailored approach to the community's needs.  
+3. The program contributes to improved public safety and justice for Indigenous communities by addressing the specific factors related to missing persons cases within these populations.  
+4. Training and awareness efforts, like those initiated by the U.S. Attorney's Office, empower law enforcement and the public to respond effectively when a loved one goes missing.  
+5. Overall, the collaboration fosters stronger partnerships between Tribal authorities and federal agencies, enhancing the capacity to address the Missing and Murdered Indigenous Persons crisis comprehensively.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>1. The legislation lacks specific mechanisms for evaluation, making it difficult to assess the effectiveness of the initiatives and the impact on Indigenous communities over time.
-2. There is no mention of input or advocacy from MMIP survivors, relatives, or Indigenous politicians, which may lead to the program not fully addressing the needs and concerns of those directly affected.
-3. The focus on five designated regions might limit the program's reach and fail to address the crises in other areas with significant Indigenous populations.
-4. While the program aims to combat violence and improve safety, it does not provide detailed strategies or methods for how these goals will be realized in practice.
-5. The absence of clear partnerships or consultation with Indigenous communities may result in the implementation of initiatives that do not align with community priorities or cultural considerations.</t>
+          <t>1. The legislation lacks specific mechanisms for evaluation, making it difficult to measure the effectiveness and impact of the Tribal Community Response Plan over time.  
+2. There is no detailed mention of direct input from MMIP survivors or their relatives, which may result in the program not fully addressing the needs and concerns of those directly affected.  
+3. The focus on developing a response plan only for the Confederated Salish and Kootenai Tribes may limit the program's broader applicability and fail to benefit other Indigenous communities facing similar issues.  
+4. While training and resources are provided, the foundational outcomes and ongoing support for communities after the pilot project ends are not clearly defined.  
+5. Although the initiative aims to improve public safety, the approach may not account for specific cultural or social dynamics within different Indigenous communities, potentially reducing its effectiveness.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -643,7 +643,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>The legislation specifically refers to the "Missing or Murdered Indigenous Persons (MMIP)" crisis, which broadens the focus beyond just women to include all missing or murdered Indigenous individuals. This terminology indicates an inclusive approach, recognizing the experiences of Indigenous men, women, and non-binary individuals. Additionally, the language used throughout the document maintains neutrality and does not prioritize one gender over another.</t>
+          <t>The legislation specifically refers to the "Missing and Murdered Indigenous Persons (MMIP)" crisis, which includes all Indigenous individuals, thereby broadening the focus beyond just women. This terminology reflects an inclusive approach that recognizes the experiences of Indigenous men, women, and non-binary individuals. Furthermore, the language throughout the document maintains neutrality, avoiding gender-specific references that prioritize one group over another.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -653,9 +653,13 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1. "The Justice Department today announced the creation of the Missing or Murdered Indigenous Persons (MMIP) Regional Outreach Program, which permanently places MMIP Assistant U.S. Attorneys (AUSA) and MMIP Coordinators in five designated regions across the United States to aid in the prevention and response to missing or murdered Indigenous people and provide specialized support to United States Attorneys’ offices to address and combat the issues of MMIP."  
-2. "These AUSAs may participate in special district programs and initiatives designed to partner with and assist federally recognized Tribes in combatting emerging public safety issues."  
-3. "Our office is committed to combating violence in Alaska Native communities across the state and reducing the high rates of domestic violence, sexual assault, and trafficking in these communities."</t>
+          <t>1. "The Pilot Project Will Develop Guidelines to Improve Community Responses to American Indian and Alaska Native Missing Person Cases."  
+2. "The goal of a TCRP is to improve responses to emergent American Indian and Alaska Native (AI/AN) missing person cases by establishing a collaborative response from Tribal governments, law enforcement, and other partners through culturally appropriate guidelines."  
+3. "The U.S. Department of Justice and other federal agencies developed draft guides to assist in developing plans with input from tribal leaders, tribal law enforcement and their communities."  
+4. "The Council also hosted a training on human trafficking and its correlation to MMIP and held numerous community meetings on safety awareness."  
+5. "The U.S. Attorney’s Office for Montana...held two statewide trainings for law enforcement on how to use missing person databases and alerts (such as Amber Alerts), and for the public on what to do when a loved one goes missing."  
+6. "Brought trainers from the National Missing and Unidentified Persons System (NAMUS) to all seven Montana reservations to train community members on how to use that system when a loved one goes missing."  
+7. "Developed a public service announcement to inform the public about what to do when a loved one goes missing."</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -665,18 +669,22 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Somewhat - While the legislation mentions input from tribal leaders and the involvement of the Confederated Salish and Kootenai Tribes in developing a Tribal Community Response Plan, it does not specifically detail the level of input from MMIP survivors or their relatives. However, the focus on collaboration with tribal governments suggests some acknowledgment of community needs. Overall, there is an indication of community involvement, but it lacks explicit mention of direct input from survivors or relatives.</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Lane Tucker [U.S. Attorney, District of Alaska], Merrick B. Garland [Attorney General], Lisa O. Monaco [Deputy Attorney General]</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr"/>
+          <t>Kurt Alme [U.S. Attorney, District of Montana], Shelly R. Fyant [Chairwoman, Confederated Salish and Kootenai Tribes], Melissa Schlichting [Presiding Officer, Montana Missing Indigenous Persons Task Force]</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Shelly R. Fyant [Confederated Salish and Kootenai Tribes]</t>
+        </is>
+      </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>Biden Administration, 2020 - 2024</t>
+          <t>Trump Administration, 2016 - 2020</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -686,7 +694,7 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>2023-06-28</t>
+          <t>2020-12-01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tweaks to initial implemenation prompts
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -563,19 +563,15 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>AK</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>U.S. Attorney Kurt Alme and the Confederated Salish and Kootenai Tribes Launch Pilot Project to Address Missing and Murdered Indigenous Persons</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>DOJ20-1111</t>
-        </is>
-      </c>
+          <t>Justice Department Launches Missing or Murdered Indigenous Persons Regional Outreach Program</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>Passed</t>
@@ -593,37 +589,37 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>December 1, 2020 - Immediate release, U.S. Attorney's Office, District of Montana</t>
+          <t>June 28, 2023 - Immediate release, U.S. Attorney's Office, District of Alaska</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://www.justice.gov/usao-mt/pr/us-attorney-kurt-alme-and-confederated-salish-and-kootenai-tribes-launch-pilot-project</t>
+          <t>https://www.justice.gov/usao-ak/pr/justice-department-launches-missing-or-murdered-indigenous-persons-regional-outreach</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>The U.S. Attorney's Office in Montana, led by Kurt Alme, has launched a pilot project in collaboration with the Confederated Salish and Kootenai Tribes to develop a Tribal Community Response Plan (TCRP) aimed at improving responses to missing American Indian and Alaska Native individuals. This initiative is part of the broader Missing and Murdered Indigenous Persons (MMIP) Initiative and seeks to establish guidelines for a collaborative response involving Tribal governments, law enforcement, and community partners. The TCRP is expected to be completed by December 11, 2020, and will be the first of its kind in the country. The project focuses on culturally appropriate solutions, incorporating input from various stakeholders, including Tribal leaders and law enforcement. It aims to enhance public safety and provide equitable justice for Indigenous communities.</t>
+          <t>The Justice Department has launched the Missing or Murdered Indigenous Persons (MMIP) Regional Outreach Program to address the crisis of missing or murdered Indigenous people by placing Assistant U.S. Attorneys and coordinators in five regions across the United States. The initiative aims to enhance collaboration between federal, Tribal, state, and local partners while providing specialized support to U.S. Attorney’s offices in prosecuting relevant federal law violations. In Alaska, three Assistant U.S. Attorneys and one MMIP Coordinator will focus on improving public safety and combating violence in Alaska Native communities. The program reflects the Justice Department's commitment to working with Tribes to promote safety and justice for American Indian and Alaska Native families. Overall, the initiative aims to mobilize resources to address the critical issues faced by Indigenous communities.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1. The initiative enhances the responsiveness to missing American Indian and Alaska Native individuals by establishing a collaborative Tribal Community Response Plan (TCRP), the first of its kind in the country.  
-2. It promotes culturally appropriate guidelines that involve input from Tribal governments, law enforcement, and community partners, ensuring a tailored approach to the community's needs.  
-3. The program contributes to improved public safety and justice for Indigenous communities by addressing the specific factors related to missing persons cases within these populations.  
-4. Training and awareness efforts, like those initiated by the U.S. Attorney's Office, empower law enforcement and the public to respond effectively when a loved one goes missing.  
-5. Overall, the collaboration fosters stronger partnerships between Tribal authorities and federal agencies, enhancing the capacity to address the Missing and Murdered Indigenous Persons crisis comprehensively.</t>
+          <t>1. The initiative establishes a dedicated program to address the crisis of missing or murdered Indigenous persons by placing Assistant U.S. Attorneys and coordinators in key regions across the U.S.  
+2. It promotes collaboration among federal, Tribal, state, and local partners, enhancing the effectiveness of responses to public safety issues in Indigenous communities.  
+3. The program allocates resources specifically for combating violence in Alaska Native communities, improving public safety and support for these populations.  
+4. By providing specialized support to U.S. Attorney’s offices, the initiative strengthens the prosecution of federal law violations related to Indigenous people.  
+5. The inclusive language acknowledges and represents all genders, ensuring that the experiences of all Indigenous people affected by violence are recognized and addressed.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>1. The legislation lacks specific mechanisms for evaluation, making it difficult to measure the effectiveness and impact of the Tribal Community Response Plan over time.  
-2. There is no detailed mention of direct input from MMIP survivors or their relatives, which may result in the program not fully addressing the needs and concerns of those directly affected.  
-3. The focus on developing a response plan only for the Confederated Salish and Kootenai Tribes may limit the program's broader applicability and fail to benefit other Indigenous communities facing similar issues.  
-4. While training and resources are provided, the foundational outcomes and ongoing support for communities after the pilot project ends are not clearly defined.  
-5. Although the initiative aims to improve public safety, the approach may not account for specific cultural or social dynamics within different Indigenous communities, potentially reducing its effectiveness.</t>
+          <t xml:space="preserve">1. The legislation does not outline any specific mechanisms for evaluation, making it challenging to assess its effectiveness and impact over time.  
+2. There is no direct input or consultation from MMIP survivors, their relatives, or Indigenous communities, which could limit the relevance and responsiveness of the program to their needs.  
+3. The absence of defined strategies for centering Indigenous voices may lead to a disconnect between the program's objectives and the actual experiences of affected communities.  
+4. The focus on federal law enforcement may be perceived as insufficient by those advocating for more comprehensive community-based approaches to address violence against Indigenous people.  
+5. Without clear data collection methods mentioned, the program may face difficulties in gathering accurate information necessary for informed decision-making and resource allocation.  </t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -633,7 +629,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>1. No specific mechanisms for evaluation are mentioned in the legislation.</t>
+          <t>1. There are no specific mechanisms for evaluation mentioned in the legislation.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -643,7 +639,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>The legislation specifically refers to the "Missing and Murdered Indigenous Persons (MMIP)" crisis, which includes all Indigenous individuals, thereby broadening the focus beyond just women. This terminology reflects an inclusive approach that recognizes the experiences of Indigenous men, women, and non-binary individuals. Furthermore, the language throughout the document maintains neutrality, avoiding gender-specific references that prioritize one group over another.</t>
+          <t>The legislation uses the term "Missing or Murdered Indigenous Persons," which explicitly includes individuals of all genders, rather than focusing solely on women. The language throughout the document is neutral and inclusive, addressing the broader issue of missing and murdered Indigenous individuals. This approach acknowledges the experiences of all Indigenous people affected by violence, ensuring that no specific gender is marginalized in the discussion.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -653,13 +649,9 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1. "The Pilot Project Will Develop Guidelines to Improve Community Responses to American Indian and Alaska Native Missing Person Cases."  
-2. "The goal of a TCRP is to improve responses to emergent American Indian and Alaska Native (AI/AN) missing person cases by establishing a collaborative response from Tribal governments, law enforcement, and other partners through culturally appropriate guidelines."  
-3. "The U.S. Department of Justice and other federal agencies developed draft guides to assist in developing plans with input from tribal leaders, tribal law enforcement and their communities."  
-4. "The Council also hosted a training on human trafficking and its correlation to MMIP and held numerous community meetings on safety awareness."  
-5. "The U.S. Attorney’s Office for Montana...held two statewide trainings for law enforcement on how to use missing person databases and alerts (such as Amber Alerts), and for the public on what to do when a loved one goes missing."  
-6. "Brought trainers from the National Missing and Unidentified Persons System (NAMUS) to all seven Montana reservations to train community members on how to use that system when a loved one goes missing."  
-7. "Developed a public service announcement to inform the public about what to do when a loved one goes missing."</t>
+          <t xml:space="preserve">1. "These AUSAs may participate in special district programs and initiatives designed to partner with and assist federally recognized Tribes in combatting emerging public safety issues."  
+2. "This new program mobilizes the Justice Department’s resources to combat the crisis of Missing or Murdered Indigenous Persons, which has shattered the lives of victims, their families, and entire Tribal communities."  
+3. "The Justice Department will continue to accelerate our efforts, in partnership with Tribes, to keep their communities safe and pursue justice for American Indian and Alaska Native families."  </t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -669,22 +661,18 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Somewhat - While the legislation mentions input from tribal leaders and the involvement of the Confederated Salish and Kootenai Tribes in developing a Tribal Community Response Plan, it does not specifically detail the level of input from MMIP survivors or their relatives. However, the focus on collaboration with tribal governments suggests some acknowledgment of community needs. Overall, there is an indication of community involvement, but it lacks explicit mention of direct input from survivors or relatives.</t>
+          <t>No</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Kurt Alme [U.S. Attorney, District of Montana], Shelly R. Fyant [Chairwoman, Confederated Salish and Kootenai Tribes], Melissa Schlichting [Presiding Officer, Montana Missing Indigenous Persons Task Force]</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>Shelly R. Fyant [Confederated Salish and Kootenai Tribes]</t>
-        </is>
-      </c>
+          <t>Merrick B. Garland [Attorney General], Lisa O. Monaco [Deputy Attorney General]</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr">
         <is>
-          <t>Trump Administration, 2016 - 2020</t>
+          <t>Biden Administration, 2020 - 2024</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -694,7 +682,7 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>2020-12-01</t>
+          <t>2023-06-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tweaked indigenous sponsors prompt
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -563,15 +563,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>National</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Justice Department Launches Missing or Murdered Indigenous Persons Regional Outreach Program</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>Justice Department Strengthens Efforts, Builds Partnerships to Address the Crisis of Missing or Murdered Indigenous Persons</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>DOJ24-118</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>Passed</t>
@@ -589,37 +593,39 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>June 28, 2023 - Immediate release, U.S. Attorney's Office, District of Alaska</t>
+          <t>May 3, 2024 - Immediate release, U.S. Attorney's Office, District of Montana</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://www.justice.gov/usao-ak/pr/justice-department-launches-missing-or-murdered-indigenous-persons-regional-outreach</t>
+          <t>https://www.justice.gov/usao-mt/pr/justice-department-strengthens-efforts-builds-partnerships-address-crisis-missing-or</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>The Justice Department has launched the Missing or Murdered Indigenous Persons (MMIP) Regional Outreach Program to address the crisis of missing or murdered Indigenous people by placing Assistant U.S. Attorneys and coordinators in five regions across the United States. The initiative aims to enhance collaboration between federal, Tribal, state, and local partners while providing specialized support to U.S. Attorney’s offices in prosecuting relevant federal law violations. In Alaska, three Assistant U.S. Attorneys and one MMIP Coordinator will focus on improving public safety and combating violence in Alaska Native communities. The program reflects the Justice Department's commitment to working with Tribes to promote safety and justice for American Indian and Alaska Native families. Overall, the initiative aims to mobilize resources to address the critical issues faced by Indigenous communities.</t>
+          <t>The Justice Department's initiative aims to address the crisis of missing or murdered Indigenous persons (MMIP) by building partnerships with federal, state, and tribal communities. It highlights the recognition of May 5 as National MMIP Awareness Day and underscores ongoing efforts to mitigate violence against American Indian and Alaska Native communities. U.S. Attorney Merrick B. Garland emphasized the commitment to honor the victims and improve public safety in tribal areas. The initiative includes the creation of the MMIP Regional Outreach Program, which will deploy attorneys and coordinators to focus on MMIP cases across designated regions. The collaboration also involves insights from various tribal leaders, showcasing a united front to combat these public safety challenges.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1. The initiative establishes a dedicated program to address the crisis of missing or murdered Indigenous persons by placing Assistant U.S. Attorneys and coordinators in key regions across the U.S.  
-2. It promotes collaboration among federal, Tribal, state, and local partners, enhancing the effectiveness of responses to public safety issues in Indigenous communities.  
-3. The program allocates resources specifically for combating violence in Alaska Native communities, improving public safety and support for these populations.  
-4. By providing specialized support to U.S. Attorney’s offices, the initiative strengthens the prosecution of federal law violations related to Indigenous people.  
-5. The inclusive language acknowledges and represents all genders, ensuring that the experiences of all Indigenous people affected by violence are recognized and addressed.</t>
+          <t xml:space="preserve">1. Enhances collaboration between federal, state, and tribal communities to address the crisis of missing or murdered Indigenous persons (MMIP).  
+2. Recognizes May 5 as National MMIP Awareness Day, raising awareness about violence against American Indian and Alaska Native communities.  
+3. Establishes the MMIP Regional Outreach Program, deploying attorneys and coordinators to focus on MMIP cases across designated regions.  
+4. Employs gender-inclusive language to encompass all Indigenous individuals affected by the crisis.  
+5. Strengthens partnerships with tribal leadership and law enforcement to improve public safety and address ongoing violence in tribal areas.  
+6. Commits to finding missing individuals and holding perpetrators accountable through enhanced law enforcement collaboration.  
+7. Acknowledges and addresses the higher rates of violence faced by Indigenous women and children in the community.  </t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The legislation does not outline any specific mechanisms for evaluation, making it challenging to assess its effectiveness and impact over time.  
-2. There is no direct input or consultation from MMIP survivors, their relatives, or Indigenous communities, which could limit the relevance and responsiveness of the program to their needs.  
-3. The absence of defined strategies for centering Indigenous voices may lead to a disconnect between the program's objectives and the actual experiences of affected communities.  
-4. The focus on federal law enforcement may be perceived as insufficient by those advocating for more comprehensive community-based approaches to address violence against Indigenous people.  
-5. Without clear data collection methods mentioned, the program may face difficulties in gathering accurate information necessary for informed decision-making and resource allocation.  </t>
+          <t xml:space="preserve">1. The legislation does not explicitly mention direct input from MMIP survivors or relatives of victims, limiting the representation of their voices in the initiative.  
+2. While it emphasizes collaboration with tribal leadership, it may not fully account for the diverse needs and perspectives of individual tribal communities.  
+3. There is a lack of specific, quantified data on the effectiveness of the MMIP Regional Outreach Program and how it will be evaluated over time.  
+4. The initiative may face challenges in implementation due to varying levels of resources and support across different federal, state, and tribal entities.  
+5. Potential reliance on external partners might create inconsistencies in the approach to addressing violence within different tribal areas.  </t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -629,7 +635,10 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>1. There are no specific mechanisms for evaluation mentioned in the legislation.</t>
+          <t>1. The legislation mentions a "joint response to the Not Invisible Act Commission’s recommendations on how to combat the missing or murdered Indigenous peoples (MMIP) and human trafficking crisis."
+2. It emphasizes the importance of "collaborative investigation" involving federal, local, and tribal law enforcement partners.
+3. It discusses "meeting regularly with tribal leadership" to address issues facing tribal communities. 
+4. It includes a commitment to "forge stronger partnerships with federal and Tribal law enforcement partners" to address public safety challenges.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -639,7 +648,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>The legislation uses the term "Missing or Murdered Indigenous Persons," which explicitly includes individuals of all genders, rather than focusing solely on women. The language throughout the document is neutral and inclusive, addressing the broader issue of missing and murdered Indigenous individuals. This approach acknowledges the experiences of all Indigenous people affected by violence, ensuring that no specific gender is marginalized in the discussion.</t>
+          <t>The legislation employs gender-inclusive language by referring to the "Missing or Murdered Indigenous Persons" (MMIP) crisis, which encompasses all Indigenous individuals rather than exclusively focusing on women. By acknowledging the broader community affected by violence and disappearance, it demonstrates an awareness of the varied experiences that Indigenous people face. The use of terms like "every person" and "Indigenous men, women or child" reflects an effort to be inclusive and address the issue comprehensively.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -649,9 +658,9 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. "These AUSAs may participate in special district programs and initiatives designed to partner with and assist federally recognized Tribes in combatting emerging public safety issues."  
-2. "This new program mobilizes the Justice Department’s resources to combat the crisis of Missing or Murdered Indigenous Persons, which has shattered the lives of victims, their families, and entire Tribal communities."  
-3. "The Justice Department will continue to accelerate our efforts, in partnership with Tribes, to keep their communities safe and pursue justice for American Indian and Alaska Native families."  </t>
+          <t>1. "The Justice Department joins its partners across the federal government, as well as people throughout American Indian and Alaska Native communities, in recognizing May 5 as National Missing or Murdered Indigenous Persons (MMIP) Awareness Day."
+2. "We also acknowledge that Indigenous women and children face disproportionally higher rates of violence and sexual abuse. And we reaffirm our commitment to do everything we can to find the missing, hold killers accountable and seek justice for the missing or murdered by continuing to work with all our federal, state, tribal and local law enforcement partners."
+3. "The MMIP Regional Outreach Program prioritizes MMIP cases consistent with the Deputy Attorney General’s July 2022 directive to U.S. Attorneys’ offices promoting public safety in Indian country."</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -661,15 +670,19 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Somewhat. The legislation acknowledges the importance of consulting with tribal leadership and working closely with various tribes, including the Blackfeet Nation, Rocky Boy's Reservation, and others, to address the issues of missing or murdered Indigenous persons. While it emphasizes collaboration and partnership with these communities and their leaders, it does not explicitly mention direct input from survivors or relatives of MMIP victims. However, the commitment to engage with tribal leadership suggests a degree of community involvement in shaping the initiative.</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Merrick B. Garland [Attorney General], Lisa O. Monaco [Deputy Attorney General]</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr"/>
+          <t>Merrick B. Garland [U.S. Attorney General], Jesse Laslovich [U.S. Attorney for the District of Montana], Christopher Wray [FBI Director], Anne Milgram [DEA Administrator], Blackfeet Nation, Rocky Boy's Reservation, Fort Belknap Indian Community, Fort Peck Tribes, Crow Tribe, Northern Cheyenne Tribe, Confederated Salish and Kootenai Tribes</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Blackfeet Nation, Rocky Boy's Reservation, Fort Belknap Indian Community, Fort Peck Tribes, Crow Tribe, Northern Cheyenne Tribe, Confederated Salish and Kootenai Tribes</t>
+        </is>
+      </c>
       <c r="X2" t="inlineStr">
         <is>
           <t>Biden Administration, 2020 - 2024</t>
@@ -677,12 +690,12 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Taskforce, US Law Enforcement, Tribal Law Enforcement, Data Collection</t>
+          <t>Day of Recognition, US Law Enforcement, Tribal Law Enforcement, Taskforce</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>2023-06-28</t>
+          <t>2024-05-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fine-tuned sponsor GPT ask
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -563,17 +563,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>National</t>
+          <t>AK</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Justice Department Strengthens Efforts, Builds Partnerships to Address the Crisis of Missing or Murdered Indigenous Persons</t>
+          <t>U.S. Attorney Tucker Issues Savanna’s Act Guidelines for Alaska</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DOJ24-118</t>
+          <t>DOJ19-087</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -593,52 +593,50 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>May 3, 2024 - Immediate release, U.S. Attorney's Office, District of Montana</t>
+          <t>August 30, 2022 - For Immediate Release, U.S. Attorney's Office, District of Alaska</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://www.justice.gov/usao-mt/pr/justice-department-strengthens-efforts-builds-partnerships-address-crisis-missing-or</t>
+          <t>https://www.justice.gov/usao-ak/pr/us-attorney-tucker-issues-savanna-s-act-guidelines-alaska</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>The Justice Department's initiative aims to address the crisis of missing or murdered Indigenous persons (MMIP) by building partnerships with federal, state, and tribal communities. It highlights the recognition of May 5 as National MMIP Awareness Day and underscores ongoing efforts to mitigate violence against American Indian and Alaska Native communities. U.S. Attorney Merrick B. Garland emphasized the commitment to honor the victims and improve public safety in tribal areas. The initiative includes the creation of the MMIP Regional Outreach Program, which will deploy attorneys and coordinators to focus on MMIP cases across designated regions. The collaboration also involves insights from various tribal leaders, showcasing a united front to combat these public safety challenges.</t>
+          <t>The Savanna’s Act Guidelines for Alaska, announced by U.S. Attorney S. Lane Tucker, aim to improve the government’s response to the crisis of missing and murdered Indigenous persons through enhanced coordination among law enforcement agencies. The guidelines are based on extensive consultations with Alaska Tribes, victim service providers, and various law enforcement entities. They focus on developing best practices for communication, data collection, reporting, and culturally appropriate victim services. The initiative is designed to address the high rates of violence against Alaska Natives and American Indians while ensuring ongoing opportunities for input and recommendations from the community. Overall, it seeks to strengthen partnerships across different levels of law enforcement to bring justice for victims and their families.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Enhances collaboration between federal, state, and tribal communities to address the crisis of missing or murdered Indigenous persons (MMIP).  
-2. Recognizes May 5 as National MMIP Awareness Day, raising awareness about violence against American Indian and Alaska Native communities.  
-3. Establishes the MMIP Regional Outreach Program, deploying attorneys and coordinators to focus on MMIP cases across designated regions.  
-4. Employs gender-inclusive language to encompass all Indigenous individuals affected by the crisis.  
-5. Strengthens partnerships with tribal leadership and law enforcement to improve public safety and address ongoing violence in tribal areas.  
-6. Commits to finding missing individuals and holding perpetrators accountable through enhanced law enforcement collaboration.  
-7. Acknowledges and addresses the higher rates of violence faced by Indigenous women and children in the community.  </t>
+          <t xml:space="preserve">1. The Savanna’s Act Guidelines for Alaska enhance coordination among law enforcement agencies, improving the efficiency and effectiveness of responses to missing and murdered Indigenous persons.  
+2. Extensive consultations with Alaska Tribes and victim service providers ensure that the guidelines are informed by the needs and experiences of the community, fostering trust and collaboration.  
+3. The focus on best practices for data collection and culturally appropriate victim services aims to address the high rates of violence against Alaska Natives and American Indians comprehensively.  
+4. Ongoing opportunities for input and recommendations allow for adaptability and continuous improvement of the guidelines based on feedback from stakeholders.  
+5. The gender-inclusive language acknowledges and represents all Indigenous individuals affected by violence and missing person cases, promoting a holistic understanding of the crisis.  </t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The legislation does not explicitly mention direct input from MMIP survivors or relatives of victims, limiting the representation of their voices in the initiative.  
-2. While it emphasizes collaboration with tribal leadership, it may not fully account for the diverse needs and perspectives of individual tribal communities.  
-3. There is a lack of specific, quantified data on the effectiveness of the MMIP Regional Outreach Program and how it will be evaluated over time.  
-4. The initiative may face challenges in implementation due to varying levels of resources and support across different federal, state, and tribal entities.  
-5. Potential reliance on external partners might create inconsistencies in the approach to addressing violence within different tribal areas.  </t>
+          <t xml:space="preserve">1. The reliance on consultations with Tribes and victim service providers may not fully represent the viewpoints of all MMIP survivors and their families, leading to potential gaps in addressing specific needs.  
+2. While the guidelines emphasize coordination among law enforcement agencies, there may be challenges in implementation due to differing priorities or lack of resources among the involved agencies.  
+3. The effectiveness of the guidelines depends on ongoing funding and support, which may fluctuate or be subject to political changes, impacting the sustainability of the initiative.  
+4. The focus on law enforcement may overshadow broader social issues, such as poverty, historical trauma, and systemic inequalities that contribute to the crisis of missing and murdered Indigenous persons.  
+5. Without specific accountability measures or timelines for implementing the guidelines, there is a risk that progress may be slow or inadequately monitored over time.  </t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>1. The legislation mentions a "joint response to the Not Invisible Act Commission’s recommendations on how to combat the missing or murdered Indigenous peoples (MMIP) and human trafficking crisis."
-2. It emphasizes the importance of "collaborative investigation" involving federal, local, and tribal law enforcement partners.
-3. It discusses "meeting regularly with tribal leadership" to address issues facing tribal communities. 
-4. It includes a commitment to "forge stronger partnerships with federal and Tribal law enforcement partners" to address public safety challenges.</t>
+          <t xml:space="preserve">1. "It also provides guidance on the collection, reporting and analysis of MMIP data; offers resource information for Tribal governments; and provides best practices for culturally appropriate victim services and for returning a loved one home."  
+2. "Specifically, it directs the U.S. Department of Justice to develop guidelines to continually improve communication and coordination among tribal, federal, state and local law enforcement agencies in response to MMIP situations."  
+3. "These guidelines are evergreen with ongoing opportunities for input and recommendations."  
+4. "Following hundreds of hours of consultation with Alaska Tribes and tribal agencies, federal, state, local and tribal law enforcement and victim service providers."  </t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -648,7 +646,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>The legislation employs gender-inclusive language by referring to the "Missing or Murdered Indigenous Persons" (MMIP) crisis, which encompasses all Indigenous individuals rather than exclusively focusing on women. By acknowledging the broader community affected by violence and disappearance, it demonstrates an awareness of the varied experiences that Indigenous people face. The use of terms like "every person" and "Indigenous men, women or child" reflects an effort to be inclusive and address the issue comprehensively.</t>
+          <t>The legislation addresses the initiative by referring to "missing and murdered Alaska Natives and Native Americans," which includes all Indigenous individuals, not just women. It consistently uses terms like "missing indigenous people" and "missing persons," ensuring that the language remains gender-neutral throughout the document. This approach acknowledges the experiences of all members of Indigenous communities affected by violence and missing person cases.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -658,44 +656,39 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1. "The Justice Department joins its partners across the federal government, as well as people throughout American Indian and Alaska Native communities, in recognizing May 5 as National Missing or Murdered Indigenous Persons (MMIP) Awareness Day."
-2. "We also acknowledge that Indigenous women and children face disproportionally higher rates of violence and sexual abuse. And we reaffirm our commitment to do everything we can to find the missing, hold killers accountable and seek justice for the missing or murdered by continuing to work with all our federal, state, tribal and local law enforcement partners."
-3. "The MMIP Regional Outreach Program prioritizes MMIP cases consistent with the Deputy Attorney General’s July 2022 directive to U.S. Attorneys’ offices promoting public safety in Indian country."</t>
+          <t xml:space="preserve">1. "Federal prosecutors and the FBI are to enhance investigations into missing persons, develop protocols for law enforcement, improve data collection and analysis, and provide training and technical assistance."  
+2. "The MMIP Coordinator will work closely with federal, tribal, state, and local agencies to develop common protocols and procedures for responding to reports of missing or murdered indigenous people."  </t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Somewhat</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Somewhat. The legislation acknowledges the importance of consulting with tribal leadership and working closely with various tribes, including the Blackfeet Nation, Rocky Boy's Reservation, and others, to address the issues of missing or murdered Indigenous persons. While it emphasizes collaboration and partnership with these communities and their leaders, it does not explicitly mention direct input from survivors or relatives of MMIP victims. However, the commitment to engage with tribal leadership suggests a degree of community involvement in shaping the initiative.</t>
+          <t>Yes. The legislation indicates that there have been "hundreds of hours of consultation with Alaska Tribes, tribal agencies, victim service providers, and federal, state, local, and tribal law enforcement," showcasing a significant level of input from various stakeholders, including those from Indigenous communities. Additionally, the ongoing opportunities for input and recommendations suggest that the voices of MMIP survivors and their families are being considered in the development of the guidelines. Thus, the level of input is not only present but is also emphasized as crucial to the initiative's effectiveness.</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Merrick B. Garland [U.S. Attorney General], Jesse Laslovich [U.S. Attorney for the District of Montana], Christopher Wray [FBI Director], Anne Milgram [DEA Administrator], Blackfeet Nation, Rocky Boy's Reservation, Fort Belknap Indian Community, Fort Peck Tribes, Crow Tribe, Northern Cheyenne Tribe, Confederated Salish and Kootenai Tribes</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>Blackfeet Nation, Rocky Boy's Reservation, Fort Belknap Indian Community, Fort Peck Tribes, Crow Tribe, Northern Cheyenne Tribe, Confederated Salish and Kootenai Tribes</t>
-        </is>
-      </c>
+          <t>S. Lane Tucker [U.S. Attorney, District of Alaska], Lisa Murkowski [U.S. Senator, Alaska], Ingrid Cumberlidge [MMIP Program Coordinator, U.S. Attorney's Office]</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr">
         <is>
-          <t>Biden Administration, 2020 - 2024</t>
+          <t>Biden Administration, 2020-2024</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Day of Recognition, US Law Enforcement, Tribal Law Enforcement, Taskforce</t>
+          <t>Taskforce, US Law Enforcement, Tribal Law Enforcement, Data Collection</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>2024-05-03</t>
+          <t>2022-08-30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improved indigenous sponsor / partner match
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -563,17 +563,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AK</t>
+          <t>OR</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>U.S. Attorney Tucker Issues Savanna’s Act Guidelines for Alaska</t>
+          <t>U.S. Attorney's Office Joins in Recognizing Missing and Murdered Indigenous Persons Awareness Day and Announces Appointment of Regional MMIP Coordinator</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DOJ19-087</t>
+          <t>DOJ24-570</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -593,102 +593,106 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>August 30, 2022 - For Immediate Release, U.S. Attorney's Office, District of Alaska</t>
+          <t>May 3, 2024 - Immediate Release, U.S. Attorney's Office, District of Oregon</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://www.justice.gov/usao-ak/pr/us-attorney-tucker-issues-savanna-s-act-guidelines-alaska</t>
+          <t>https://www.justice.gov/usao-or/pr/us-attorneys-office-joins-recognizing-missing-and-murdered-indigenous-persons-1</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>The Savanna’s Act Guidelines for Alaska, announced by U.S. Attorney S. Lane Tucker, aim to improve the government’s response to the crisis of missing and murdered Indigenous persons through enhanced coordination among law enforcement agencies. The guidelines are based on extensive consultations with Alaska Tribes, victim service providers, and various law enforcement entities. They focus on developing best practices for communication, data collection, reporting, and culturally appropriate victim services. The initiative is designed to address the high rates of violence against Alaska Natives and American Indians while ensuring ongoing opportunities for input and recommendations from the community. Overall, it seeks to strengthen partnerships across different levels of law enforcement to bring justice for victims and their families.</t>
+          <t>The U.S. Attorney's Office for the District of Oregon recognizes May 5, 2024, as National Missing and Murdered Indigenous Persons (MMIP) Awareness Day and appoints Cedar Wilkie Gillette as the regional MMIP Coordinator for the Northwest Region. This initiative is part of the Justice Department's MMIP Regional Outreach Program, which aims to address the crisis of missing and murdered Indigenous people through collaboration among various law enforcement agencies. The program focuses on enhancing responses to unresolved MMIP cases and allocates significant funding to support Tribal justice systems. U.S. Attorney Natalie Wight and Attorney General Merrick B. Garland emphasize the commitment to improving safety and justice for Tribal communities. The initiative reflects a broader effort to tackle violence against Indigenous peoples and strengthen community support.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The Savanna’s Act Guidelines for Alaska enhance coordination among law enforcement agencies, improving the efficiency and effectiveness of responses to missing and murdered Indigenous persons.  
-2. Extensive consultations with Alaska Tribes and victim service providers ensure that the guidelines are informed by the needs and experiences of the community, fostering trust and collaboration.  
-3. The focus on best practices for data collection and culturally appropriate victim services aims to address the high rates of violence against Alaska Natives and American Indians comprehensively.  
-4. Ongoing opportunities for input and recommendations allow for adaptability and continuous improvement of the guidelines based on feedback from stakeholders.  
-5. The gender-inclusive language acknowledges and represents all Indigenous individuals affected by violence and missing person cases, promoting a holistic understanding of the crisis.  </t>
+          <t xml:space="preserve">1. Recognizes May 5, 2024, as National Missing and Murdered Indigenous Persons Awareness Day, raising awareness about the ongoing crisis within Indigenous communities.  
+2. Appoints Cedar Wilkie Gillette as the regional MMIP Coordinator, providing dedicated leadership to focus on the issue.  
+3. Facilitates collaboration among federal, tribal, local, and state law enforcement agencies to improve responses to unresolved MMIP cases.  
+4. Utilizes gender-inclusive language, addressing the concerns of all Indigenous individuals impacted by violence and promoting a broader understanding of the crisis.  
+5. Allocates $268 million in grants to enhance Tribal justice systems and strengthen law enforcement capabilities, thereby improving community safety.  
+6. Encourages input from Indigenous communities through partnerships with various Tribes, ensuring that the initiative is informed by their perspectives and needs.  
+7. Reflects a comprehensive approach to tackling violence against Indigenous peoples and demonstrates a commitment to justice and safety for Tribal communities.  </t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The reliance on consultations with Tribes and victim service providers may not fully represent the viewpoints of all MMIP survivors and their families, leading to potential gaps in addressing specific needs.  
-2. While the guidelines emphasize coordination among law enforcement agencies, there may be challenges in implementation due to differing priorities or lack of resources among the involved agencies.  
-3. The effectiveness of the guidelines depends on ongoing funding and support, which may fluctuate or be subject to political changes, impacting the sustainability of the initiative.  
-4. The focus on law enforcement may overshadow broader social issues, such as poverty, historical trauma, and systemic inequalities that contribute to the crisis of missing and murdered Indigenous persons.  
-5. Without specific accountability measures or timelines for implementing the guidelines, there is a risk that progress may be slow or inadequately monitored over time.  </t>
+          <t>1. The legislation lacks specified mechanisms for evaluation, leaving uncertainty about how success will be measured or activities assessed.  
+2. There is no mention of direct input or consultation from MMIP survivors and relatives, which may limit responsiveness to their specific needs and concerns.  
+3. The absence of a final report or data collection efforts may hinder the ability to track progress and identify effective strategies over time.  
+4. While it supports law enforcement, the focus may not fully address the root causes of violence against Indigenous peoples, such as socio-economic disparities.  
+5. The language and initiatives may require more specificity on implementation timelines and accountability structures to ensure meaningful action is taken.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>1. The legislation does not specify any mechanisms for evaluation such as a final report, consultation with community, tribal consultation, a Tribal Crisis Response Plan (TCRP), monitoring, or data collection.</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1. "It also provides guidance on the collection, reporting and analysis of MMIP data; offers resource information for Tribal governments; and provides best practices for culturally appropriate victim services and for returning a loved one home."  
-2. "Specifically, it directs the U.S. Department of Justice to develop guidelines to continually improve communication and coordination among tribal, federal, state and local law enforcement agencies in response to MMIP situations."  
-3. "These guidelines are evergreen with ongoing opportunities for input and recommendations."  
-4. "Following hundreds of hours of consultation with Alaska Tribes and tribal agencies, federal, state, local and tribal law enforcement and victim service providers."  </t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>The legislation employs gender-inclusive language by using the term "missing and murdered Indigenous persons," which encompasses all Indigenous individuals affected by violence, not just women. This approach acknowledges that both men and women within Indigenous communities face threats and violence. Such terminology promotes a broader understanding of the crisis and highlights the need for inclusive responses that address the experiences of all Indigenous individuals.</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>The legislation addresses the initiative by referring to "missing and murdered Alaska Natives and Native Americans," which includes all Indigenous individuals, not just women. It consistently uses terms like "missing indigenous people" and "missing persons," ensuring that the language remains gender-neutral throughout the document. This approach acknowledges the experiences of all members of Indigenous communities affected by violence and missing person cases.</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. "Federal prosecutors and the FBI are to enhance investigations into missing persons, develop protocols for law enforcement, improve data collection and analysis, and provide training and technical assistance."  
-2. "The MMIP Coordinator will work closely with federal, tribal, state, and local agencies to develop common protocols and procedures for responding to reports of missing or murdered indigenous people."  </t>
+          <t xml:space="preserve">1. "This program is a critical next step in the department’s ongoing effort to address this crisis, which has affected tribes and communities across our region and country."  
+2. “This support includes assisting in the investigation of unresolved MMIP cases and related crimes, and promoting communication, coordination, and collaboration among federal, tribal, local, and state law enforcement and non-governmental partners on MMIP issues.”  
+3. “The Department awarded $268 million in grants to help enhance Tribal justice systems and strengthen law enforcement responses.”  </t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Somewhat</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Yes. The legislation indicates that there have been "hundreds of hours of consultation with Alaska Tribes, tribal agencies, victim service providers, and federal, state, local, and tribal law enforcement," showcasing a significant level of input from various stakeholders, including those from Indigenous communities. Additionally, the ongoing opportunities for input and recommendations suggest that the voices of MMIP survivors and their families are being considered in the development of the guidelines. Thus, the level of input is not only present but is also emphasized as crucial to the initiative's effectiveness.</t>
+          <t>Yes. The legislation emphasizes the involvement of Indigenous communities and leaders through partnerships with representatives from each of the nine federally recognized Tribes in Oregon, which suggests a level of input from those communities. Cedar Wilkie Gillette's role as a coordinator also indicates direct Indigenous leadership and perspective in addressing the MMIP crisis, strengthening the initiative's responsiveness to the needs of MMIP survivors and their families. Additionally, the collaboration with various stakeholders implies an effort to incorporate diverse voices and experiences into the initiative.</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>S. Lane Tucker [U.S. Attorney, District of Alaska], Lisa Murkowski [U.S. Senator, Alaska], Ingrid Cumberlidge [MMIP Program Coordinator, U.S. Attorney's Office]</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr"/>
+          <t>Cedar Wilkie Gillette [Mandan, Hidatsa, Arikara Nation], Representative from each of the nine federally recognized Tribes in Oregon [Burns Paiute Tribe], Representative from each of the nine federally recognized Tribes in Oregon [Confederated Tribes of Grand Ronde], Representative from each of the nine federally recognized Tribes in Oregon [Confederated Tribes of Siletz Indians], Representative from each of the nine federally recognized Tribes in Oregon [Confederated Tribes of the Umatilla Indian Reservation], Representative from each of the nine federally recognized Tribes in Oregon [Confederated Tribes of the Warm Springs Reservation], Representative from each of the nine federally recognized Tribes in Oregon [Klamath Tribes], Representative from each of the nine federally recognized Tribes in Oregon [Coquille Indian Tribe], Representative from each of the nine federally recognized Tribes in Oregon [Cow Creek Band of Umpqua Tribe of Indians], Representative from each of the nine federally recognized Tribes in Oregon [Confederated Tribes of the Malheur Reservation], Natalie Wight [U.S. Attorney for the District of Oregon], Merrick B. Garland [Attorney General of the United States].</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Cedar Wilkie Gillette [Mandan, Hidatsa, Arikara Nation], Burns Paiute Tribe, Confederated Tribes of Grand Ronde, Confederated Tribes of Siletz Indians, Confederated Tribes of the Umatilla Indian Reservation, Confederated Tribes of the Warm Springs Reservation, Klamath Tribes, Coquille Indian Tribe, Cow Creek Band of Umpqua Tribe of Indians, Confederated Tribes of the Malheur Reservation.</t>
+        </is>
+      </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>Biden Administration, 2020-2024</t>
+          <t>Biden Administration, 2020 - 2024</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Taskforce, US Law Enforcement, Tribal Law Enforcement, Data Collection</t>
+          <t>Day of Recognition, US Law Enforcement, Tribal Law Enforcement</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>2022-08-30</t>
+          <t>2024-05-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adds DB ethnicity to Indigenous sponsors
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -593,7 +593,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>May 3, 2024 - Immediate Release, U.S. Attorney's Office, District of Oregon</t>
+          <t>May 3, 2024 - Immediate release, U.S. Attorney's Office, District of Oregon</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -605,27 +605,26 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>The U.S. Attorney's Office for the District of Oregon recognizes May 5, 2024, as National Missing and Murdered Indigenous Persons (MMIP) Awareness Day and appoints Cedar Wilkie Gillette as the regional MMIP Coordinator for the Northwest Region. This initiative is part of the Justice Department's MMIP Regional Outreach Program, which aims to address the crisis of missing and murdered Indigenous people through collaboration among various law enforcement agencies. The program focuses on enhancing responses to unresolved MMIP cases and allocates significant funding to support Tribal justice systems. U.S. Attorney Natalie Wight and Attorney General Merrick B. Garland emphasize the commitment to improving safety and justice for Tribal communities. The initiative reflects a broader effort to tackle violence against Indigenous peoples and strengthen community support.</t>
+          <t>The U.S. Attorney's Office for the District of Oregon is announcing the recognition of May 5, 2024, as National Missing and Murdered Indigenous Persons (MMIP) Awareness Day and the appointment of Cedar Wilkie Gillette as the MMIP Regional Coordinator for the Northwest Region. This initiative aims to address the crisis of missing and murdered Indigenous people through the Justice Department’s MMIP Regional Outreach Program, which launched in July 2023. The program will place 10 attorneys and coordinators across five regions to support investigations and promote collaboration among various law enforcement and community partners. The announcement highlights the importance of partnership with Tribal communities and acknowledges the need for continued efforts to ensure safety and justice. The initiative also includes support from multiple federal and state agencies, aiming to enhance Tribal justice systems and respond effectively to MMIP cases.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Recognizes May 5, 2024, as National Missing and Murdered Indigenous Persons Awareness Day, raising awareness about the ongoing crisis within Indigenous communities.  
-2. Appoints Cedar Wilkie Gillette as the regional MMIP Coordinator, providing dedicated leadership to focus on the issue.  
-3. Facilitates collaboration among federal, tribal, local, and state law enforcement agencies to improve responses to unresolved MMIP cases.  
-4. Utilizes gender-inclusive language, addressing the concerns of all Indigenous individuals impacted by violence and promoting a broader understanding of the crisis.  
-5. Allocates $268 million in grants to enhance Tribal justice systems and strengthen law enforcement capabilities, thereby improving community safety.  
-6. Encourages input from Indigenous communities through partnerships with various Tribes, ensuring that the initiative is informed by their perspectives and needs.  
-7. Reflects a comprehensive approach to tackling violence against Indigenous peoples and demonstrates a commitment to justice and safety for Tribal communities.  </t>
+          <t xml:space="preserve">1. Recognizes May 5, 2024, as National Missing and Murdered Indigenous Persons (MMIP) Awareness Day, raising awareness about the crisis affecting Indigenous communities.  
+2. Appoints a MMIP Regional Coordinator to enhance coordination and support for investigations in the Northwest Region.  
+3. Establishes the MMIP Regional Outreach Program to place 10 attorneys and coordinators in key regions, promoting collaboration among law enforcement and community partners.  
+4. Aims to improve safety and justice for Indigenous peoples by fostering partnerships with Tribal communities.  
+5. Enhances the capacity of federal and state agencies to respond effectively to MMIP cases and strengthen Tribal justice systems.  
+6. Utilizes gender-inclusive language, addressing the crisis of missing and murdered Indigenous persons across all gender identities.  </t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>1. The legislation lacks specified mechanisms for evaluation, leaving uncertainty about how success will be measured or activities assessed.  
-2. There is no mention of direct input or consultation from MMIP survivors and relatives, which may limit responsiveness to their specific needs and concerns.  
-3. The absence of a final report or data collection efforts may hinder the ability to track progress and identify effective strategies over time.  
-4. While it supports law enforcement, the focus may not fully address the root causes of violence against Indigenous peoples, such as socio-economic disparities.  
-5. The language and initiatives may require more specificity on implementation timelines and accountability structures to ensure meaningful action is taken.</t>
+          <t>1. There are no specific mechanisms for evaluation mentioned in the legislation, which may limit accountability and assessment of effectiveness.  
+2. The legislation does not provide explicit details regarding consultations or direct input from MMIP survivors or relatives, which may hinder the inclusivity of Indigenous voices in the initiative.  
+3. While it acknowledges partnerships with Tribal communities, the lack of detailed engagement strategies may result in missed opportunities for deeper collaboration.  
+4. The focus on awareness and coordination does not directly address systemic issues contributing to the MMIP crisis, such as root causes of violence against Indigenous peoples.  
+5. The effectiveness of the MMIP Regional Outreach Program may depend on the availability of resources and commitment from federal and state agencies, which could vary.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -635,7 +634,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>1. The legislation does not specify any mechanisms for evaluation such as a final report, consultation with community, tribal consultation, a Tribal Crisis Response Plan (TCRP), monitoring, or data collection.</t>
+          <t>1. None mentioned.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -645,7 +644,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>The legislation employs gender-inclusive language by using the term "missing and murdered Indigenous persons," which encompasses all Indigenous individuals affected by violence, not just women. This approach acknowledges that both men and women within Indigenous communities face threats and violence. Such terminology promotes a broader understanding of the crisis and highlights the need for inclusive responses that address the experiences of all Indigenous individuals.</t>
+          <t>The legislation uses gender inclusive language by referring to the broader crisis of missing and murdered Indigenous persons (MMIP) rather than limiting the focus solely to women. This approach acknowledges that individuals of all genders can be affected by this issue, thereby fostering a more comprehensive understanding of the crisis. Additionally, language such as "people throughout American Indian and Alaska Native communities" reinforces inclusivity.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -655,9 +654,10 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. "This program is a critical next step in the department’s ongoing effort to address this crisis, which has affected tribes and communities across our region and country."  
-2. “This support includes assisting in the investigation of unresolved MMIP cases and related crimes, and promoting communication, coordination, and collaboration among federal, tribal, local, and state law enforcement and non-governmental partners on MMIP issues.”  
-3. “The Department awarded $268 million in grants to help enhance Tribal justice systems and strengthen law enforcement responses.”  </t>
+          <t xml:space="preserve">1. "Launched in July 2023, the MMIP Regional Outreach Program permanently places 10 attorneys and coordinators in five designated regions across the United States to aid in the prevention and response to missing or murdered indigenous people." 
+2. "This support includes assisting in the investigation of unresolved MMIP cases and related crimes, and promoting communication, coordination, and collaboration among federal, tribal, local, and state law enforcement and non-governmental partners on MMIP issues." 
+3. "We seek to honor those who are still missing, those who were stolen from their communities, and their loved ones who are left with unimaginable pain." 
+4. "This program is a critical next step in the department’s ongoing effort to address this crisis, which has affected tribes and communities across our region and country." </t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -667,17 +667,17 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Yes. The legislation emphasizes the involvement of Indigenous communities and leaders through partnerships with representatives from each of the nine federally recognized Tribes in Oregon, which suggests a level of input from those communities. Cedar Wilkie Gillette's role as a coordinator also indicates direct Indigenous leadership and perspective in addressing the MMIP crisis, strengthening the initiative's responsiveness to the needs of MMIP survivors and their families. Additionally, the collaboration with various stakeholders implies an effort to incorporate diverse voices and experiences into the initiative.</t>
+          <t>Somewhat. The legislation acknowledges the ongoing collaboration with Tribal communities and mentions that the U.S. Attorney’s Office for the District of Oregon is partnering with various stakeholders, which can include survivors and their families. However, specific details regarding consultations or direct input from MMIP survivors or relatives are not explicitly outlined in the text.</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Cedar Wilkie Gillette [Mandan, Hidatsa, Arikara Nation], Representative from each of the nine federally recognized Tribes in Oregon [Burns Paiute Tribe], Representative from each of the nine federally recognized Tribes in Oregon [Confederated Tribes of Grand Ronde], Representative from each of the nine federally recognized Tribes in Oregon [Confederated Tribes of Siletz Indians], Representative from each of the nine federally recognized Tribes in Oregon [Confederated Tribes of the Umatilla Indian Reservation], Representative from each of the nine federally recognized Tribes in Oregon [Confederated Tribes of the Warm Springs Reservation], Representative from each of the nine federally recognized Tribes in Oregon [Klamath Tribes], Representative from each of the nine federally recognized Tribes in Oregon [Coquille Indian Tribe], Representative from each of the nine federally recognized Tribes in Oregon [Cow Creek Band of Umpqua Tribe of Indians], Representative from each of the nine federally recognized Tribes in Oregon [Confederated Tribes of the Malheur Reservation], Natalie Wight [U.S. Attorney for the District of Oregon], Merrick B. Garland [Attorney General of the United States].</t>
+          <t>Cedar Wilkie Gillette [Mandan, Hidatsa, Arikara Nation], Bree R. Black Horse [Assistant U.S. Attorney, Eastern District of Washington], Natalie Wight [U.S. Attorney for the District of Oregon], Merrick B. Garland [Attorney General of the United States]</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>Cedar Wilkie Gillette [Mandan, Hidatsa, Arikara Nation], Burns Paiute Tribe, Confederated Tribes of Grand Ronde, Confederated Tribes of Siletz Indians, Confederated Tribes of the Umatilla Indian Reservation, Confederated Tribes of the Warm Springs Reservation, Klamath Tribes, Coquille Indian Tribe, Cow Creek Band of Umpqua Tribe of Indians, Confederated Tribes of the Malheur Reservation.</t>
+          <t>Cedar Wilkie Gillette [Mandan, Hidatsa, Arikara Nation, Turtle Mountain Band of Chippewa]</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">

</xml_diff>

<commit_message>
Updates sponsors, indigenous sponsors, with DB
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -593,7 +593,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>May 3, 2024 - Immediate release, U.S. Attorney's Office, District of Oregon</t>
+          <t>May 3, 2024 - For Immediate Release, U.S. Attorney's Office, District of Oregon</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -605,26 +605,25 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>The U.S. Attorney's Office for the District of Oregon is announcing the recognition of May 5, 2024, as National Missing and Murdered Indigenous Persons (MMIP) Awareness Day and the appointment of Cedar Wilkie Gillette as the MMIP Regional Coordinator for the Northwest Region. This initiative aims to address the crisis of missing and murdered Indigenous people through the Justice Department’s MMIP Regional Outreach Program, which launched in July 2023. The program will place 10 attorneys and coordinators across five regions to support investigations and promote collaboration among various law enforcement and community partners. The announcement highlights the importance of partnership with Tribal communities and acknowledges the need for continued efforts to ensure safety and justice. The initiative also includes support from multiple federal and state agencies, aiming to enhance Tribal justice systems and respond effectively to MMIP cases.</t>
+          <t>The U.S. Attorney's Office for the District of Oregon recognizes May 5, 2024, as National Missing and Murdered Indigenous Persons (MMIP) Awareness Day and announces the appointment of Cedar Wilkie Gillette as the MMIP Regional Coordinator for the Northwest Region. This initiative is part of the Justice Department’s MMIP Regional Outreach Program, which aims to address the crisis affecting Indigenous communities by placing coordinators and attorneys in designated regions. The program promotes collaboration among federal, tribal, local, and state law enforcement agencies to improve the investigation and handling of unresolved MMIP cases. The announcement highlights ongoing efforts to honor missing Indigenous individuals and support their communities. Additionally, the initiative aligns with various directives aimed at enhancing public safety for Native Americans and addressing related violence issues.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Recognizes May 5, 2024, as National Missing and Murdered Indigenous Persons (MMIP) Awareness Day, raising awareness about the crisis affecting Indigenous communities.  
-2. Appoints a MMIP Regional Coordinator to enhance coordination and support for investigations in the Northwest Region.  
-3. Establishes the MMIP Regional Outreach Program to place 10 attorneys and coordinators in key regions, promoting collaboration among law enforcement and community partners.  
-4. Aims to improve safety and justice for Indigenous peoples by fostering partnerships with Tribal communities.  
-5. Enhances the capacity of federal and state agencies to respond effectively to MMIP cases and strengthen Tribal justice systems.  
-6. Utilizes gender-inclusive language, addressing the crisis of missing and murdered Indigenous persons across all gender identities.  </t>
+          <t xml:space="preserve">1. Raises awareness for the crisis of Missing and Murdered Indigenous Persons (MMIP) by designating a specific day of recognition.  
+2. Appoints a dedicated MMIP Regional Coordinator to enhance efforts in addressing and responding to MMIP cases within designated regions.  
+3. Promotes collaboration and communication among federal, tribal, local, and state law enforcement agencies, improving the investigation of unresolved MMIP cases.  
+4. Provides support to Indigenous communities by recognizing their specific issues and challenges related to violence and safety.  
+5. Aligns with ongoing directives aimed at enhancing public safety for Native Americans, thereby addressing related violence issues more effectively.  </t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>1. There are no specific mechanisms for evaluation mentioned in the legislation, which may limit accountability and assessment of effectiveness.  
-2. The legislation does not provide explicit details regarding consultations or direct input from MMIP survivors or relatives, which may hinder the inclusivity of Indigenous voices in the initiative.  
-3. While it acknowledges partnerships with Tribal communities, the lack of detailed engagement strategies may result in missed opportunities for deeper collaboration.  
-4. The focus on awareness and coordination does not directly address systemic issues contributing to the MMIP crisis, such as root causes of violence against Indigenous peoples.  
-5. The effectiveness of the MMIP Regional Outreach Program may depend on the availability of resources and commitment from federal and state agencies, which could vary.</t>
+          <t xml:space="preserve">1. The legislation does not specify mechanisms for evaluation or feedback from Indigenous communities, which could limit accountability and effectiveness.  
+2. There is a lack of explicit involvement or consultation with MMIP survivors and their families, potentially undermining the initiative's connection to those most affected by the crisis.  
+3. While it promotes collaboration among law enforcement agencies, it may not adequately address the systemic barriers and challenges that prevent effective responses to MMIP cases.  
+4. The focus on awareness and coordination may not be sufficient to produce tangible outcomes without a concrete action plan or measurable goals.  
+5. The reliance on federal and state law enforcement might alienate some Indigenous communities that prefer self-determined approaches to justice and safety.  </t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -634,7 +633,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>1. None mentioned.</t>
+          <t>The legislation does not explicitly mention specific mechanisms for evaluation such as a final report, consultation with community, tribal consultation, a Tribal Crisis Response Plan (TCRP), monitoring, or data collection. Therefore, there are no entries to list.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -644,7 +643,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>The legislation uses gender inclusive language by referring to the broader crisis of missing and murdered Indigenous persons (MMIP) rather than limiting the focus solely to women. This approach acknowledges that individuals of all genders can be affected by this issue, thereby fostering a more comprehensive understanding of the crisis. Additionally, language such as "people throughout American Indian and Alaska Native communities" reinforces inclusivity.</t>
+          <t>Yes, the legislation uses gender inclusive language by referring to the crisis as the Missing and Murdered Indigenous Persons (MMIP) Awareness Day, which encompasses both women and men, rather than focusing solely on women. Additionally, it addresses the broader impact of violence affecting Indigenous communities, explicitly recognizing the issues faced by both genders. This approach emphasizes a collective responsibility and partnership to address the crisis among all Indigenous people.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -654,10 +653,9 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. "Launched in July 2023, the MMIP Regional Outreach Program permanently places 10 attorneys and coordinators in five designated regions across the United States to aid in the prevention and response to missing or murdered indigenous people." 
-2. "This support includes assisting in the investigation of unresolved MMIP cases and related crimes, and promoting communication, coordination, and collaboration among federal, tribal, local, and state law enforcement and non-governmental partners on MMIP issues." 
-3. "We seek to honor those who are still missing, those who were stolen from their communities, and their loved ones who are left with unimaginable pain." 
-4. "This program is a critical next step in the department’s ongoing effort to address this crisis, which has affected tribes and communities across our region and country." </t>
+          <t>1. "The U.S. Attorney’s Office for the District of Oregon joins its partners across the federal government, as well as people throughout American Indian and Alaska Native communities, in recognizing May 5, 2024, as National Missing and Murdered Indigenous Persons (MMIP) Awareness Day."
+2. "Launched in July 2023, the MMIP Regional Outreach Program permanently places 10 attorneys and coordinators in five designated regions across the United States to aid in the prevention and response to missing or murdered indigenous people."
+3. "This support includes assisting in the investigation of unresolved MMIP cases and related crimes, and promoting communication, coordination, and collaboration among federal, tribal, local, and state law enforcement and non-governmental partners on MMIP issues."</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -667,12 +665,12 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Somewhat. The legislation acknowledges the ongoing collaboration with Tribal communities and mentions that the U.S. Attorney’s Office for the District of Oregon is partnering with various stakeholders, which can include survivors and their families. However, specific details regarding consultations or direct input from MMIP survivors or relatives are not explicitly outlined in the text.</t>
+          <t>Somewhat. The legislation acknowledges the involvement of the U.S. Attorney’s Office for the District of Oregon and various federal partners in recognizing Missing and Murdered Indigenous Persons Awareness Day, indicating a level of engagement with Indigenous communities. However, while it mentions efforts to promote communication and collaboration among federal, tribal, local, and state law enforcement, it doesn’t specify direct input or consultations with MMIP survivors or their families, suggesting that while there is some input, it may not be comprehensive.</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Cedar Wilkie Gillette [Mandan, Hidatsa, Arikara Nation], Bree R. Black Horse [Assistant U.S. Attorney, Eastern District of Washington], Natalie Wight [U.S. Attorney for the District of Oregon], Merrick B. Garland [Attorney General of the United States]</t>
+          <t>Cedar Wilkie Gillette [Mandan, Hidatsa, Arikara Nation, Turtle Mountain Band of Chippewa], Bree R. Black Horse, Natalie Wight [U.S. Attorney for the District of Oregon], Merrick B. Garland [Attorney General]</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">

</xml_diff>

<commit_message>
Clears chat history after bill processing
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:Z3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -563,12 +563,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>OR</t>
+          <t>National</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>U.S. Attorney's Office Joins in Recognizing Missing and Murdered Indigenous Persons Awareness Day and Announces Appointment of Regional MMIP Coordinator</t>
+          <t>Justice Department Strengthens Efforts, Builds Partnerships to Address the Crisis of Missing or Murdered Indigenous Persons</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -588,42 +588,42 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Department of Justice</t>
+          <t>Department of Justice, Department of the Interior</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>May 3, 2024 - For Immediate Release, U.S. Attorney's Office, District of Oregon</t>
+          <t>May 3, 2024 - For Immediate Release, U.S. Attorney's Office, Eastern District of Oklahoma</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://www.justice.gov/usao-or/pr/us-attorneys-office-joins-recognizing-missing-and-murdered-indigenous-persons-1</t>
+          <t>https://www.justice.gov/usao-edok/pr/justice-department-strengthens-efforts-builds-partnerships-address-crisis-missing-or</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>The U.S. Attorney's Office for the District of Oregon recognizes May 5, 2024, as National Missing and Murdered Indigenous Persons (MMIP) Awareness Day and announces the appointment of Cedar Wilkie Gillette as the MMIP Regional Coordinator for the Northwest Region. This initiative is part of the Justice Department’s MMIP Regional Outreach Program, which aims to address the crisis affecting Indigenous communities by placing coordinators and attorneys in designated regions. The program promotes collaboration among federal, tribal, local, and state law enforcement agencies to improve the investigation and handling of unresolved MMIP cases. The announcement highlights ongoing efforts to honor missing Indigenous individuals and support their communities. Additionally, the initiative aligns with various directives aimed at enhancing public safety for Native Americans and addressing related violence issues.</t>
+          <t>The Justice Department is strengthening efforts and building partnerships to address the crisis of missing or murdered Indigenous persons (MMIP), particularly in American Indian and Alaska Native communities. The initiative coincides with the recognition of May 5 as National MMIP Awareness Day and focuses on tackling human trafficking and public safety challenges within Tribal communities. Attorney General Merrick B. Garland emphasized the need for enhanced collaboration and acknowledgment of the violence these communities have faced. The department's strategy includes the establishment of a Missing or Murdered Indigenous Persons Regional Outreach Program to prioritize MMIP cases and increase resources dedicated to these issues. Additionally, collaborative responses to recommendations from the Not Invisible Act Commission aim to combat this ongoing crisis and support healing for Indigenous peoples.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Raises awareness for the crisis of Missing and Murdered Indigenous Persons (MMIP) by designating a specific day of recognition.  
-2. Appoints a dedicated MMIP Regional Coordinator to enhance efforts in addressing and responding to MMIP cases within designated regions.  
-3. Promotes collaboration and communication among federal, tribal, local, and state law enforcement agencies, improving the investigation of unresolved MMIP cases.  
-4. Provides support to Indigenous communities by recognizing their specific issues and challenges related to violence and safety.  
-5. Aligns with ongoing directives aimed at enhancing public safety for Native Americans, thereby addressing related violence issues more effectively.  </t>
+          <t>1. Strengthens efforts to address the crisis of missing or murdered Indigenous persons (MMIP) specifically in American Indian and Alaska Native communities.
+2. Establishes National MMIP Awareness Day to promote recognition and support for affected communities.
+3. Fosters enhanced collaboration between the Justice Department and Tribal communities to tackle human trafficking and public safety challenges.
+4. Introduces the Missing or Murdered Indigenous Persons Regional Outreach Program to prioritize MMIP cases and allocate necessary resources.
+5. Provides $268 million in grants to enhance Tribal justice systems and improve responses to related issues, including child abuse and domestic violence.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The legislation does not specify mechanisms for evaluation or feedback from Indigenous communities, which could limit accountability and effectiveness.  
-2. There is a lack of explicit involvement or consultation with MMIP survivors and their families, potentially undermining the initiative's connection to those most affected by the crisis.  
-3. While it promotes collaboration among law enforcement agencies, it may not adequately address the systemic barriers and challenges that prevent effective responses to MMIP cases.  
-4. The focus on awareness and coordination may not be sufficient to produce tangible outcomes without a concrete action plan or measurable goals.  
-5. The reliance on federal and state law enforcement might alienate some Indigenous communities that prefer self-determined approaches to justice and safety.  </t>
+          <t>1. The legislation does not include specific mechanisms for evaluation, making it difficult to assess the effectiveness of the initiatives implemented.  
+2. There is limited detail on the extent of input from MMIP survivors, their relatives, or Indigenous politicians, which may lead to gaps in representation and responsiveness to community needs.  
+3. While the legislation emphasizes partnerships, it lacks concrete strategies for engaging Indigenous communities meaningfully in the decision-making process.  
+4. Funding allocations, while significant, may not sufficiently address the root causes of violence and crime affecting Indigenous peoples beyond immediate law enforcement responses.  
+5. The focus on awareness days and programs may not translate into sustained action or long-term solutions for the underlying issues faced by MMIP communities.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -633,7 +633,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>The legislation does not explicitly mention specific mechanisms for evaluation such as a final report, consultation with community, tribal consultation, a Tribal Crisis Response Plan (TCRP), monitoring, or data collection. Therefore, there are no entries to list.</t>
+          <t>1. There are no specific mechanisms for evaluation mentioned in the legislation.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -643,7 +643,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Yes, the legislation uses gender inclusive language by referring to the crisis as the Missing and Murdered Indigenous Persons (MMIP) Awareness Day, which encompasses both women and men, rather than focusing solely on women. Additionally, it addresses the broader impact of violence affecting Indigenous communities, explicitly recognizing the issues faced by both genders. This approach emphasizes a collective responsibility and partnership to address the crisis among all Indigenous people.</t>
+          <t>The legislation uses gender-inclusive language by addressing the crisis as the "Missing or Murdered Indigenous Persons" (MMIP) rather than exclusively focusing on women. This broader terminology acknowledges that individuals of all genders can be affected by this crisis, reflecting a more inclusive approach. Additionally, the language emphasizes the collective impact on families and communities, further supporting inclusivity.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -653,9 +653,10 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1. "The U.S. Attorney’s Office for the District of Oregon joins its partners across the federal government, as well as people throughout American Indian and Alaska Native communities, in recognizing May 5, 2024, as National Missing and Murdered Indigenous Persons (MMIP) Awareness Day."
-2. "Launched in July 2023, the MMIP Regional Outreach Program permanently places 10 attorneys and coordinators in five designated regions across the United States to aid in the prevention and response to missing or murdered indigenous people."
-3. "This support includes assisting in the investigation of unresolved MMIP cases and related crimes, and promoting communication, coordination, and collaboration among federal, tribal, local, and state law enforcement and non-governmental partners on MMIP issues."</t>
+          <t>1. "The Justice Department joins its partners across the federal government, as well as people throughout American Indian and Alaska Native communities, in recognizing May 5 as National Missing or Murdered Indigenous Persons (MMIP) Awareness Day."  
+2. "The MMIP Regional Outreach Program prioritizes MMIP cases consistent with the Deputy Attorney General’s July 2022 directive to U.S. Attorneys’ offices promoting public safety in Indian country."  
+3. "The Department awarded $268 million in grants to help enhance Tribal justice systems and strengthen law enforcement responses."  
+4. "These awards have also gone toward improving the handling of child abuse cases, combating domestic and sexual violence, supporting Tribal youth programs, and strengthening victim services in Tribal communities."</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -665,19 +666,15 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Somewhat. The legislation acknowledges the involvement of the U.S. Attorney’s Office for the District of Oregon and various federal partners in recognizing Missing and Murdered Indigenous Persons Awareness Day, indicating a level of engagement with Indigenous communities. However, while it mentions efforts to promote communication and collaboration among federal, tribal, local, and state law enforcement, it doesn’t specify direct input or consultations with MMIP survivors or their families, suggesting that while there is some input, it may not be comprehensive.</t>
+          <t>Somewhat. The legislation acknowledges the importance of partnerships with Tribal communities and emphasizes honoring those who are missing, which indicates a level of input from Indigenous communities. However, it does not explicitly detail the extent of involvement from MMIP survivors, their relatives, or Indigenous politicians in shaping or influencing the initiatives discussed.</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Cedar Wilkie Gillette [Mandan, Hidatsa, Arikara Nation, Turtle Mountain Band of Chippewa], Bree R. Black Horse, Natalie Wight [U.S. Attorney for the District of Oregon], Merrick B. Garland [Attorney General]</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>Cedar Wilkie Gillette [Mandan, Hidatsa, Arikara Nation, Turtle Mountain Band of Chippewa]</t>
-        </is>
-      </c>
+          <t>Merrick B. Garland [U.S. Attorney General], Christopher J. Wilson [United States Attorney for the Eastern District of Oklahoma], Christopher Wray [FBI Director], Anne Milgram [DEA Administrator]</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr">
         <is>
           <t>Biden Administration, 2020 - 2024</t>
@@ -691,6 +688,140 @@
       <c r="Z2" t="inlineStr">
         <is>
           <t>2024-05-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>National</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Justice Department Strengthens Efforts to Address the Crisis of Missing or Murdered Indigenous Persons</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Department of Justice</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Friday, May 5, 2023 - For Immediate Release, U.S. Attorney's Office, Northern District of California</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>https://www.justice.gov/usao-ndca/pr/justice-department-strengthens-efforts-address-crisis-missing-or-murdered-indigenous</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>The Justice Department has strengthened its efforts to address the crisis of Missing or Murdered Indigenous Persons (MMIP), emphasizing the need for a coordinated response across government agencies and partnerships with Tribal communities. Acknowledging the unacceptable levels of violence affecting American Indian and Alaska Native populations, the department has launched initiatives and provided resources to enhance public safety in Indian country. The Not Invisible Act Commission, co-launched by Deputy Attorney General Lisa Monaco and Secretary of the Interior Deb Haaland, aims to reduce violence against these communities. The initiative also involves updating policies, developing response plans for missing persons cases, and increasing grant funding to support Tribal nations. Overall, the department is committed to utilizing all available resources to combat the MMIP crisis and support affected communities.</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Strengthens coordinated efforts across government agencies and Tribal communities to address the MMIP crisis effectively.  
+2. Promotes a more inclusive approach by recognizing the experiences of all Indigenous individuals affected by violence, not just women.  
+3. Establishes initiatives such as the Not Invisible Act Commission to develop targeted recommendations for reducing violence against Indigenous populations.  
+4. Enhances public safety in Indian country through updated policies, response plans for missing persons, and increased grant funding to support Tribal nations.  
+5. Amplifies the voices of MMIP survivors and their families by involving Indigenous communities in the decision-making processes and initiatives.  
+6. Provides a national platform to raise awareness and acknowledge the crisis through events like the National Missing or Murdered Indigenous Persons Awareness Day.  
+7. Implements mechanisms for data collection, analysis, and reporting strategies that will inform future efforts and resource allocation related to MMIP cases.  </t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Implementation challenges may arise due to the complexity of coordinating multiple government agencies and Tribal communities, potentially slowing down progress.  
+2. The effectiveness of the initiatives may be limited if sufficient funding and resources are not consistently allocated to support ongoing efforts.  
+3. Some individuals may feel that awareness efforts alone, such as the National Missing or Murdered Indigenous Persons Awareness Day, do not lead to substantial action or change in systemic issues.  
+4. Reliance on government-led initiatives may overlook or undervalue grassroots efforts or solutions proposed by Indigenous communities themselves.  
+5. The potential for insufficient follow-up on recommendations made by the Not Invisible Act Commission could undermine the intended impact of the initiatives.  </t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>1. "The Commission will deliver recommendations for addressing the MMIP crisis to the Attorney General and the Secretary."
+2. "The Department of Justice and the Department of the Interior submitted a report pursuant to Sections 2 and 4(a) of Executive Order 14053."
+3. "It will inform long-term data collection, analysis, and reporting strategies on MMIP cases."</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>The legislation refers to the "Missing or Murdered Indigenous Persons (MMIP)" crisis, intentionally broadening the focus beyond just women to include all Indigenous individuals who may be affected. By using the term "Persons" instead of specifying gender, it promotes a more inclusive approach to addressing this issue. This language shift acknowledges the experiences of all genders within Indigenous communities, aligning with contemporary discussions about inclusivity and diversity.</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>1. "The Justice Department joins its partners across the federal government, as well as people throughout American Indian and Alaska Native communities, in recognizing May 5, 2023 as National Missing or Murdered Indigenous Persons Awareness Day."
+2. "Acknowledging the many American Indian and Alaska Native people who have suffered, and continue to suffer, from the pain of a missing loved one or of violent crime serves as an important reminder of the urgency and importance of the department’s work to respond to the crisis of missing or murdered indigenous persons."
+3. "In addition to our core law-enforcement work, we are providing grant funding and guidance to help Tribes develop response plans for missing-persons cases, partner effectively with local law enforcement, and provide resources for victims of crime."</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Somewhat</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Yes. The legislation highlights the involvement of Indigenous communities and leaders, emphasizing the collaboration between the Justice Department and Tribal governments to address the crisis of Missing or Murdered Indigenous Persons (MMIP). Specifically, it references the Not Invisible Act Commission, which includes participation from department leaders and subject matter experts who are engaging with community representatives to deliver recommendations for addressing the issue. Additionally, the establishment of the National Native American Outreach Services Liaison indicates a commitment to amplifying the voices of crime victims and their families from Indigenous communities.</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Lisa Monaco [Deputy Attorney General], Deb Haaland [Laguna Pueblo], Merrick B. Garland [Attorney General], Ismail Ramsey [U.S. Attorney for the Northern District of California]</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Deb Haaland [Laguna Pueblo]</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>Biden Administration, 2020-2024</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>Taskforce, Day of Recognition, US Law Enforcement, Tribal Law Enforcement, Data Collection</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>2023-05-05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Split centering Indigenous voices and survivor voices into their dedicated columns
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z3"/>
+  <dimension ref="A1:AB2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -526,35 +526,45 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
+          <t>Level of Survivor / Relative Input?</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
           <t>Level of Survivor / Relative Input</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Centering of Indigenous Voices?</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Centering of Indigenous Voices</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Sponsors</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Indigenous Sponsorship</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Session</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Categories</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Last Update</t>
         </is>
@@ -563,17 +573,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>National</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Justice Department Strengthens Efforts, Builds Partnerships to Address the Crisis of Missing or Murdered Indigenous Persons</t>
+          <t>Establishes a task force on missing women and girls who are black, indigenous and people of color (BIPOC) to develop policy changes that will work to address the lack of care and concern for missing and murdered BIPOC women and girls with New York state governmental agencies.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DOJ24-570</t>
+          <t>S04266</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -588,240 +598,123 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Department of Justice, Department of the Interior</t>
+          <t>Senate</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>May 3, 2024 - For Immediate Release, U.S. Attorney's Office, Eastern District of Oklahoma</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
+          <t>2023-12-21 - S: APPROVAL MEMO.58</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://legiscan.com/NY/bill/S04266/2023</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://www.justice.gov/usao-edok/pr/justice-department-strengthens-efforts-builds-partnerships-address-crisis-missing-or</t>
+          <t>https://legiscan.com/NY/bill/S04266/2023</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>The Justice Department is strengthening efforts and building partnerships to address the crisis of missing or murdered Indigenous persons (MMIP), particularly in American Indian and Alaska Native communities. The initiative coincides with the recognition of May 5 as National MMIP Awareness Day and focuses on tackling human trafficking and public safety challenges within Tribal communities. Attorney General Merrick B. Garland emphasized the need for enhanced collaboration and acknowledgment of the violence these communities have faced. The department's strategy includes the establishment of a Missing or Murdered Indigenous Persons Regional Outreach Program to prioritize MMIP cases and increase resources dedicated to these issues. Additionally, collaborative responses to recommendations from the Not Invisible Act Commission aim to combat this ongoing crisis and support healing for Indigenous peoples.</t>
+          <t>The legislation establishes a task force in New York to address the crisis of missing women and girls who are Black, Indigenous, and people of color (BIPOC). The task force will consist of various government officials and appointed members representing impacted communities and will focus on policy changes, education, data collection, and awareness campaigns related to this issue. It aims to improve the cultural competency of first responders and develop strategies to prevent the abduction of BIPOC women and girls. The task force is required to hold public hearings and submit a report with findings and recommendations within two years. The act will take effect 60 days after becoming law and will expire three years later.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1. Strengthens efforts to address the crisis of missing or murdered Indigenous persons (MMIP) specifically in American Indian and Alaska Native communities.
-2. Establishes National MMIP Awareness Day to promote recognition and support for affected communities.
-3. Fosters enhanced collaboration between the Justice Department and Tribal communities to tackle human trafficking and public safety challenges.
-4. Introduces the Missing or Murdered Indigenous Persons Regional Outreach Program to prioritize MMIP cases and allocate necessary resources.
-5. Provides $268 million in grants to enhance Tribal justice systems and improve responses to related issues, including child abuse and domestic violence.</t>
+          <t xml:space="preserve">1. Establishes a dedicated task force to specifically address the crisis of missing women and girls who are Black, Indigenous, and people of color (BIPOC), ensuring focused attention on an urgent issue.  
+2. Promotes policy changes and cultural competency among first responders, which can lead to improved responses to cases involving missing BIPOC individuals.  
+3. Facilitates community engagement through public hearings and written input, allowing the voices of MMIP survivors and their relatives to be heard.  
+4. Develops a strategy for data collection, enhancing the understanding of the issue and supporting informed decision-making.  
+5. Implements educational and awareness campaigns to better inform BIPOC communities about prevention and protection protocols regarding missing individuals.  
+6. Allows for periodic reporting and public dissemination of findings, promoting transparency and accountability in addressing the crisis.  
+7. Engages Indigenous organizations and advocates in the process, ensuring that their unique perspectives and needs are considered.  </t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>1. The legislation does not include specific mechanisms for evaluation, making it difficult to assess the effectiveness of the initiatives implemented.  
-2. There is limited detail on the extent of input from MMIP survivors, their relatives, or Indigenous politicians, which may lead to gaps in representation and responsiveness to community needs.  
-3. While the legislation emphasizes partnerships, it lacks concrete strategies for engaging Indigenous communities meaningfully in the decision-making process.  
-4. Funding allocations, while significant, may not sufficiently address the root causes of violence and crime affecting Indigenous peoples beyond immediate law enforcement responses.  
-5. The focus on awareness days and programs may not translate into sustained action or long-term solutions for the underlying issues faced by MMIP communities.</t>
+          <t>1. The legislation primarily focuses on missing women and girls without addressing the broader issue of all missing Indigenous people, lacking gender-neutral language that could encompass all individuals.  
+2. While the task force aims to represent impacted communities, the specifics regarding Indigenous representation and the roles of Indigenous politicians are not clearly detailed, which may limit authentic community engagement.  
+3. The effectiveness of the legislation may be hindered by its temporary nature, as it will expire three years after enactment, potentially leaving critical issues unaddressed.  
+4. The requirement for public hearings and input may not sufficiently capture the voices of all affected individuals, particularly those who may not have access or resources to participate.  
+5. Although the task force will collect data, there is no mention of how this data will be used to implement actionable change or follow-up on the cases of missing persons.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. The task force shall submit to the temporary president of the senate, the speaker of the assembly, the minority leader of the senate and the minority leader of the assembly a report containing its findings and recommendations. 
+2. Such reports shall be made available to the public. 
+3. In carrying out the duties of the task force, such task force shall seek public input by holding public hearings in each region of the state and accepting public input in writing. 
+4. Develop a strategy to collect statistics, demographics, surveys, oral histories, and data analysis. </t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>1. There are no specific mechanisms for evaluation mentioned in the legislation.</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>The legislation primarily focuses on missing women and girls, specifically noting "Black, Indigenous, and people of color," which emphasizes gender in its language. While it highlights the experiences of women and girls, it does not expand its scope to include all missing Indigenous people or use gender-neutral terms that could encompass a wider demographic. Therefore, it lacks gender-inclusive language that recognizes the broader issue of missing individuals regardless of gender.</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>The legislation uses gender-inclusive language by addressing the crisis as the "Missing or Murdered Indigenous Persons" (MMIP) rather than exclusively focusing on women. This broader terminology acknowledges that individuals of all genders can be affected by this crisis, reflecting a more inclusive approach. Additionally, the language emphasizes the collective impact on families and communities, further supporting inclusivity.</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>1. "ensure BIPOC communities are educated and trained on the prevention, protection, and protocols relating to missing BIPOC women and girls as it relates to social media;"
+2. "create a state-wide awareness campaign."</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>1. "The Justice Department joins its partners across the federal government, as well as people throughout American Indian and Alaska Native communities, in recognizing May 5 as National Missing or Murdered Indigenous Persons (MMIP) Awareness Day."  
-2. "The MMIP Regional Outreach Program prioritizes MMIP cases consistent with the Deputy Attorney General’s July 2022 directive to U.S. Attorneys’ offices promoting public safety in Indian country."  
-3. "The Department awarded $268 million in grants to help enhance Tribal justice systems and strengthen law enforcement responses."  
-4. "These awards have also gone toward improving the handling of child abuse cases, combating domestic and sexual violence, supporting Tribal youth programs, and strengthening victim services in Tribal communities."</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Somewhat. The legislation acknowledges the importance of partnerships with Tribal communities and emphasizes honoring those who are missing, which indicates a level of input from Indigenous communities. However, it does not explicitly detail the extent of involvement from MMIP survivors, their relatives, or Indigenous politicians in shaping or influencing the initiatives discussed.</t>
+          <t>The legislation establishes a task force that includes members representative of communities experiencing the crisis, indicating an intention to involve those directly impacted, such as MMIP survivors and their relatives. Additionally, it emphasizes the importance of public input through hearings and written submissions, which provides avenues for survivors and their families to voice their experiences and perspectives. Moreover, the reference to the Sovereign Bodies Institute, an indigenous-led organization that focuses on missing and murdered Indigenous people, further supports the conclusion that the legislation seeks to incorporate input from these communities</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Merrick B. Garland [U.S. Attorney General], Christopher J. Wilson [United States Attorney for the Eastern District of Oklahoma], Christopher Wray [FBI Director], Anne Milgram [DEA Administrator]</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr"/>
+          <t>Somewhat</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>The legislation establishes a task force that includes members representative of communities experiencing the crisis, which suggests an intention to include individuals who may have been directly impacted, such as MMIP survivors and their relatives. Additionally, it mandates public hearings and the acceptance of written input, indicating a mechanism for community engagement. However, while Indigenous politicians are sponsoring the legislation, the specifics of their roles or direct representation of Indigenous communities within the task force are not clearly detailed, leading to an assessment of "somewhat" in terms of inclusive input.</t>
+        </is>
+      </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>Biden Administration, 2020 - 2024</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>Day of Recognition, US Law Enforcement, Tribal Law Enforcement</t>
-        </is>
-      </c>
+          <t>Sen Lea Webb (D) - District SD-052, Sen Cordell Cleare (D) - District SD-030, Sen Leroy Comrie (D) - District SD-014, Sen Jeremy Cooney (D) - District SD-056, Sen Nathalia Fernandez (D) - District SD-034, Sen Brad Hoylman-Sigal (D) - District SD-047, Sen Timothy Kennedy (D) - District SD-063, Sen Monica Martinez (D) - District SD-004, Sen Jessica Ramos (D) - District SD-013, Sen Julia Salazar (D) - District SD-018</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>2024-05-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>National</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Justice Department Strengthens Efforts to Address the Crisis of Missing or Murdered Indigenous Persons</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Department of Justice</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Friday, May 5, 2023 - For Immediate Release, U.S. Attorney's Office, Northern District of California</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>https://www.justice.gov/usao-ndca/pr/justice-department-strengthens-efforts-address-crisis-missing-or-murdered-indigenous</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>The Justice Department has strengthened its efforts to address the crisis of Missing or Murdered Indigenous Persons (MMIP), emphasizing the need for a coordinated response across government agencies and partnerships with Tribal communities. Acknowledging the unacceptable levels of violence affecting American Indian and Alaska Native populations, the department has launched initiatives and provided resources to enhance public safety in Indian country. The Not Invisible Act Commission, co-launched by Deputy Attorney General Lisa Monaco and Secretary of the Interior Deb Haaland, aims to reduce violence against these communities. The initiative also involves updating policies, developing response plans for missing persons cases, and increasing grant funding to support Tribal nations. Overall, the department is committed to utilizing all available resources to combat the MMIP crisis and support affected communities.</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1. Strengthens coordinated efforts across government agencies and Tribal communities to address the MMIP crisis effectively.  
-2. Promotes a more inclusive approach by recognizing the experiences of all Indigenous individuals affected by violence, not just women.  
-3. Establishes initiatives such as the Not Invisible Act Commission to develop targeted recommendations for reducing violence against Indigenous populations.  
-4. Enhances public safety in Indian country through updated policies, response plans for missing persons, and increased grant funding to support Tribal nations.  
-5. Amplifies the voices of MMIP survivors and their families by involving Indigenous communities in the decision-making processes and initiatives.  
-6. Provides a national platform to raise awareness and acknowledge the crisis through events like the National Missing or Murdered Indigenous Persons Awareness Day.  
-7. Implements mechanisms for data collection, analysis, and reporting strategies that will inform future efforts and resource allocation related to MMIP cases.  </t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1. Implementation challenges may arise due to the complexity of coordinating multiple government agencies and Tribal communities, potentially slowing down progress.  
-2. The effectiveness of the initiatives may be limited if sufficient funding and resources are not consistently allocated to support ongoing efforts.  
-3. Some individuals may feel that awareness efforts alone, such as the National Missing or Murdered Indigenous Persons Awareness Day, do not lead to substantial action or change in systemic issues.  
-4. Reliance on government-led initiatives may overlook or undervalue grassroots efforts or solutions proposed by Indigenous communities themselves.  
-5. The potential for insufficient follow-up on recommendations made by the Not Invisible Act Commission could undermine the intended impact of the initiatives.  </t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>1. "The Commission will deliver recommendations for addressing the MMIP crisis to the Attorney General and the Secretary."
-2. "The Department of Justice and the Department of the Interior submitted a report pursuant to Sections 2 and 4(a) of Executive Order 14053."
-3. "It will inform long-term data collection, analysis, and reporting strategies on MMIP cases."</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>The legislation refers to the "Missing or Murdered Indigenous Persons (MMIP)" crisis, intentionally broadening the focus beyond just women to include all Indigenous individuals who may be affected. By using the term "Persons" instead of specifying gender, it promotes a more inclusive approach to addressing this issue. This language shift acknowledges the experiences of all genders within Indigenous communities, aligning with contemporary discussions about inclusivity and diversity.</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>1. "The Justice Department joins its partners across the federal government, as well as people throughout American Indian and Alaska Native communities, in recognizing May 5, 2023 as National Missing or Murdered Indigenous Persons Awareness Day."
-2. "Acknowledging the many American Indian and Alaska Native people who have suffered, and continue to suffer, from the pain of a missing loved one or of violent crime serves as an important reminder of the urgency and importance of the department’s work to respond to the crisis of missing or murdered indigenous persons."
-3. "In addition to our core law-enforcement work, we are providing grant funding and guidance to help Tribes develop response plans for missing-persons cases, partner effectively with local law enforcement, and provide resources for victims of crime."</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>Somewhat</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Yes. The legislation highlights the involvement of Indigenous communities and leaders, emphasizing the collaboration between the Justice Department and Tribal governments to address the crisis of Missing or Murdered Indigenous Persons (MMIP). Specifically, it references the Not Invisible Act Commission, which includes participation from department leaders and subject matter experts who are engaging with community representatives to deliver recommendations for addressing the issue. Additionally, the establishment of the National Native American Outreach Services Liaison indicates a commitment to amplifying the voices of crime victims and their families from Indigenous communities.</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>Lisa Monaco [Deputy Attorney General], Deb Haaland [Laguna Pueblo], Merrick B. Garland [Attorney General], Ismail Ramsey [U.S. Attorney for the Northern District of California]</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>Deb Haaland [Laguna Pueblo]</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>Biden Administration, 2020-2024</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>Taskforce, Day of Recognition, US Law Enforcement, Tribal Law Enforcement, Data Collection</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>2023-05-05</t>
+          <t>2023-2024 Regular Session</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Taskforce, Data Collection, MMIP Relatives</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>2023-12-21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
User input no longer requires comma seperated lists
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AB3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -619,27 +619,25 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>The legislation establishes a task force in New York to address the crisis of missing women and girls who are Black, Indigenous, and people of color (BIPOC). The task force will consist of various government officials and appointed members representing impacted communities and will focus on policy changes, education, data collection, and awareness campaigns related to this issue. It aims to improve the cultural competency of first responders and develop strategies to prevent the abduction of BIPOC women and girls. The task force is required to hold public hearings and submit a report with findings and recommendations within two years. The act will take effect 60 days after becoming law and will expire three years later.</t>
+          <t>The legislation establishes a task force in New York focused on addressing the crisis of missing women and girls who are Black, Indigenous, and People of Color (BIPOC). This task force will consist of various state officials and representatives from affected communities, aiming to develop policy changes, raise public awareness, and improve data collection regarding missing BIPOC individuals. It seeks to enhance cultural competency among first responders and recommend preventive measures to ensure the safety of these vulnerable populations. The task force is required to hold public hearings and submit a report with findings and recommendations two years after its formation. The act will take effect 60 days after becoming law and will expire three years later.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Establishes a dedicated task force to specifically address the crisis of missing women and girls who are Black, Indigenous, and people of color (BIPOC), ensuring focused attention on an urgent issue.  
-2. Promotes policy changes and cultural competency among first responders, which can lead to improved responses to cases involving missing BIPOC individuals.  
-3. Facilitates community engagement through public hearings and written input, allowing the voices of MMIP survivors and their relatives to be heard.  
-4. Develops a strategy for data collection, enhancing the understanding of the issue and supporting informed decision-making.  
-5. Implements educational and awareness campaigns to better inform BIPOC communities about prevention and protection protocols regarding missing individuals.  
-6. Allows for periodic reporting and public dissemination of findings, promoting transparency and accountability in addressing the crisis.  
-7. Engages Indigenous organizations and advocates in the process, ensuring that their unique perspectives and needs are considered.  </t>
+          <t xml:space="preserve">1. Establishes a dedicated task force focused on the crisis of missing women and girls who are Black, Indigenous, and People of Color (BIPOC), facilitating targeted attention to this urgent issue.  
+2. Aims to develop policy changes that enhance the care and concern for missing and murdered BIPOC women and girls, thus improving the response from state governmental agencies.  
+3. Requires public hearings and the collection of community input, ensuring that the voices of affected individuals, including MMIP survivors and their relatives, are considered in the decision-making process.  
+4. Promotes awareness and education within BIPOC communities regarding prevention and protection strategies, which can help mitigate future incidents.  
+5. Develops mechanisms for data collection, allowing for better tracking and analysis of cases involving missing BIPOC individuals, which can drive informed policymaking and resource allocation.  </t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>1. The legislation primarily focuses on missing women and girls without addressing the broader issue of all missing Indigenous people, lacking gender-neutral language that could encompass all individuals.  
-2. While the task force aims to represent impacted communities, the specifics regarding Indigenous representation and the roles of Indigenous politicians are not clearly detailed, which may limit authentic community engagement.  
-3. The effectiveness of the legislation may be hindered by its temporary nature, as it will expire three years after enactment, potentially leaving critical issues unaddressed.  
-4. The requirement for public hearings and input may not sufficiently capture the voices of all affected individuals, particularly those who may not have access or resources to participate.  
-5. Although the task force will collect data, there is no mention of how this data will be used to implement actionable change or follow-up on the cases of missing persons.</t>
+          <t xml:space="preserve">1. The legislation's focus primarily on women and girls may overlook the broader issue of missing Indigenous people, failing to employ gender-neutral language consistently.  
+2. There are no specific Indigenous organizations mentioned in the legislation, which may limit direct representation and input from those who are most affected by the crisis.  
+3. The task force is set to expire three years after its formation, which may limit the long-term impact and sustainability of the proposed measures.  
+4. While public hearings are required, the effectiveness of community engagement may vary based on participation and outreach efforts, potentially resulting in inadequate representation of all affected voices.  
+5. The lack of explicit details regarding the direct involvement of MMIP survivors or Indigenous politicians in the formulation of the legislation may hinder the authenticity and relevance of the proposed solutions.  </t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -649,10 +647,9 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The task force shall submit to the temporary president of the senate, the speaker of the assembly, the minority leader of the senate and the minority leader of the assembly a report containing its findings and recommendations. 
-2. Such reports shall be made available to the public. 
-3. In carrying out the duties of the task force, such task force shall seek public input by holding public hearings in each region of the state and accepting public input in writing. 
-4. Develop a strategy to collect statistics, demographics, surveys, oral histories, and data analysis. </t>
+          <t>1. The task force shall submit a report containing its findings and recommendations to various legislative leaders (Section 2.e).
+2. The task force shall seek public input by holding public hearings in each region of the state (Section 2.d).
+3. The task force shall develop a strategy to collect statistics, demographics, surveys, oral histories, and data analysis (Section 2.c.iv).</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -662,7 +659,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>The legislation primarily focuses on missing women and girls, specifically noting "Black, Indigenous, and people of color," which emphasizes gender in its language. While it highlights the experiences of women and girls, it does not expand its scope to include all missing Indigenous people or use gender-neutral terms that could encompass a wider demographic. Therefore, it lacks gender-inclusive language that recognizes the broader issue of missing individuals regardless of gender.</t>
+          <t>The legislation primarily focuses on women and girls, specifically highlighting issues related to missing Black and Indigenous women and girls, which suggests a gender-specific approach. While it does include the term "people of color," the language does not broadly address issues concerning missing Indigenous people or use gender-neutral terms consistently. Consequently, the legislation does not fully encompass gender-inclusive language throughout its provisions.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -671,48 +668,193 @@
         </is>
       </c>
       <c r="S2" t="inlineStr">
+        <is>
+          <t>1. "ensure BIPOC communities are educated and trained on the prevention, protection, and protocols relating to missing BIPOC women and girls as it relates to social media" (Section 2.c.iii).
+2. "create a state-wide awareness campaign" (Section 2.c.vii).</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Somewhat</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>The legislation indicates that the task force will be composed of individuals who reflect the diversity of New York State and are representative of the communities experiencing the crisis, which suggests an intent to include voices from impacted groups, including MMIP survivors and their relatives. Furthermore, the task force is required to seek public input through regional hearings and written submissions, which provides a platform for these individuals to share their experiences and perspectives. However, specific organizations directly representing MMIP survivors are not explicitly mentioned in the text, leading to a "Somewhat" designation regarding the level of input from these groups</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Somewhat</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>The legislation establishes a task force that is required to seek public input by holding public hearings in each region of the state and accepting written submissions, indicating some level of engagement with affected communities, including MMIP survivors and relatives. Additionally, the language specifies that task force members should be representative of the communities experiencing this crisis, suggesting an effort to include voices from Indigenous communities. However, the specific details regarding the direct involvement of MMIP survivors or Indigenous politicians in the formulation of the legislation are not explicitly outlined, resulting in a "Somewhat" designation for input.</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Sen Lea Webb (D) - District SD-052, Sen Cordell Cleare (D) - District SD-030, Sen Leroy Comrie (D) - District SD-014, Sen Jeremy Cooney (D) - District SD-056, Sen Nathalia Fernandez (D) - District SD-034, Sen Brad Hoylman-Sigal (D) - District SD-047, Sen Timothy Kennedy (D) - District SD-063, Sen Monica Martinez (D) - District SD-004, Sen Jessica Ramos (D) - District SD-013, Sen Julia Salazar (D) - District SD-018</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>2023-2024 Regular Session</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Taskforce, Data Collection, MMIP Relatives</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>2023-12-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Establishes a task force on missing women and girls who are black, indigenous and people of color (BIPOC) to develop policy changes that will work to address the lack of care and concern for missing and murdered BIPOC women and girls with New York state governmental agencies.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>S04266</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Senate</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2023-12-21 - S: APPROVAL MEMO.58</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://legiscan.com/NY/bill/S04266/2023</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>https://legiscan.com/NY/bill/S04266/2023</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>The legislation establishes a task force in New York dedicated to addressing the issue of missing women and girls who are Black, Indigenous, and People of Color (BIPOC). It aims to develop policy changes, improve data collection, and raise public awareness about the circumstances surrounding missing BIPOC women and girls. The task force will include representatives from relevant state agencies and community members and will seek public input through hearings. It is required to submit a report with findings and recommendations within two years. The act will take effect 60 days after becoming law and will expire three years later.</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1. Establishes a task force focused on addressing the issue of missing BIPOC women and girls, promoting targeted policy changes.
+2. Facilitates improved data collection and analysis to better understand and address the crisis of missing individuals.
+3. Includes provisions for public input through hearings, allowing community members, including MMIP survivors and their relatives, to voice their concerns and experiences.
+4. Creates educational and awareness programs aimed at preventing the disappearance of BIPOC women and girls.
+5. Ensures representation from affected communities within the task force, fostering inclusivity in policy development and decision-making.</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>1. The legislation primarily focuses on missing women and girls, which may exclude broader representation of missing Indigenous individuals beyond this demographic.
+2. The language used in the legislation does not consistently employ gender-neutral terms, potentially limiting inclusivity for non-binary or gender-diverse individuals experiencing similar issues.
+3. The act has a limited duration of three years before it expires, which may hinder long-term efforts and sustainability in addressing the crisis.
+4. There is no specific mention of Indigenous organizations or partnerships that could provide cultural context and support to the task force’s initiatives.
+5. The effectiveness of the task force’s recommendations relies heavily on the cooperation and engagement of various state agencies, which may vary and impact implementation.</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>1. "On or before two years after the effective date of this act, the task force shall submit to the temporary president of the senate, the speaker of the assembly, the minority leader of the senate and the minority leader of the assembly a report containing its findings and recommendations."
+2. "In carrying out the duties of the task force, such task force shall seek public input by holding public hearings in each region of the state and accepting public input in writing."
+3. "develop a strategy to collect statistics, demographics, surveys, oral histories, and data analysis."</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>The legislation primarily focuses on missing women and girls, explicitly naming Black, Indigenous, and People of Color (BIPOC) women and girls throughout. While it addresses the significant issue of missing Indigenous individuals, it does not consistently use gender-neutral language or include a broader representation of missing Indigenous people beyond women and girls. As a result, it does not fully encompass gender inclusivity in its language.</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
         <is>
           <t>1. "ensure BIPOC communities are educated and trained on the prevention, protection, and protocols relating to missing BIPOC women and girls as it relates to social media;"
 2. "create a state-wide awareness campaign."</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>The legislation establishes a task force that includes members representative of communities experiencing the crisis, indicating an intention to involve those directly impacted, such as MMIP survivors and their relatives. Additionally, it emphasizes the importance of public input through hearings and written submissions, which provides avenues for survivors and their families to voice their experiences and perspectives. Moreover, the reference to the Sovereign Bodies Institute, an indigenous-led organization that focuses on missing and murdered Indigenous people, further supports the conclusion that the legislation seeks to incorporate input from these communities</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>Somewhat</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>The legislation establishes a task force that includes members representative of communities experiencing the crisis, which suggests an intention to include individuals who may have been directly impacted, such as MMIP survivors and their relatives. Additionally, it mandates public hearings and the acceptance of written input, indicating a mechanism for community engagement. However, while Indigenous politicians are sponsoring the legislation, the specifics of their roles or direct representation of Indigenous communities within the task force are not clearly detailed, leading to an assessment of "somewhat" in terms of inclusive input.</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>The legislation establishes a task force specifically designed to address the issues faced by missing women and girls, particularly those who are Black, Indigenous, and People of Color (BIPOC). It mandates that members of the task force be representative of the communities affected, including directly impacted individuals, which suggests inclusion of MMIP survivors and their relatives. Additionally, the task force is required to seek public input through hearings and written submissions, further indicating an effort to incorporate the perspectives of those directly affected by the crisis</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>The legislation explicitly states that the task force shall include members representing the communities experiencing the crisis, including directly impacted individuals. It also mandates public input through hearings and written submissions from the public across various regions of the state. This indicates a deliberate effort to include the voices of MMIP survivors, their relatives, and Indigenous communities in the policymaking process.</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
         <is>
           <t>Sen Lea Webb (D) - District SD-052, Sen Cordell Cleare (D) - District SD-030, Sen Leroy Comrie (D) - District SD-014, Sen Jeremy Cooney (D) - District SD-056, Sen Nathalia Fernandez (D) - District SD-034, Sen Brad Hoylman-Sigal (D) - District SD-047, Sen Timothy Kennedy (D) - District SD-063, Sen Monica Martinez (D) - District SD-004, Sen Jessica Ramos (D) - District SD-013, Sen Julia Salazar (D) - District SD-018</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr">
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr">
         <is>
           <t>2023-2024 Regular Session</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AA3" t="inlineStr">
         <is>
           <t>Taskforce, Data Collection, MMIP Relatives</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AB3" t="inlineStr">
         <is>
           <t>2023-12-21</t>
         </is>

</xml_diff>

<commit_message>
Improved Indigenous sponsors formatting
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB3"/>
+  <dimension ref="A1:AB2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -573,17 +573,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>AK</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Establishes a task force on missing women and girls who are black, indigenous and people of color (BIPOC) to develop policy changes that will work to address the lack of care and concern for missing and murdered BIPOC women and girls with New York state governmental agencies.</t>
+          <t>U.S. Attorney Tucker Issues Savanna’s Act Guidelines for Alaska</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>S04266</t>
+          <t>DOJ</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -598,46 +598,43 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Senate</t>
+          <t>Department of Justice</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2023-12-21 - S: APPROVAL MEMO.58</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>https://legiscan.com/NY/bill/S04266/2023</t>
-        </is>
-      </c>
+          <t>August 30, 2022 - For Immediate Release, U.S. Attorney's Office, District of Alaska</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://legiscan.com/NY/bill/S04266/2023</t>
+          <t>https://www.justice.gov/usao-ak/pr/us-attorney-tucker-issues-savanna-s-act-guidelines-alaska</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>The legislation establishes a task force in New York focused on addressing the crisis of missing women and girls who are Black, Indigenous, and People of Color (BIPOC). This task force will consist of various state officials and representatives from affected communities, aiming to develop policy changes, raise public awareness, and improve data collection regarding missing BIPOC individuals. It seeks to enhance cultural competency among first responders and recommend preventive measures to ensure the safety of these vulnerable populations. The task force is required to hold public hearings and submit a report with findings and recommendations two years after its formation. The act will take effect 60 days after becoming law and will expire three years later.</t>
+          <t>The U.S. Attorney's Office for the District of Alaska announced the completion of the Savanna’s Act Guidelines, aimed at improving responses to missing and murdered Indigenous persons (MMIP) through enhanced coordination among law enforcement agencies. Co-sponsored by Senator Lisa Murkowski, the initiative focuses on facilitating communication and implementing best practices for addressing these critical issues faced by Alaska Natives and American Indians. The guidelines include provisions for data collection and culturally appropriate victim services, ensuring ongoing collaboration with Alaska Tribes and relevant stakeholders. U.S. Attorney S. Lane Tucker emphasized the importance of these guidelines in providing justice and answers for victims and their families. This effort is part of a broader commitment to combat violence against Indigenous communities and improve law enforcement responses.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Establishes a dedicated task force focused on the crisis of missing women and girls who are Black, Indigenous, and People of Color (BIPOC), facilitating targeted attention to this urgent issue.  
-2. Aims to develop policy changes that enhance the care and concern for missing and murdered BIPOC women and girls, thus improving the response from state governmental agencies.  
-3. Requires public hearings and the collection of community input, ensuring that the voices of affected individuals, including MMIP survivors and their relatives, are considered in the decision-making process.  
-4. Promotes awareness and education within BIPOC communities regarding prevention and protection strategies, which can help mitigate future incidents.  
-5. Develops mechanisms for data collection, allowing for better tracking and analysis of cases involving missing BIPOC individuals, which can drive informed policymaking and resource allocation.  </t>
+          <t>1. Enhances coordination among law enforcement agencies to improve responses to missing and murdered Indigenous persons (MMIP).  
+2. Utilizes gender inclusive language, addressing the crisis as one affecting all Indigenous individuals rather than just women.  
+3. Incorporates mechanisms for data collection and culturally appropriate victim services, fostering better understanding and support for affected communities.  
+4. Provides ongoing opportunities for input and recommendations from Alaska Tribes, ensuring the inclusion of Indigenous perspectives in decision-making.  
+5. Aims to strengthen partnerships and improve the justice system’s responsiveness to the needs of victims and their families.  
+6. Involves Indigenous organizations that support MMIP survivors, enhancing community engagement and resource availability.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The legislation's focus primarily on women and girls may overlook the broader issue of missing Indigenous people, failing to employ gender-neutral language consistently.  
-2. There are no specific Indigenous organizations mentioned in the legislation, which may limit direct representation and input from those who are most affected by the crisis.  
-3. The task force is set to expire three years after its formation, which may limit the long-term impact and sustainability of the proposed measures.  
-4. While public hearings are required, the effectiveness of community engagement may vary based on participation and outreach efforts, potentially resulting in inadequate representation of all affected voices.  
-5. The lack of explicit details regarding the direct involvement of MMIP survivors or Indigenous politicians in the formulation of the legislation may hinder the authenticity and relevance of the proposed solutions.  </t>
+          <t>1. The legislation does not specify explicit mechanisms for ongoing involvement or feedback from MMIP survivors and their families, which may limit their influence on future decisions.  
+2. While there is substantial consultation mentioned, the effectiveness of that consultation in producing actionable results is not clearly defined.  
+3. The focus on data collection and analysis may face challenges related to privacy concerns and the safe handling of sensitive information regarding victims and Indigenous communities.  
+4. There may be potential gaps in funding or resources to implement the guidelines effectively, which could hinder their overall impact.  
+5. The guidelines rely on collaboration with various agencies, which could lead to inconsistencies in enforcement and application across different jurisdictions.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -647,19 +644,18 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>1. The task force shall submit a report containing its findings and recommendations to various legislative leaders (Section 2.e).
-2. The task force shall seek public input by holding public hearings in each region of the state (Section 2.d).
-3. The task force shall develop a strategy to collect statistics, demographics, surveys, oral histories, and data analysis (Section 2.c.iv).</t>
+          <t>1. Guidance on the collection, reporting and analysis of MMIP data
+2. Ongoing opportunities for input and recommendations</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>The legislation primarily focuses on women and girls, specifically highlighting issues related to missing Black and Indigenous women and girls, which suggests a gender-specific approach. While it does include the term "people of color," the language does not broadly address issues concerning missing Indigenous people or use gender-neutral terms consistently. Consequently, the legislation does not fully encompass gender-inclusive language throughout its provisions.</t>
+          <t>The legislation uses gender inclusive language by referring to the crisis as one involving missing and murdered Indigenous persons rather than solely focusing on women. This broader terminology acknowledges the impact of violence on all Indigenous individuals, regardless of gender. Additionally, the text emphasizes a collaborative approach to improving responses to these cases, which includes both male and female victims.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -669,194 +665,55 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1. "ensure BIPOC communities are educated and trained on the prevention, protection, and protocols relating to missing BIPOC women and girls as it relates to social media" (Section 2.c.iii).
-2. "create a state-wide awareness campaign" (Section 2.c.vii).</t>
+          <t xml:space="preserve">1. “These guidelines will help us to further strengthen our partnerships and push ourselves to constantly improve our response to bring answers and justice for the victims and families.”  
+2. “Savanna’s Act aims to improve the government’s response to the crisis of missing and murdered Indigenous persons through increased coordination and the development of best practices.”  
+3. “It also provides guidance on the collection, reporting and analysis of MMIP data; offers resource information for Tribal governments; and provides best practices for culturally appropriate victim services and for returning a loved one home.”   
+4. “Ongoing opportunities for input and recommendations.”  </t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>The legislation highlights that it was developed following "hundreds of hours of consultation with Alaska Tribes, tribal agencies, victim service providers, and federal, state, local, and tribal law enforcement," indicating a collaborative approach that likely includes input from various stakeholders. Additionally, it mentions "ongoing opportunities for input and recommendations," suggesting that the voices and perspectives of MMIP survivors and their families are indeed considered in the process. Furthermore, the involvement of Indigenous organizations such as the Alaska Native Women’s Resource Center, which supports victims of violence against Indigenous women, further reinforces that the legislation accounts for feedback and input from those directly affected, including survivors and their relatives</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
           <t>Somewhat</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>The legislation indicates that the task force will be composed of individuals who reflect the diversity of New York State and are representative of the communities experiencing the crisis, which suggests an intent to include voices from impacted groups, including MMIP survivors and their relatives. Furthermore, the task force is required to seek public input through regional hearings and written submissions, which provides a platform for these individuals to share their experiences and perspectives. However, specific organizations directly representing MMIP survivors are not explicitly mentioned in the text, leading to a "Somewhat" designation regarding the level of input from these groups</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>Somewhat</t>
-        </is>
-      </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>The legislation establishes a task force that is required to seek public input by holding public hearings in each region of the state and accepting written submissions, indicating some level of engagement with affected communities, including MMIP survivors and relatives. Additionally, the language specifies that task force members should be representative of the communities experiencing this crisis, suggesting an effort to include voices from Indigenous communities. However, the specific details regarding the direct involvement of MMIP survivors or Indigenous politicians in the formulation of the legislation are not explicitly outlined, resulting in a "Somewhat" designation for input.</t>
+          <t>The legislation indicates that there has been substantial consultation with Alaska Tribes and various stakeholders, including victim service providers and law enforcement, which suggests some level of input from Indigenous communities. It also highlights ongoing opportunities for input and recommendations, implying that the perspectives of MMIP survivors and their families are considered in the development of strategies. However, it does not specify explicit mechanisms for ongoing involvement or feedback from these groups, leading to a determination of "somewhat" regarding their level of input.</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>Sen Lea Webb (D) - District SD-052, Sen Cordell Cleare (D) - District SD-030, Sen Leroy Comrie (D) - District SD-014, Sen Jeremy Cooney (D) - District SD-056, Sen Nathalia Fernandez (D) - District SD-034, Sen Brad Hoylman-Sigal (D) - District SD-047, Sen Timothy Kennedy (D) - District SD-063, Sen Monica Martinez (D) - District SD-004, Sen Jessica Ramos (D) - District SD-013, Sen Julia Salazar (D) - District SD-018</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr"/>
+          <t>S. Lane Tucker [U.S. Attorney, District of Alaska], Lisa Murkowski [U.S. Senator, Alaska], Rob Heun [U.S. Marshal, District of Alaska], Ingrid Cumberlidge [MMIP Program Coordinator - Aleut, Tlingit], Ahtna Region, Orutsararmiut Native Council, Sun’aq Tribe of Kodiak, Arctic Slope Native Association, Central Council of Tlingit and Haida Indian Tribes of Alaska, Native Village of Kotzebue, Maniilaq Association, Native Village of White Mountain Village, Curyung Tribal Council of Dillingham, Native Village of Unalakleet, Koyukuk Native Village.</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Ingrid Cumberlidge [MMIP Program Coordinator - Aleut, Tlingit]</t>
+        </is>
+      </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>2023-2024 Regular Session</t>
+          <t>Biden Administration, 2020-2024</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>Taskforce, Data Collection, MMIP Relatives</t>
+          <t>Taskforce, US Law Enforcement, Tribal Law Enforcement, Data Collection, MMIP Relatives</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>2023-12-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Establishes a task force on missing women and girls who are black, indigenous and people of color (BIPOC) to develop policy changes that will work to address the lack of care and concern for missing and murdered BIPOC women and girls with New York state governmental agencies.</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>S04266</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Passed</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Senate</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2023-12-21 - S: APPROVAL MEMO.58</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>https://legiscan.com/NY/bill/S04266/2023</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>https://legiscan.com/NY/bill/S04266/2023</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>The legislation establishes a task force in New York dedicated to addressing the issue of missing women and girls who are Black, Indigenous, and People of Color (BIPOC). It aims to develop policy changes, improve data collection, and raise public awareness about the circumstances surrounding missing BIPOC women and girls. The task force will include representatives from relevant state agencies and community members and will seek public input through hearings. It is required to submit a report with findings and recommendations within two years. The act will take effect 60 days after becoming law and will expire three years later.</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>1. Establishes a task force focused on addressing the issue of missing BIPOC women and girls, promoting targeted policy changes.
-2. Facilitates improved data collection and analysis to better understand and address the crisis of missing individuals.
-3. Includes provisions for public input through hearings, allowing community members, including MMIP survivors and their relatives, to voice their concerns and experiences.
-4. Creates educational and awareness programs aimed at preventing the disappearance of BIPOC women and girls.
-5. Ensures representation from affected communities within the task force, fostering inclusivity in policy development and decision-making.</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>1. The legislation primarily focuses on missing women and girls, which may exclude broader representation of missing Indigenous individuals beyond this demographic.
-2. The language used in the legislation does not consistently employ gender-neutral terms, potentially limiting inclusivity for non-binary or gender-diverse individuals experiencing similar issues.
-3. The act has a limited duration of three years before it expires, which may hinder long-term efforts and sustainability in addressing the crisis.
-4. There is no specific mention of Indigenous organizations or partnerships that could provide cultural context and support to the task force’s initiatives.
-5. The effectiveness of the task force’s recommendations relies heavily on the cooperation and engagement of various state agencies, which may vary and impact implementation.</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>1. "On or before two years after the effective date of this act, the task force shall submit to the temporary president of the senate, the speaker of the assembly, the minority leader of the senate and the minority leader of the assembly a report containing its findings and recommendations."
-2. "In carrying out the duties of the task force, such task force shall seek public input by holding public hearings in each region of the state and accepting public input in writing."
-3. "develop a strategy to collect statistics, demographics, surveys, oral histories, and data analysis."</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>The legislation primarily focuses on missing women and girls, explicitly naming Black, Indigenous, and People of Color (BIPOC) women and girls throughout. While it addresses the significant issue of missing Indigenous individuals, it does not consistently use gender-neutral language or include a broader representation of missing Indigenous people beyond women and girls. As a result, it does not fully encompass gender inclusivity in its language.</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>1. "ensure BIPOC communities are educated and trained on the prevention, protection, and protocols relating to missing BIPOC women and girls as it relates to social media;"
-2. "create a state-wide awareness campaign."</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>The legislation establishes a task force specifically designed to address the issues faced by missing women and girls, particularly those who are Black, Indigenous, and People of Color (BIPOC). It mandates that members of the task force be representative of the communities affected, including directly impacted individuals, which suggests inclusion of MMIP survivors and their relatives. Additionally, the task force is required to seek public input through hearings and written submissions, further indicating an effort to incorporate the perspectives of those directly affected by the crisis</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>The legislation explicitly states that the task force shall include members representing the communities experiencing the crisis, including directly impacted individuals. It also mandates public input through hearings and written submissions from the public across various regions of the state. This indicates a deliberate effort to include the voices of MMIP survivors, their relatives, and Indigenous communities in the policymaking process.</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>Sen Lea Webb (D) - District SD-052, Sen Cordell Cleare (D) - District SD-030, Sen Leroy Comrie (D) - District SD-014, Sen Jeremy Cooney (D) - District SD-056, Sen Nathalia Fernandez (D) - District SD-034, Sen Brad Hoylman-Sigal (D) - District SD-047, Sen Timothy Kennedy (D) - District SD-063, Sen Monica Martinez (D) - District SD-004, Sen Jessica Ramos (D) - District SD-013, Sen Julia Salazar (D) - District SD-018</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>2023-2024 Regular Session</t>
-        </is>
-      </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>Taskforce, Data Collection, MMIP Relatives</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>2023-12-21</t>
+          <t>2022-08-30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improved sponsors formatting II
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -581,11 +581,7 @@
           <t>U.S. Attorney Tucker Issues Savanna’s Act Guidelines for Alaska</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>DOJ</t>
-        </is>
-      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>Passed</t>
@@ -603,7 +599,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>August 30, 2022 - For Immediate Release, U.S. Attorney's Office, District of Alaska</t>
+          <t>Tuesday, August 30, 2022 - For Immediate Release, U.S. Attorney's Office, District of Alaska</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -615,26 +611,27 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>The U.S. Attorney's Office for the District of Alaska announced the completion of the Savanna’s Act Guidelines, aimed at improving responses to missing and murdered Indigenous persons (MMIP) through enhanced coordination among law enforcement agencies. Co-sponsored by Senator Lisa Murkowski, the initiative focuses on facilitating communication and implementing best practices for addressing these critical issues faced by Alaska Natives and American Indians. The guidelines include provisions for data collection and culturally appropriate victim services, ensuring ongoing collaboration with Alaska Tribes and relevant stakeholders. U.S. Attorney S. Lane Tucker emphasized the importance of these guidelines in providing justice and answers for victims and their families. This effort is part of a broader commitment to combat violence against Indigenous communities and improve law enforcement responses.</t>
+          <t>The U.S. Attorney's Office for the District of Alaska has released the Savanna’s Act Guidelines aimed at addressing the crisis of missing and murdered Indigenous persons (MMIP) through improved coordination among law enforcement and victim service providers. This initiative, which followed extensive consultation with Alaska Tribes and various agencies, emphasizes the need for culturally appropriate victim services and better data collection related to MMIP cases. U.S. Attorney S. Lane Tucker highlighted the importance of tackling the disproportionately high rates of violence experienced by Alaska Natives and American Indians. The guidelines are designed to enhance communication and ensure ongoing input from tribal communities. Overall, the initiative seeks to strengthen partnerships and improve responses to MMIP situations across Alaska.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1. Enhances coordination among law enforcement agencies to improve responses to missing and murdered Indigenous persons (MMIP).  
-2. Utilizes gender inclusive language, addressing the crisis as one affecting all Indigenous individuals rather than just women.  
-3. Incorporates mechanisms for data collection and culturally appropriate victim services, fostering better understanding and support for affected communities.  
-4. Provides ongoing opportunities for input and recommendations from Alaska Tribes, ensuring the inclusion of Indigenous perspectives in decision-making.  
-5. Aims to strengthen partnerships and improve the justice system’s responsiveness to the needs of victims and their families.  
-6. Involves Indigenous organizations that support MMIP survivors, enhancing community engagement and resource availability.</t>
+          <t>1. Improved coordination among law enforcement and victim service providers to address the crisis of missing and murdered Indigenous persons (MMIP).  
+2. Enhanced culturally appropriate victim services and better data collection related to MMIP cases.  
+3. Ongoing opportunities for input and recommendations from tribal communities.  
+4. Use of gender-inclusive language that acknowledges the experiences of all genders within Indigenous communities.  
+5. Strengthened partnerships aimed at increasing the effectiveness of responses to MMIP situations across Alaska.  
+6. Extensive consultation with Alaska Tribes, ensuring that Indigenous voices and experiences are central to the initiative's development.  
+7. Support from organizations that advocate for Indigenous women and MMIP survivors.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>1. The legislation does not specify explicit mechanisms for ongoing involvement or feedback from MMIP survivors and their families, which may limit their influence on future decisions.  
-2. While there is substantial consultation mentioned, the effectiveness of that consultation in producing actionable results is not clearly defined.  
-3. The focus on data collection and analysis may face challenges related to privacy concerns and the safe handling of sensitive information regarding victims and Indigenous communities.  
-4. There may be potential gaps in funding or resources to implement the guidelines effectively, which could hinder their overall impact.  
-5. The guidelines rely on collaboration with various agencies, which could lead to inconsistencies in enforcement and application across different jurisdictions.</t>
+          <t>1. The implementation of the guidelines may face challenges due to varying levels of cooperation and resources among local, state, and federal law enforcement agencies.  
+2. There is a reliance on ongoing input and recommendations, which may lead to inconsistencies in application if feedback mechanisms are not effectively managed.  
+3. While the guidelines promote cultural sensitivity, there may be difficulties in uniformly applying these practices across diverse tribal communities.  
+4. The focus on data collection may raise concerns about privacy and the responsiveness of agencies in protecting sensitive information related to survivors and their families.  
+5. There is potential for limited funding and resources to adequately support the extensive training and implementation required by the guidelines.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -644,8 +641,10 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>1. Guidance on the collection, reporting and analysis of MMIP data
-2. Ongoing opportunities for input and recommendations</t>
+          <t xml:space="preserve">1. Ongoing opportunities for input and recommendations.  
+2. Guidance on the collection, reporting and analysis of MMIP data.  
+3. Consultation with Alaska Tribes and tribal agencies.  
+4. Development of best practices for culturally appropriate victim services.  </t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -655,7 +654,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>The legislation uses gender inclusive language by referring to the crisis as one involving missing and murdered Indigenous persons rather than solely focusing on women. This broader terminology acknowledges the impact of violence on all Indigenous individuals, regardless of gender. Additionally, the text emphasizes a collaborative approach to improving responses to these cases, which includes both male and female victims.</t>
+          <t>The legislation uses gender-inclusive language by framing the crisis as one affecting "missing and murdered Indigenous persons" rather than solely focusing on women. This broader terminology recognizes that individuals of all genders can be victims of violence and supports a more comprehensive approach to addressing the issue. By emphasizing "persons," the language aligns with a commitment to inclusivity and acknowledges the varied experiences within Indigenous communities.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -665,10 +664,9 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. “These guidelines will help us to further strengthen our partnerships and push ourselves to constantly improve our response to bring answers and justice for the victims and families.”  
-2. “Savanna’s Act aims to improve the government’s response to the crisis of missing and murdered Indigenous persons through increased coordination and the development of best practices.”  
-3. “It also provides guidance on the collection, reporting and analysis of MMIP data; offers resource information for Tribal governments; and provides best practices for culturally appropriate victim services and for returning a loved one home.”   
-4. “Ongoing opportunities for input and recommendations.”  </t>
+          <t>1. "These guidelines will help us to further strengthen our partnerships and push ourselves to constantly improve our response to bring answers and justice for the victims and families."
+2. "Savanna’s Act... aims to improve the government’s response to the crisis of missing and murdered Indigenous persons through increased coordination and the development of best practices."
+3. "These guidelines are evergreen with ongoing opportunities for input and recommendations."</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -678,27 +676,27 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>The legislation highlights that it was developed following "hundreds of hours of consultation with Alaska Tribes, tribal agencies, victim service providers, and federal, state, local, and tribal law enforcement," indicating a collaborative approach that likely includes input from various stakeholders. Additionally, it mentions "ongoing opportunities for input and recommendations," suggesting that the voices and perspectives of MMIP survivors and their families are indeed considered in the process. Furthermore, the involvement of Indigenous organizations such as the Alaska Native Women’s Resource Center, which supports victims of violence against Indigenous women, further reinforces that the legislation accounts for feedback and input from those directly affected, including survivors and their relatives</t>
+          <t>The legislation specifies that it was developed following "hundreds of hours of consultation with Alaska Tribes and tribal agencies," which implies that there was an effort to gather input from various stakeholders, potentially including MMIP survivors and their relatives. Additionally, the mention of organizations such as the Alaska Native Women’s Resource Center, which is known for advocating on behalf of Indigenous women, suggests a focus on supporting MMIP survivors. These elements collectively indicate that the legislation incorporates input from affected individuals and communities in its development</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Somewhat</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>The legislation indicates that there has been substantial consultation with Alaska Tribes and various stakeholders, including victim service providers and law enforcement, which suggests some level of input from Indigenous communities. It also highlights ongoing opportunities for input and recommendations, implying that the perspectives of MMIP survivors and their families are considered in the development of strategies. However, it does not specify explicit mechanisms for ongoing involvement or feedback from these groups, leading to a determination of "somewhat" regarding their level of input.</t>
+          <t>The legislation emphasizes extensive consultation with Alaska Tribes and tribal agencies, which indicates an effort to incorporate input from Indigenous communities, including MMIP survivors and their families. The guidelines are described as being developed through "hundreds of hours of consultation," suggesting proactive engagement with affected parties. Furthermore, the involvement of Ingrid Cumberlidge, an Indigenous politician and MMIP Coordinator, highlights the commitment to centering Indigenous voices in addressing the crisis.</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>S. Lane Tucker [U.S. Attorney, District of Alaska], Lisa Murkowski [U.S. Senator, Alaska], Rob Heun [U.S. Marshal, District of Alaska], Ingrid Cumberlidge [MMIP Program Coordinator - Aleut, Tlingit], Ahtna Region, Orutsararmiut Native Council, Sun’aq Tribe of Kodiak, Arctic Slope Native Association, Central Council of Tlingit and Haida Indian Tribes of Alaska, Native Village of Kotzebue, Maniilaq Association, Native Village of White Mountain Village, Curyung Tribal Council of Dillingham, Native Village of Unalakleet, Koyukuk Native Village.</t>
+          <t>S. Lane Tucker (District of Alaska) - U.S. Attorney, Lisa Murkowski - U.S. Senator (R), Ingrid Cumberlidge (Aleut, Tlingit) - MMIP Coordinator (District of Alaska), Rob Heun - U.S. Marshal (District of Alaska), Tribal representatives from Ahtna Region, Orutsararmiut Native Council, Sun’aq Tribe of Kodiak, Arctic Slope Native Association, Central Council of Tlingit and Haida Indian Tribes of Alaska, Native Village of Kotzebue, Maniilaq Association, Native Village of White Mountain Village, Advocates from Victims for Justice, Alaska Native Women’s Resource Center.</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Ingrid Cumberlidge [MMIP Program Coordinator - Aleut, Tlingit]</t>
+          <t>Ingrid Cumberlidge (Aleut, Tlingit) - MMIP Coordinator (District of Alaska)</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">

</xml_diff>

<commit_message>
API compatibility with Federal Register
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -573,17 +573,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>National</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Proclamation Recognizing May 5, 2021 as Missing and Murdered Indigenous Women’s Day in North Carolina.</t>
+          <t>National Native American Heritage Month, 2024</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>P12345</t>
+          <t>P10853</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -603,37 +603,37 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>May 5, 2021 - Proclamation signed and Enacted</t>
+          <t>October 31, 2024 - Proclamation signed and Enacted</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://governor.nc.gov/documents/files/governor-proclaims-day-awareness-missing-and-murdered-indigenous-women-2021/open</t>
+          <t>https://www.federalregister.gov/documents/2024/11/05/2024-25808/national-native-american-heritage-month-2024</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>The document is a proclamation recognizing May 5, 2021, as Missing and Murdered Indigenous Women’s Day in North Carolina. It aims to bring awareness to the crisis of violence against Indigenous women and girls, particularly focusing on the disproportionate rates of missing and murdered cases within Indigenous communities. The proclamation acknowledges the cultural and societal impacts of this issue and calls for community action and support. It encourages North Carolinians to recognize and address the systemic causes of this violence. The initiative emphasizes the importance of amplifying the voices of Indigenous people and ensuring justice for victims and their families.</t>
+          <t>The document is Proclamation 10853, declaring November 2024 as National Native American Heritage Month. It honors the history, cultures, and contributions of Native peoples, emphasizing the importance of respecting Tribal sovereignty and partnerships between the U.S. government and Tribal Nations. The proclamation acknowledges the past injustices faced by Indigenous peoples, including the impacts of Federal Indian Boarding Schools. It also highlights the Biden Administration's commitment to improving the socioeconomic conditions of Native communities through significant investments and policy initiatives. The proclamation calls for all Americans to observe the month with appropriate programs and emphasizes healing and moving forward together.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Raises awareness about the crisis of Missing and Murdered Indigenous Women and the broader issue of violence affecting Indigenous communities.  
-2. Acknowledges the cultural and societal impacts of violence against Indigenous people, promoting community action and support.  
-3. Emphasizes the importance of amplifying the voices of Indigenous populations and advocating for justice for victims and their families.  
-4. Encourages North Carolinians to recognize and address systemic causes of violence, fostering a more inclusive understanding of the issue.  
-5. Establishes May 5 as a dedicated day for recognition, promoting ongoing dialogue and awareness around this critical issue.  </t>
+          <t>1. The proclamation honors and recognizes the history, cultures, and contributions of Native peoples, fostering greater appreciation and awareness among the general public.  
+2. It emphasizes the importance of respecting Tribal sovereignty and partnerships between the U.S. government and Tribal Nations, promoting collaborative efforts for mutual benefit.  
+3. The legislation highlights significant investments and policy initiatives aimed at improving the socioeconomic conditions of Native communities, which can lead to enhanced resources and support.  
+4. It promotes gender-inclusive language, acknowledging the diverse experiences of Indigenous peoples, particularly in relation to the epidemic of missing and murdered Indigenous peoples.  
+5. The proclamation serves as a call to action for all Americans to celebrate and engage with Native communities, encouraging healing and a collective move towards a better future.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Lacks specific mechanisms for evaluation, which may hinder accountability and the ability to measure the effectiveness of the initiative.  
-2. Does not include detailed references to community involvement or consultation with MMIP survivors and their relatives, limiting the representation of their voices.  
-3. Focuses primarily on raising awareness rather than implementing actionable prevention strategies or support systems.  
-4. Fails to establish formal channels for Indigenous organizations to contribute to the legislative process, which could enhance community engagement.  
-5. While acknowledging the broader issue of violence, it still primarily centers the narrative around Indigenous women, potentially overlooking the experiences of all Indigenous individuals affected by violence.  </t>
+          <t xml:space="preserve">1. The legislation lacks specific mechanisms for evaluation, making it difficult to assess the effectiveness and outcomes of its initiatives.  
+2. There is no direct input or consultation from MMIP survivors or their families, which may limit the relevance and responsiveness of policy measures to their experiences and needs.  
+3. While it emphasizes partnerships, the level of centering Indigenous voices is only somewhat, indicating that Indigenous communities may not have been fully engaged in the legislative process.  
+4. The proclamation does not detail specific programs or activities that will be implemented during National Native American Heritage Month, leaving the effectiveness of the observance open to interpretation.  
+5. Although the document highlights the crisis of missing and murdered Indigenous peoples, it may not provide sufficient actionable strategies or resources specifically targeting this issue.  </t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -643,7 +643,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>The document does not mention any specific mechanisms for evaluation such as a final report, community consultation, tribal consultation, a Tribal Crisis Response Plan (TCRP), monitoring, or data collection. Therefore, there are no items to list.</t>
+          <t>1. No specific mechanisms for evaluation are mentioned in the legislation.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -653,7 +653,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>The legislation specifically recognizes the crisis of Missing and Murdered Indigenous Women, but it also emphasizes the broader issue of violence affecting Indigenous communities. By acknowledging the systemic causes of violence and calling for action to support all Indigenous people, it implies a recognition beyond just women. This approach aligns with efforts to raise awareness for the entire Indigenous population impacted by the crisis.</t>
+          <t>Yes, the legislation uses gender-inclusive language by referring to the "epidemic of missing and murdered Indigenous peoples," which encompasses individuals of all genders. This broader terminology acknowledges the crisis affecting not only women but also men and non-binary individuals within Indigenous communities. Additionally, the proclamation emphasizes partnerships and shared concerns across all Native peoples, reinforcing an inclusive approach.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -663,48 +663,54 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
+          <t>1. "My Administration is also working to ensure that Native communities are safe and secure and have the resources they need to thrive."
+2. "I signed an Executive Order that improves the Federal response to the epidemic of missing and murdered Indigenous peoples."
+3. "We included historic provisions to reaffirm Tribal sovereignty and expand Tribal jurisdiction in cases where outside perpetrators harm members of their Nation."</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Somewhat</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>The legislation does not provide specific instances of input from MMIP survivors, their relatives, or Indigenous communities. It primarily focuses on raising awareness about the issue but lacks detailed references to community involvement or consultation in the legislative process. As a result, there is no evidence to indicate any formal input from the identified groups.</t>
+          <t>The proclamation emphasizes a commitment to respecting Tribal sovereignty and working in partnership with Tribal Nations, suggesting some level of collaboration with Indigenous communities. It mentions historic provisions in the reauthorization of the Violence Against Women Act, which aim to expand Tribal jurisdiction, indicating responsiveness to the needs expressed by those affected by the MMIP crisis. However, it lacks specific references to direct input or consultation from MMIP survivors or their families, limiting the indication of their involvement in shaping the legislation.</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>The document does not specify individual tribal members, representatives, organizations, or any supporting officials.</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr"/>
+          <t>Deb Haaland (Laguna Pueblo) - 54th United States Secretary of the Interior, 2021–present, Joseph R. Biden Jr. - President of the United States</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Deb Haaland (Laguna Pueblo) - 54th United States Secretary of the Interior, 2021–present</t>
+        </is>
+      </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>Biden Administration, 2020 - 2024</t>
+          <t>Biden Administration, 2020-2024</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>Day of Recognition</t>
+          <t>Day of Recognition, US Law Enforcement, Tribal Law Enforcement</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>2021-05-05</t>
+          <t>2024-10-31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
More robust search and match for Indigenous sponsors
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -615,25 +615,25 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>The document is Proclamation 10853, declaring November 2024 as National Native American Heritage Month. It honors the history, cultures, and contributions of Native peoples, emphasizing the importance of respecting Tribal sovereignty and partnerships between the U.S. government and Tribal Nations. The proclamation acknowledges the past injustices faced by Indigenous peoples, including the impacts of Federal Indian Boarding Schools. It also highlights the Biden Administration's commitment to improving the socioeconomic conditions of Native communities through significant investments and policy initiatives. The proclamation calls for all Americans to observe the month with appropriate programs and emphasizes healing and moving forward together.</t>
+          <t>The document is Proclamation 10853, declaring November 2024 as National Native American Heritage Month. It honors the history, cultures, and contributions of Native peoples and emphasizes the importance of respecting Tribal sovereignty and self-determination. The proclamation reflects on the past injustices faced by Indigenous communities, including the impacts of Federal Indian Boarding Schools. It acknowledges the resilience of Native communities and highlights the Biden Administration's commitment to investing in Tribal Nations and addressing issues such as missing and murdered Indigenous peoples. The proclamation encourages all Americans to observe the month with appropriate programs and activities.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1. The proclamation honors and recognizes the history, cultures, and contributions of Native peoples, fostering greater appreciation and awareness among the general public.  
-2. It emphasizes the importance of respecting Tribal sovereignty and partnerships between the U.S. government and Tribal Nations, promoting collaborative efforts for mutual benefit.  
-3. The legislation highlights significant investments and policy initiatives aimed at improving the socioeconomic conditions of Native communities, which can lead to enhanced resources and support.  
-4. It promotes gender-inclusive language, acknowledging the diverse experiences of Indigenous peoples, particularly in relation to the epidemic of missing and murdered Indigenous peoples.  
-5. The proclamation serves as a call to action for all Americans to celebrate and engage with Native communities, encouraging healing and a collective move towards a better future.</t>
+          <t xml:space="preserve">1. The proclamation honors the history, cultures, and contributions of Native peoples, increasing awareness and appreciation among the general public.  
+2. It emphasizes the importance of respecting Tribal sovereignty and self-determination, promoting a stronger partnership between the federal government and Tribal Nations.  
+3. The legislation reflects a commitment to invest in Tribal Nations and address critical issues such as missing and murdered Indigenous peoples, which can lead to improved support and resources for affected communities.  
+4. By encouraging all Americans to observe National Native American Heritage Month with appropriate programs and activities, it fosters community engagement and education about Indigenous issues.  
+5. The gender-inclusive language acknowledges the experiences of both men and women, promoting a more comprehensive understanding of the challenges faced by Indigenous communities.  </t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The legislation lacks specific mechanisms for evaluation, making it difficult to assess the effectiveness and outcomes of its initiatives.  
-2. There is no direct input or consultation from MMIP survivors or their families, which may limit the relevance and responsiveness of policy measures to their experiences and needs.  
-3. While it emphasizes partnerships, the level of centering Indigenous voices is only somewhat, indicating that Indigenous communities may not have been fully engaged in the legislative process.  
-4. The proclamation does not detail specific programs or activities that will be implemented during National Native American Heritage Month, leaving the effectiveness of the observance open to interpretation.  
-5. Although the document highlights the crisis of missing and murdered Indigenous peoples, it may not provide sufficient actionable strategies or resources specifically targeting this issue.  </t>
+          <t xml:space="preserve">1. The legislation does not include explicit mechanisms for evaluation, making it difficult to assess the effectiveness of its initiatives and commitments.  
+2. There is a lack of direct input or consultation from MMIP survivors or their relatives, which may limit the relevance and responsiveness of the efforts to the needs of affected communities.  
+3. While it acknowledges Indigenous communities, the absence of detailed examples of community engagement suggests that voices from these communities may not be fully centered in the legislative process.  
+4. The reliance on partnerships with Tribal Nations without specifying how these partnerships will be structured may lead to inconsistencies in the implementation of initiatives across different regions.  
+5. The focus on broad awareness and recognition may not translate into tangible actions or changes for Indigenous communities facing ongoing challenges.  </t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -643,7 +643,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>1. No specific mechanisms for evaluation are mentioned in the legislation.</t>
+          <t>1. No mechanisms for evaluation are explicitly mentioned in the legislation.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -653,7 +653,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Yes, the legislation uses gender-inclusive language by referring to the "epidemic of missing and murdered Indigenous peoples," which encompasses individuals of all genders. This broader terminology acknowledges the crisis affecting not only women but also men and non-binary individuals within Indigenous communities. Additionally, the proclamation emphasizes partnerships and shared concerns across all Native peoples, reinforcing an inclusive approach.</t>
+          <t>The legislation refers to the "epidemic of missing and murdered Indigenous peoples," which broadens the focus beyond just women to include all Indigenous individuals. This language shift promotes inclusivity and acknowledges the experiences of both men and women in these crises. Overall, it reflects a more comprehensive approach to addressing issues affecting Indigenous communities.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -665,7 +665,7 @@
         <is>
           <t>1. "My Administration is also working to ensure that Native communities are safe and secure and have the resources they need to thrive."
 2. "I signed an Executive Order that improves the Federal response to the epidemic of missing and murdered Indigenous peoples."
-3. "We included historic provisions to reaffirm Tribal sovereignty and expand Tribal jurisdiction in cases where outside perpetrators harm members of their Nation."</t>
+3. "When we reauthorized the Violence Against Women Act in 2022, we included historic provisions to reaffirm Tribal sovereignty and expand Tribal jurisdiction in cases where outside perpetrators harm members of their Nation."</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -685,12 +685,12 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>The proclamation emphasizes a commitment to respecting Tribal sovereignty and working in partnership with Tribal Nations, suggesting some level of collaboration with Indigenous communities. It mentions historic provisions in the reauthorization of the Violence Against Women Act, which aim to expand Tribal jurisdiction, indicating responsiveness to the needs expressed by those affected by the MMIP crisis. However, it lacks specific references to direct input or consultation from MMIP survivors or their families, limiting the indication of their involvement in shaping the legislation.</t>
+          <t>The legislation does not explicitly mention direct input from MMIP survivors or their relatives but emphasizes partnerships with Tribal Nations, which suggests a level of inclusion. Indigenous politicians, like Deb Haaland, are highlighted in their roles, indicating representation at high government levels, but specific community engagement is not detailed. Overall, the language reflects an acknowledgment of Indigenous communities while lacking concrete examples of their input in shaping the legislation.</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>Deb Haaland (Laguna Pueblo) - 54th United States Secretary of the Interior, 2021–present, Joseph R. Biden Jr. - President of the United States</t>
+          <t>Deb Haaland (Laguna Pueblo) - 54th United States Secretary of the Interior, 2021–present</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -705,7 +705,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>Day of Recognition, US Law Enforcement, Tribal Law Enforcement</t>
+          <t>Taskforce, Day of Recognition, US Law Enforcement, Tribal Law Enforcement, Data Collection</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">

</xml_diff>

<commit_message>
Added exponential backoff to try and catch GPT fetches
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AB3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -573,17 +573,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>National</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>National Native American Heritage Month, 2024</t>
+          <t>Justice Department Strengthens Efforts, Builds Partnerships to Address the Crisis of Missing or Murdered Indigenous Persons</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>P10853</t>
+          <t>DOJ24-570</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -598,52 +598,54 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Proclamation</t>
+          <t>Department of Justice</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>October 31, 2024 - Proclamation signed and Enacted</t>
+          <t>May 3, 2024 - Immediate release, U.S. Attorney's Office, Southern District of Mississippi</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://www.federalregister.gov/documents/2024/11/05/2024-25808/national-native-american-heritage-month-2024</t>
+          <t>https://www.justice.gov/usao-sdms/pr/justice-department-strengthens-efforts-builds-partnerships-address-crisis-missing-or</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>The document is Proclamation 10853, declaring November 2024 as National Native American Heritage Month. It honors the history, cultures, and contributions of Native peoples and emphasizes the importance of respecting Tribal sovereignty and self-determination. The proclamation reflects on the past injustices faced by Indigenous communities, including the impacts of Federal Indian Boarding Schools. It acknowledges the resilience of Native communities and highlights the Biden Administration's commitment to investing in Tribal Nations and addressing issues such as missing and murdered Indigenous peoples. The proclamation encourages all Americans to observe the month with appropriate programs and activities.</t>
+          <t>The Justice Department is enhancing its efforts to address the crisis of missing or murdered Indigenous persons through partnerships with various federal, state, and tribal agencies, particularly focusing on the Mississippi Band of Choctaw Indians. This initiative coincides with the recognition of May 5 as National Missing or Murdered Indigenous Persons Awareness Day, emphasizing ongoing challenges faced by Tribal communities, including violence and human trafficking. The Department of Justice has established the Missing or Murdered Indigenous Persons Regional Outreach Program to bolster law enforcement cooperation and ensure better responses to these cases. Key officials, including U.S. Attorney Todd Gee and FBI Director Christopher Wray, stress the importance of collaboration to support affected communities. Overall, the initiative aims to create safer environments for Indigenous populations while addressing public safety challenges.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The proclamation honors the history, cultures, and contributions of Native peoples, increasing awareness and appreciation among the general public.  
-2. It emphasizes the importance of respecting Tribal sovereignty and self-determination, promoting a stronger partnership between the federal government and Tribal Nations.  
-3. The legislation reflects a commitment to invest in Tribal Nations and address critical issues such as missing and murdered Indigenous peoples, which can lead to improved support and resources for affected communities.  
-4. By encouraging all Americans to observe National Native American Heritage Month with appropriate programs and activities, it fosters community engagement and education about Indigenous issues.  
-5. The gender-inclusive language acknowledges the experiences of both men and women, promoting a more comprehensive understanding of the challenges faced by Indigenous communities.  </t>
+          <t>1. Enhances cooperation between federal, state, and tribal agencies to address the crisis of missing or murdered Indigenous persons.
+2. Recognizes May 5 as National Missing or Murdered Indigenous Persons Awareness Day, raising public awareness about ongoing challenges in Tribal communities.
+3. Establishes the Missing or Murdered Indigenous Persons Regional Outreach Program to improve prevention and response efforts across designated regions.
+4. Expands the focus to include all Indigenous persons affected by violence, promoting a gender-inclusive approach in addressing these issues.
+5. Strengthens partnerships with Indigenous organizations, exemplified by collaboration with the Mississippi Band of Choctaw Indians, fostering community involvement.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The legislation does not include explicit mechanisms for evaluation, making it difficult to assess the effectiveness of its initiatives and commitments.  
-2. There is a lack of direct input or consultation from MMIP survivors or their relatives, which may limit the relevance and responsiveness of the efforts to the needs of affected communities.  
-3. While it acknowledges Indigenous communities, the absence of detailed examples of community engagement suggests that voices from these communities may not be fully centered in the legislative process.  
-4. The reliance on partnerships with Tribal Nations without specifying how these partnerships will be structured may lead to inconsistencies in the implementation of initiatives across different regions.  
-5. The focus on broad awareness and recognition may not translate into tangible actions or changes for Indigenous communities facing ongoing challenges.  </t>
+          <t xml:space="preserve">1. There is a lack of explicit references to direct input or involvement from MMIP survivors or their relatives in shaping the legislative initiatives.  
+2. Although the legislation acknowledges partnerships with Indigenous communities, it does not detail how these collaborations specifically influence decisions or outcomes regarding the crisis.  
+3. The focus on collaborative efforts may lead to potential gaps in accountability or effectiveness if community voices are not adequately represented in the decision-making process.  
+4. The articulation of the input from Indigenous politicians and community stakeholders is somewhat vague, limiting the perception of genuine engagement.  
+5. The absence of a clear mechanism to incorporate survivor experiences or feedback means that the initiative may not fully address the specific needs of those most affected by the crisis.  </t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>1. No mechanisms for evaluation are explicitly mentioned in the legislation.</t>
+          <t>1. The response to the Not Invisible Act Commission’s recommendations on how to combat the missing or murdered Indigenous peoples (MMIP) and human trafficking crisis.
+2. Consultation with the Bureau of Indian Affairs’ Missing and Murdered Unit regarding cases concerning reports of missing or murdered Indigenous persons. 
+3. The creation of the Missing or Murdered Indigenous Persons (MMIP) Regional Outreach Program, which includes placing attorneys and coordinators in designated regions to aid in prevention and response activities.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -653,7 +655,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>The legislation refers to the "epidemic of missing and murdered Indigenous peoples," which broadens the focus beyond just women to include all Indigenous individuals. This language shift promotes inclusivity and acknowledges the experiences of both men and women in these crises. Overall, it reflects a more comprehensive approach to addressing issues affecting Indigenous communities.</t>
+          <t>The legislation expands the focus from solely missing and murdered Indigenous women to encompass the broader category of missing or murdered Indigenous persons, indicating a gender-inclusive approach. It uses phrases like "missing or murdered Indigenous persons" rather than exclusively highlighting women, thereby acknowledging the impact of this crisis on all gender identities within Indigenous communities. This broader language reflects an awareness of the various individuals affected by violence in these communities.</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -663,19 +665,19 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1. "My Administration is also working to ensure that Native communities are safe and secure and have the resources they need to thrive."
-2. "I signed an Executive Order that improves the Federal response to the epidemic of missing and murdered Indigenous peoples."
-3. "When we reauthorized the Violence Against Women Act in 2022, we included historic provisions to reaffirm Tribal sovereignty and expand Tribal jurisdiction in cases where outside perpetrators harm members of their Nation."</t>
+          <t>1. “In recognition of the National Day of Awareness for Missing and Murdered Indigenous Women, the United States Attorney’s Office has joined forces with the Mississippi Band of Choctaw Indians to raise awareness for MMIW by asking everyone to wear red on Friday, May 3, 2024, to make visible those indigenous women that have disappeared and/or been murdered.” 
+2. “The Justice Department joins its partners across the federal government, as well as people throughout American Indian and Alaska Native communities, in recognizing May 5 as National Missing or Murdered Indigenous Persons (MMIP) Awareness Day.” 
+3. “Last July, the Justice Department announced the creation of the Missing or Murdered Indigenous Persons (MMIP) Regional Outreach Program, which permanently places 10 attorneys and coordinators in five designated regions across the United States to aid in the prevention and response to missing or murdered Indigenous people.”</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Somewhat</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>The legislation emphasizes collaboration with the Mississippi Band of Choctaw Indians and mentions partnerships with federal and state law enforcement agencies to address the crisis of Missing and Murdered Indigenous Persons. However, there is a lack of explicit references to direct input or involvement from MMIP survivors or their relatives in shaping the legislative initiatives. While the presence of the Mississippi Band of Choctaw Indians indicates potential community engagement, the text does not detail how survivors' voices or experiences have specifically influenced the legislation or its implementation. Therefore, the level of input is assessed as "Somewhat."</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -685,19 +687,15 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>The legislation does not explicitly mention direct input from MMIP survivors or their relatives but emphasizes partnerships with Tribal Nations, which suggests a level of inclusion. Indigenous politicians, like Deb Haaland, are highlighted in their roles, indicating representation at high government levels, but specific community engagement is not detailed. Overall, the language reflects an acknowledgment of Indigenous communities while lacking concrete examples of their input in shaping the legislation.</t>
+          <t>The legislation acknowledges the importance of partnerships with the Mississippi Band of Choctaw Indians and highlights efforts to work collaboratively with various stakeholders, including Tribal law enforcement and community members, to address the crisis of Missing and Murdered Indigenous Persons. It references a joint response to recommendations from the Not Invisible Act Commission, indicating a broader consultation process, but does not explicitly detail direct input from survivors or their relatives. Therefore, while there is recognition of community involvement, the specifics of survivor input are not clearly articulated in the text.</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>Deb Haaland (Laguna Pueblo) - 54th United States Secretary of the Interior, 2021–present</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>Deb Haaland (Laguna Pueblo) - 54th United States Secretary of the Interior, 2021–present</t>
-        </is>
-      </c>
+          <t>U.S. Attorney Todd Gee - U.S. Attorney's Office for the Southern District of Mississippi, FBI Director Christopher Wray - Federal Bureau of Investigation, DEA Administrator Anne Milgram - Drug Enforcement Administration, Cyrus Ben (Mississippi Band of Choctaw Indians) - Tribal Chief, Dianne Maxwell (Choctaw Nation) - Choctaw Attorney General, Brian K. Burns - M.B.C.I. Special Assistant United States Attorney.</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr">
         <is>
           <t>Biden Administration, 2020-2024</t>
@@ -705,12 +703,161 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>Taskforce, Day of Recognition, US Law Enforcement, Tribal Law Enforcement, Data Collection</t>
+          <t>Taskforce, Day of Recognition, US Law Enforcement, Tribal Law Enforcement</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>2024-10-31</t>
+          <t>2024-05-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>National</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Justice Department Strengthens Efforts to Address the Crisis of Missing or Murdered Indigenous Persons</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Department of Justice</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>May 5, 2023 - For Immediate Release, U.S. Attorney's Office, District of Colorado</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>https://www.justice.gov/usao-co/pr/justice-department-strengthens-efforts-address-crisis-missing-or-murdered-indigenous</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>The document outlines the Justice Department's commitment to addressing the crisis of Missing or Murdered Indigenous Persons (MMIP), highlighted by the recognition of May 5, 2023, as National Missing or Murdered Indigenous Persons Awareness Day. It emphasizes a collaborative approach involving federal, state, and tribal organizations to combat violence against American Indian and Alaska Native communities. Key initiatives include the Not Invisible Act Commission and the provision of resources for Tribes to develop response plans for missing persons cases. The department's ongoing efforts include updated guidelines for victim support and federal strategies to improve safety in Indian country. Overall, the initiative aims to reduce violence and support victims while enhancing coordination among law enforcement agencies.</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1. Establishes a holistic approach to addressing the crisis of Missing or Murdered Indigenous Persons (MMIP) through collaboration among federal, state, and tribal organizations.  
+2. Recognizes May 5, 2023, as National Missing or Murdered Indigenous Persons Awareness Day, raising public awareness of the issue.  
+3. Supports the creation of the Not Invisible Act Commission, which provides a platform for input from survivors and their families.  
+4. Offers resources for Indigenous tribes to develop response plans for missing persons cases tailored to their specific needs and cultural contexts.  
+5. Expands guidelines for victim support, ensuring that victims' voices are heard during criminal proceedings.  
+6. Provides grant funding and support to tribal communities for awareness efforts and response strategies related to missing persons cases.  
+7. Promotes data collection and research on MMIP cases, informing effective strategies to reduce violence and support affected communities.</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Although the legislation acknowledges the input of MMIP survivors and their families, specific details or mechanisms for directly incorporating their voices are limited.  
+2. The focus on a collaborative approach may lead to slower implementation of much-needed immediate actions to address the crisis.  
+3. While it establishes several initiatives, there is no clear timeline for the delivery of recommendations or the effectiveness of the responses involved.  
+4. The effectiveness of resources allocated to Tribes may vary, and there is a risk that some communities may not fully benefit from the support provided.  
+5. The document does not outline specific accountability measures to ensure that the commitments made will be followed through effectively.  </t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. "Later this year, the Commission will deliver recommendations for addressing the MMIP crisis to the Attorney General and the Secretary."  
+2. "The department published a Guide to Developing a Tribal Community Response Plan for Missing Persons Cases."  
+3. "The department’s National Institute of Justice (NIJ) funded a study that will provide vital information regarding the prevalence and context of cases of MMIP in New Mexico and, importantly, will inform long-term data collection, analysis, and reporting strategies on MMIP cases."  </t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>The document uses gender-inclusive language by referring to the crisis as "Missing or Murdered Indigenous Persons" instead of solely focusing on women. This broader terminology acknowledges that individuals of all genders can be affected by violence and goes beyond the traditional framing of the issue. By doing so, it promotes a more comprehensive understanding of the crisis impacting Indigenous communities.</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. "Responding to the unacceptable levels of violence that have led to the crisis of Missing or Murdered Indigenous Persons (MMIP) is a priority of the Department of Justice every day."  
+2. "The department remains steadfast in its commitment to addressing the MMIP crisis."  
+3. "Missing or Murdered Indigenous Persons Awareness Day calls on our nation to pause and honor the loved ones who have gone missing or who have been the victims of violent crime."  
+4. "The Justice Department is committed to using every resource at its disposal to combat the Missing or Murdered Indigenous Persons Crisis."  
+5. "We are providing grant funding and guidance to help Tribes develop response plans for missing-persons cases, partner effectively with local law enforcement, and provide resources for victims of crime."  
+6. "This Guide is a resource for Tribes interested in developing a plan to respond to missing person cases that is tailored to the specific needs, resources, and culture of Tribal communities."  
+7. "The department’s Office for Victims of Crime (OVC) expanded the scope of allowable activities under its Tribal Victim Services Set-Aside (TVSSA) grant program to permit Tribal communities to pay for costs related to generating awareness of individual missing persons cases involving American Indians and Alaska Native persons."  
+8. "Government-to-Government Tribal Consultation on Violence Against Women ... conducted annual government-to-government consultations with the leaders of all Federally recognized Indian Tribal governments on behalf of the Attorney General."  </t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>The legislation includes references to the creation of the Not Invisible Act Commission, which is designed to address the crisis of Missing or Murdered Indigenous Persons (MMIP). This commission suggests an organized approach to gather input from various stakeholders, including MMIP survivors and their families. Additionally, the text mentions plans for consultations and discussions with Tribal leaders and governments, indicating an intention to incorporate Indigenous perspectives and experiences, further supporting the notion that the legislation seeks to involve those affected by the crisis</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Somewhat</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>The legislation mentions the creation of the Not Invisible Act Commission, which aims to address violence against American Indians and Alaska Natives, implying a platform for input from various stakeholders, including MMIP survivors and their families. Additionally, the initiative's commitment to working with Tribal governments and communities suggests an intent to involve Indigenous voices in the process. However, while there are references to collaborative efforts, specific details on direct input from survivors or Indigenous politicians are limited.</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>Deputy Attorney General Lisa Monaco - Department of Justice, Secretary Deb Haaland (Laguna Pueblo) - 54th United States Secretary of the Interior, 2021–2025, Cole Finegan - U.S. Attorney for the District of Colorado, Attorney General Merrick B. Garland - Department of Justice, Associate Attorney General Vanita Gupta - Department of Justice</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>Secretary Deb Haaland (Laguna Pueblo) - 54th United States Secretary of the Interior, 2021–2025</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>Biden Administration, 2020-2024</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>Taskforce, Day of Recognition, US Law Enforcement, Tribal Law Enforcement, Data Collection, MMIP Relatives</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>2023-05-05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Attempt to remove erroneous error reports from try catch blocks
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -615,59 +615,60 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>The Justice Department is enhancing its efforts to address the crisis of missing or murdered Indigenous persons through partnerships with various federal, state, and tribal agencies, particularly focusing on the Mississippi Band of Choctaw Indians. This initiative coincides with the recognition of May 5 as National Missing or Murdered Indigenous Persons Awareness Day, emphasizing ongoing challenges faced by Tribal communities, including violence and human trafficking. The Department of Justice has established the Missing or Murdered Indigenous Persons Regional Outreach Program to bolster law enforcement cooperation and ensure better responses to these cases. Key officials, including U.S. Attorney Todd Gee and FBI Director Christopher Wray, stress the importance of collaboration to support affected communities. Overall, the initiative aims to create safer environments for Indigenous populations while addressing public safety challenges.</t>
+          <t>The Justice Department is enhancing its efforts to address the crisis of Missing or Murdered Indigenous Persons (MMIP), with a focus on building partnerships with Tribal communities such as the Mississippi Band of Choctaw Indians. Highlighted by Attorney General Merrick B. Garland, the initiative aims to tackle issues like violence against women, human trafficking, and the fentanyl crisis affecting Tribal populations. A regional outreach program has been established to permanently place attorneys and coordinators in five designated regions across the United States to aid in these efforts. The initiative emphasizes collaboration among federal, state, local, and Tribal law enforcement agencies to improve public safety and justice for Indigenous communities. The announcement coincides with the recognition of May 5 as National MMIP Awareness Day.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1. Enhances cooperation between federal, state, and tribal agencies to address the crisis of missing or murdered Indigenous persons.
-2. Recognizes May 5 as National Missing or Murdered Indigenous Persons Awareness Day, raising public awareness about ongoing challenges in Tribal communities.
-3. Establishes the Missing or Murdered Indigenous Persons Regional Outreach Program to improve prevention and response efforts across designated regions.
-4. Expands the focus to include all Indigenous persons affected by violence, promoting a gender-inclusive approach in addressing these issues.
-5. Strengthens partnerships with Indigenous organizations, exemplified by collaboration with the Mississippi Band of Choctaw Indians, fostering community involvement.</t>
+          <t>1. Enhances efforts to address the crisis of Missing or Murdered Indigenous Persons (MMIP) through collaboration with Tribal communities, improving public safety and justice for Indigenous populations.
+2. Emphasizes gender inclusivity by referring to the crisis as "Missing or Murdered Indigenous Persons," which addresses the needs of all genders within Indigenous communities.
+3. Establishes a regional outreach program to deploy attorneys and coordinators in multiple regions, providing dedicated resources for the prevention and response to MMIP cases.
+4. Strengthens law enforcement cooperation between federal, state, local, and Tribal agencies to effectively tackle violent crime and public safety issues in Tribal communities.
+5. Promotes awareness through initiatives like National MMIP Awareness Day, encouraging community involvement and visibility for the issue of missing and murdered Indigenous individuals.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. There is a lack of explicit references to direct input or involvement from MMIP survivors or their relatives in shaping the legislative initiatives.  
-2. Although the legislation acknowledges partnerships with Indigenous communities, it does not detail how these collaborations specifically influence decisions or outcomes regarding the crisis.  
-3. The focus on collaborative efforts may lead to potential gaps in accountability or effectiveness if community voices are not adequately represented in the decision-making process.  
-4. The articulation of the input from Indigenous politicians and community stakeholders is somewhat vague, limiting the perception of genuine engagement.  
-5. The absence of a clear mechanism to incorporate survivor experiences or feedback means that the initiative may not fully address the specific needs of those most affected by the crisis.  </t>
+          <t>1. The legislation does not provide explicit mechanisms for incorporating direct input from MMIP survivors or their relatives, limiting their voices in shaping the initiative.
+2. While community engagement is emphasized, there is a lack of detailed descriptions of how individual community members, particularly survivors and their families, will participate in the decision-making process.
+3. The initiative may not adequately address the unique needs of all Indigenous communities, potentially leading to disparities in support and resource allocation.
+4. Although partnerships with Tribal communities are highlighted, the legislation could benefit from including a broader range of Indigenous organizations that directly support MMIP survivors to enhance its effectiveness.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>1. Consultations with community
+2. Tribal consultations
+3. Monitoring
+4. Data collection</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>1. The response to the Not Invisible Act Commission’s recommendations on how to combat the missing or murdered Indigenous peoples (MMIP) and human trafficking crisis.
-2. Consultation with the Bureau of Indian Affairs’ Missing and Murdered Unit regarding cases concerning reports of missing or murdered Indigenous persons. 
-3. The creation of the Missing or Murdered Indigenous Persons (MMIP) Regional Outreach Program, which includes placing attorneys and coordinators in designated regions to aid in prevention and response activities.</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>The legislation refers to the crisis as "Missing or Murdered Indigenous Persons" (MMIP), which explicitly includes all genders rather than limiting the focus to women alone. This broadens the initiative's scope to address the needs and concerns of Indigenous communities as a whole. Additionally, throughout the text, language is used that encompasses various public safety challenges affecting Indigenous individuals regardless of gender, promoting a more inclusive approach.</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>The legislation expands the focus from solely missing and murdered Indigenous women to encompass the broader category of missing or murdered Indigenous persons, indicating a gender-inclusive approach. It uses phrases like "missing or murdered Indigenous persons" rather than exclusively highlighting women, thereby acknowledging the impact of this crisis on all gender identities within Indigenous communities. This broader language reflects an awareness of the various individuals affected by violence in these communities.</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1. “In recognition of the National Day of Awareness for Missing and Murdered Indigenous Women, the United States Attorney’s Office has joined forces with the Mississippi Band of Choctaw Indians to raise awareness for MMIW by asking everyone to wear red on Friday, May 3, 2024, to make visible those indigenous women that have disappeared and/or been murdered.” 
-2. “The Justice Department joins its partners across the federal government, as well as people throughout American Indian and Alaska Native communities, in recognizing May 5 as National Missing or Murdered Indigenous Persons (MMIP) Awareness Day.” 
-3. “Last July, the Justice Department announced the creation of the Missing or Murdered Indigenous Persons (MMIP) Regional Outreach Program, which permanently places 10 attorneys and coordinators in five designated regions across the United States to aid in the prevention and response to missing or murdered Indigenous people.”</t>
+          <t>1. "In recognition of MMIP Awareness Day, Attorney General Merrick B. Garland highlighted ongoing efforts to tackle the MMIP and human trafficking crises in American Indian and Alaska Native communities, and other pressing public safety challenges, like the fentanyl crisis, in Tribal communities."
+2. "The United States Attorney’s Office has joined forces with the Mississippi Band of Choctaw Indians to raise awareness for MMIW by asking everyone to wear red on Friday, May 3, 2024, to make visible those indigenous women that have disappeared and/or been murdered."
+3. "The Department of Justice has been working hard to strengthen law enforcement cooperation with the Mississippi Band of Choctaw Indians and other law enforcement partners in order to better address violent crime, the fentanyl crisis, and other public safety issues in Tribal communities." 
+4. "Last July, the Justice Department announced the creation of the Missing or Murdered Indigenous Persons (MMIP) Regional Outreach Program, which permanently places 10 attorneys and coordinators in five designated regions across the United States to aid in the prevention and response to missing or murdered Indigenous people."</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -677,7 +678,7 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>The legislation emphasizes collaboration with the Mississippi Band of Choctaw Indians and mentions partnerships with federal and state law enforcement agencies to address the crisis of Missing and Murdered Indigenous Persons. However, there is a lack of explicit references to direct input or involvement from MMIP survivors or their relatives in shaping the legislative initiatives. While the presence of the Mississippi Band of Choctaw Indians indicates potential community engagement, the text does not detail how survivors' voices or experiences have specifically influenced the legislation or its implementation. Therefore, the level of input is assessed as "Somewhat."</t>
+          <t>The legislation refers to the involvement of the Mississippi Band of Choctaw Indians, indicating a collaborative effort in addressing the MMIP crisis. However, it does not explicitly mention direct input or consultation from MMIP survivors or their relatives. Although the focus on awareness and community engagement suggests some level of support, there is no detailed description of processes for including individual survivor voices or experiences in shaping the initiative. Additionally, the mention of the Bureau of Indian Affairs' Missing and Murdered Unit implies organizational support, yet specific contributions from survivors or their families are not detailed</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -687,12 +688,12 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>The legislation acknowledges the importance of partnerships with the Mississippi Band of Choctaw Indians and highlights efforts to work collaboratively with various stakeholders, including Tribal law enforcement and community members, to address the crisis of Missing and Murdered Indigenous Persons. It references a joint response to recommendations from the Not Invisible Act Commission, indicating a broader consultation process, but does not explicitly detail direct input from survivors or their relatives. Therefore, while there is recognition of community involvement, the specifics of survivor input are not clearly articulated in the text.</t>
+          <t>The legislation acknowledges the importance of partnerships between the Justice Department and Tribal communities, specifically citing collaboration with the Mississippi Band of Choctaw Indians in addressing the MMIP crisis. Although it does not provide detailed mechanisms for directly incorporating input from MMIP survivors or their relatives, the emphasis on awareness events, like the MMIP Awareness Day, suggests an effort to engage these communities. Indigenous politicians, such as Tribal Chief Cyrus Ben, are referenced in supportive roles, indicating a level of involvement but not specific individual contributions from survivors or their families.</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>U.S. Attorney Todd Gee - U.S. Attorney's Office for the Southern District of Mississippi, FBI Director Christopher Wray - Federal Bureau of Investigation, DEA Administrator Anne Milgram - Drug Enforcement Administration, Cyrus Ben (Mississippi Band of Choctaw Indians) - Tribal Chief, Dianne Maxwell (Choctaw Nation) - Choctaw Attorney General, Brian K. Burns - M.B.C.I. Special Assistant United States Attorney.</t>
+          <t>U.S. Attorney Todd Gee (R) - Southern District of Mississippi, FBI Director Christopher Wray - FBI, DEA Administrator Anne Milgram - DEA, Tribal Chief Cyrus Ben (Mississippi Band of Choctaw Indians) - Mississippi Band of Choctaw Indians, Choctaw Attorney General Dianne Maxwell - Mississippi Band of Choctaw Indians, M.B.C.I. Special Assistant United States Attorney Brian K. Burns - Mississippi Band of Choctaw Indians.</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr"/>
@@ -723,7 +724,11 @@
           <t>Justice Department Strengthens Efforts to Address the Crisis of Missing or Murdered Indigenous Persons</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>DOJ23-1013</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>Passed</t>
@@ -753,27 +758,28 @@
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>The document outlines the Justice Department's commitment to addressing the crisis of Missing or Murdered Indigenous Persons (MMIP), highlighted by the recognition of May 5, 2023, as National Missing or Murdered Indigenous Persons Awareness Day. It emphasizes a collaborative approach involving federal, state, and tribal organizations to combat violence against American Indian and Alaska Native communities. Key initiatives include the Not Invisible Act Commission and the provision of resources for Tribes to develop response plans for missing persons cases. The department's ongoing efforts include updated guidelines for victim support and federal strategies to improve safety in Indian country. Overall, the initiative aims to reduce violence and support victims while enhancing coordination among law enforcement agencies.</t>
+          <t>The Justice Department has intensified its efforts to address the crisis of Missing or Murdered Indigenous Persons (MMIP), recognizing May 5, 2023, as National Missing or Murdered Indigenous Persons Awareness Day. The initiative includes the establishment of the Not Invisible Act Commission, which aims to reduce violence against American Indian and Alaska Native communities. Attorney General Merrick B. Garland and other officials emphasize a comprehensive, collaborative approach involving federal, state, and tribal partnerships to confront this crisis. The department is committed to using its resources effectively to support tribes in developing response plans for missing persons cases and to improve public safety in Indian country. Additionally, ongoing collaborations and the implementation of updated guidelines demonstrate a focused effort to respond to the needs of affected individuals and communities.</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1. Establishes a holistic approach to addressing the crisis of Missing or Murdered Indigenous Persons (MMIP) through collaboration among federal, state, and tribal organizations.  
-2. Recognizes May 5, 2023, as National Missing or Murdered Indigenous Persons Awareness Day, raising public awareness of the issue.  
-3. Supports the creation of the Not Invisible Act Commission, which provides a platform for input from survivors and their families.  
-4. Offers resources for Indigenous tribes to develop response plans for missing persons cases tailored to their specific needs and cultural contexts.  
-5. Expands guidelines for victim support, ensuring that victims' voices are heard during criminal proceedings.  
-6. Provides grant funding and support to tribal communities for awareness efforts and response strategies related to missing persons cases.  
-7. Promotes data collection and research on MMIP cases, informing effective strategies to reduce violence and support affected communities.</t>
+          <t xml:space="preserve">1. Establishes the Not Invisible Act Commission to directly address and reduce violence against American Indian and Alaska Native communities.  
+2. Recognizes May 5, 2023, as National Missing or Murdered Indigenous Persons Awareness Day, raising public awareness about the crisis.  
+3. Promotes a comprehensive and collaborative approach involving federal, state, and tribal partnerships to enhance public safety and support Indigenous communities.  
+4. Provides resources and guidance for tribes to develop tailored response plans for missing persons cases.  
+5. Expands the scope of funding under the Tribal Victim Services Set-Aside grant program, allowing tribal communities to generate awareness and support for individual missing persons cases.  
+6. Incorporates input from MMIP survivors and their families through the creation of a National Native American Outreach Services Liaison.  
+7. Acknowledges and addresses the unique challenges faced by Indigenous populations in relation to violence and abductions.  
+8. Supports data-driven decision-making regarding MMIP cases to improve future responses and strategies.  </t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Although the legislation acknowledges the input of MMIP survivors and their families, specific details or mechanisms for directly incorporating their voices are limited.  
-2. The focus on a collaborative approach may lead to slower implementation of much-needed immediate actions to address the crisis.  
-3. While it establishes several initiatives, there is no clear timeline for the delivery of recommendations or the effectiveness of the responses involved.  
-4. The effectiveness of resources allocated to Tribes may vary, and there is a risk that some communities may not fully benefit from the support provided.  
-5. The document does not outline specific accountability measures to ensure that the commitments made will be followed through effectively.  </t>
+          <t xml:space="preserve">1. The effectiveness of the initiatives may depend on the level of collaboration and commitment from multiple stakeholders, which can vary.  
+2. While the legislation promotes awareness, there may be challenges in implementing changes at the local level due to existing systemic issues and resource constraints.  
+3. The focus on grant funding may not guarantee sustained support or long-term solutions for all tribes, particularly smaller or less recognized communities.  
+4. The involvement of federal agencies could lead to concerns about sovereignty and self-determination among Indigenous communities regarding the handling of MMIP cases.  
+5. The legislation may lack explicit timelines or measurable outcomes, making it difficult to assess progress and accountability.  </t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -783,9 +789,10 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. "Later this year, the Commission will deliver recommendations for addressing the MMIP crisis to the Attorney General and the Secretary."  
-2. "The department published a Guide to Developing a Tribal Community Response Plan for Missing Persons Cases."  
-3. "The department’s National Institute of Justice (NIJ) funded a study that will provide vital information regarding the prevalence and context of cases of MMIP in New Mexico and, importantly, will inform long-term data collection, analysis, and reporting strategies on MMIP cases."  </t>
+          <t>1. "Since then, the department’s representatives on the commission—who are department leaders and subject matter experts—have participated in the Commission’s field hearings, which will continue through the summer."  
+2. "Later this year, the Commission will deliver recommendations for addressing the MMIP crisis to the Attorney General and the Secretary."  
+3. "This Guide is a resource for Tribes interested in developing a plan to respond to missing person cases that is tailored to the specific needs, resources, and culture of Tribal communities."  
+4. "These improvements will support data-driven decision-making regarding MMIP in New Mexico moving forward."</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -795,7 +802,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>The document uses gender-inclusive language by referring to the crisis as "Missing or Murdered Indigenous Persons" instead of solely focusing on women. This broader terminology acknowledges that individuals of all genders can be affected by violence and goes beyond the traditional framing of the issue. By doing so, it promotes a more comprehensive understanding of the crisis impacting Indigenous communities.</t>
+          <t>The legislation refers to the "Missing or Murdered Indigenous Persons" (MMIP) crisis, which inclusively addresses both men and women rather than focusing solely on women. This choice of language acknowledges that individuals of all genders are affected by violence and abductions within Indigenous communities. By using the term "persons," the legislation promotes a broader understanding of the issue and its impact on diverse Indigenous populations.</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -805,14 +812,11 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. "Responding to the unacceptable levels of violence that have led to the crisis of Missing or Murdered Indigenous Persons (MMIP) is a priority of the Department of Justice every day."  
-2. "The department remains steadfast in its commitment to addressing the MMIP crisis."  
-3. "Missing or Murdered Indigenous Persons Awareness Day calls on our nation to pause and honor the loved ones who have gone missing or who have been the victims of violent crime."  
-4. "The Justice Department is committed to using every resource at its disposal to combat the Missing or Murdered Indigenous Persons Crisis."  
-5. "We are providing grant funding and guidance to help Tribes develop response plans for missing-persons cases, partner effectively with local law enforcement, and provide resources for victims of crime."  
-6. "This Guide is a resource for Tribes interested in developing a plan to respond to missing person cases that is tailored to the specific needs, resources, and culture of Tribal communities."  
-7. "The department’s Office for Victims of Crime (OVC) expanded the scope of allowable activities under its Tribal Victim Services Set-Aside (TVSSA) grant program to permit Tribal communities to pay for costs related to generating awareness of individual missing persons cases involving American Indians and Alaska Native persons."  
-8. "Government-to-Government Tribal Consultation on Violence Against Women ... conducted annual government-to-government consultations with the leaders of all Federally recognized Indian Tribal governments on behalf of the Attorney General."  </t>
+          <t xml:space="preserve">1. "The Justice Department joins its partners across the federal government, as well as people throughout American Indian and Alaska Native communities, in recognizing May 5, 2023 as National Missing or Murdered Indigenous Persons Awareness Day."  
+2. "The Justice Department is committed to using every resource at its disposal to combat the Missing or Murdered Indigenous Persons Crisis."  
+3. "We are providing grant funding and guidance to help Tribes develop response plans for missing-persons cases, partner effectively with local law enforcement, and provide resources for victims of crime."  
+4. "This Guide is a resource for Tribes interested in developing a plan to respond to missing person cases that is tailored to the specific needs, resources, and culture of Tribal communities."  
+5. "The department's Office for Victims of Crime (OVC) expanded the scope of allowable activities under its Tribal Victim Services Set-Aside (TVSSA) grant program to permit Tribal communities to pay for costs related to generating awareness of individual missing persons cases involving American Indians and Alaska Native persons."  </t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -822,7 +826,7 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>The legislation includes references to the creation of the Not Invisible Act Commission, which is designed to address the crisis of Missing or Murdered Indigenous Persons (MMIP). This commission suggests an organized approach to gather input from various stakeholders, including MMIP survivors and their families. Additionally, the text mentions plans for consultations and discussions with Tribal leaders and governments, indicating an intention to incorporate Indigenous perspectives and experiences, further supporting the notion that the legislation seeks to involve those affected by the crisis</t>
+          <t>The legislation explicitly mentions the creation of a National Native American Outreach Services Liaison, which aims to amplify the voices of crime victims in Indian country, including MMIP survivors and their families. Additionally, it discusses the department's commitment to developing response plans for missing-persons cases that incorporate input from Indigenous communities, suggesting a mechanism for engagement with affected individuals. The overall focus on collaboration with Tribal governments and the acknowledgment of the unique challenges faced by MMIP cases indicate a recognition of the importance of survivor and family input in addressing this crisis</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -832,27 +836,27 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>The legislation mentions the creation of the Not Invisible Act Commission, which aims to address violence against American Indians and Alaska Natives, implying a platform for input from various stakeholders, including MMIP survivors and their families. Additionally, the initiative's commitment to working with Tribal governments and communities suggests an intent to involve Indigenous voices in the process. However, while there are references to collaborative efforts, specific details on direct input from survivors or Indigenous politicians are limited.</t>
+          <t>The legislation emphasizes a collaborative approach involving multiple stakeholders, including Indigenous communities, to address the MMIP crisis. It mentions ongoing participation from department leaders and subject matter experts in field hearings, which implies input from affected individuals and communities. Additionally, the creation of a National Native American Outreach Services Liaison suggests a structured effort to amplify the voices of MMIP survivors and their families.</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Deputy Attorney General Lisa Monaco - Department of Justice, Secretary Deb Haaland (Laguna Pueblo) - 54th United States Secretary of the Interior, 2021–2025, Cole Finegan - U.S. Attorney for the District of Colorado, Attorney General Merrick B. Garland - Department of Justice, Associate Attorney General Vanita Gupta - Department of Justice</t>
+          <t>Deputy Attorney General Lisa Monaco - Department of Justice, Secretary of the Interior Deb Haaland (Laguna Pueblo) - 54th United States Secretary of the Interior, 2021–2025, Cole Finegan - U.S. Attorney (District of Colorado), Vanita Gupta - Associate Attorney General</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Secretary Deb Haaland (Laguna Pueblo) - 54th United States Secretary of the Interior, 2021–2025</t>
+          <t>Secretary of the Interior Deb Haaland (Laguna Pueblo) - 54th United States Secretary of the Interior, 2021–2025</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>Biden Administration, 2020-2024</t>
+          <t>Biden Administration, 2020 - 2024</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>Taskforce, Day of Recognition, US Law Enforcement, Tribal Law Enforcement, Data Collection, MMIP Relatives</t>
+          <t>Taskforce, Day of Recognition, US Law Enforcement, Tribal Law Enforcement, Data Collection</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">

</xml_diff>

<commit_message>
Added CORS support for server wakeup redirect
</commit_message>
<xml_diff>
--- a/bill_details.xlsx
+++ b/bill_details.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB3"/>
+  <dimension ref="A1:AB9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -615,91 +615,91 @@
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>The Justice Department is enhancing its efforts to address the crisis of Missing or Murdered Indigenous Persons (MMIP), with a focus on building partnerships with Tribal communities such as the Mississippi Band of Choctaw Indians. Highlighted by Attorney General Merrick B. Garland, the initiative aims to tackle issues like violence against women, human trafficking, and the fentanyl crisis affecting Tribal populations. A regional outreach program has been established to permanently place attorneys and coordinators in five designated regions across the United States to aid in these efforts. The initiative emphasizes collaboration among federal, state, local, and Tribal law enforcement agencies to improve public safety and justice for Indigenous communities. The announcement coincides with the recognition of May 5 as National MMIP Awareness Day.</t>
+          <t>The Justice Department is enhancing efforts to address the crisis of Missing or Murdered Indigenous Persons (MMIP) in collaboration with tribal communities, notably the Mississippi Band of Choctaw Indians. The initiative includes recognizing May 5 as National MMIP Awareness Day and focuses on improving law enforcement cooperation to tackle violent crime and human trafficking in tribal areas. Attorney General Merrick B. Garland emphasized the need for ongoing partnerships to provide safety and justice for tribal communities. Additionally, the Department is prioritizing MMIP cases through a regional outreach program and implementing strategies to address public safety challenges in Indian country. This effort highlights a coordinated response involving various government agencies and tribal authorities.</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1. Enhances efforts to address the crisis of Missing or Murdered Indigenous Persons (MMIP) through collaboration with Tribal communities, improving public safety and justice for Indigenous populations.
-2. Emphasizes gender inclusivity by referring to the crisis as "Missing or Murdered Indigenous Persons," which addresses the needs of all genders within Indigenous communities.
-3. Establishes a regional outreach program to deploy attorneys and coordinators in multiple regions, providing dedicated resources for the prevention and response to MMIP cases.
-4. Strengthens law enforcement cooperation between federal, state, local, and Tribal agencies to effectively tackle violent crime and public safety issues in Tribal communities.
-5. Promotes awareness through initiatives like National MMIP Awareness Day, encouraging community involvement and visibility for the issue of missing and murdered Indigenous individuals.</t>
+          <t>1. Enhances efforts to address the crisis of Missing or Murdered Indigenous Persons (MMIP) through collaboration with tribal communities, improving overall community safety and justice.  
+2. Recognizes May 5 as National MMIP Awareness Day, raising awareness and promoting public education about the issue.  
+3. Strengthens law enforcement cooperation at both federal and tribal levels to tackle violent crime and human trafficking in tribal areas.  
+4. Implements a regional outreach program to prioritize MMIP cases and allocate resources effectively to respond to the crisis.  
+5. Supports a gender-inclusive approach by addressing the needs of all Indigenous persons affected by violence, not just women.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>1. The legislation does not provide explicit mechanisms for incorporating direct input from MMIP survivors or their relatives, limiting their voices in shaping the initiative.
-2. While community engagement is emphasized, there is a lack of detailed descriptions of how individual community members, particularly survivors and their families, will participate in the decision-making process.
-3. The initiative may not adequately address the unique needs of all Indigenous communities, potentially leading to disparities in support and resource allocation.
-4. Although partnerships with Tribal communities are highlighted, the legislation could benefit from including a broader range of Indigenous organizations that directly support MMIP survivors to enhance its effectiveness.</t>
+          <t>1. The legislation does not provide specific input or testimony from MMIP survivors or their relatives, potentially limiting personal perspectives and needs in the response efforts.  
+2. While it emphasizes partnerships with tribal communities, the level of engagement and direct involvement from Indigenous voices appears to be only "somewhat" included, suggesting room for improvement.  
+3. The legislation may rely heavily on law enforcement strategies without incorporating broader community-led initiatives that address underlying social issues contributing to the MMIP crisis.  
+4. Although it aims to raise awareness, there is no detailed plan for ongoing evaluation or monitoring of the initiatives' effectiveness in addressing the MMIP crisis.</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>1. "The MMIP Regional Outreach Program prioritizes MMIP cases consistent with the Deputy Attorney General’s July 2022 directive to U.S. Attorneys’ offices promoting public safety in Indian country."
+2. "The program fulfills the Justice Department’s promise to dedicate new personnel to MMIP consistent with Executive Order 14053."
+3. "The Department’s work to respond to the MMIP crisis is a whole-of-department effort." 
+4. "In March, the Departments of Justice and the Interior released their joint response to the Not Invisible Act Commission’s recommendations on how to combat the missing or murdered Indigenous peoples (MMIP) and human trafficking crisis."</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>The legislation addresses the crisis by referring to "Missing or Murdered Indigenous Persons" (MMIP), which encompasses all genders rather than focusing solely on women. This terminology reflects a broader acknowledgment of the issues faced by both men and women in Indigenous communities. Additionally, the language throughout emphasizes support for all individuals affected by violence and missing persons cases, promoting inclusivity.</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>1. "The Justice Department joins its partners across the federal government, as well as people throughout American Indian and Alaska Native communities, in recognizing May 5 as National Missing or Murdered Indigenous Persons (MMIP) Awareness Day."
+2. "In recognition of the National Day of Awareness for Missing and Murdered Indigenous Women, the United States Attorney’s Office has joined forces with the Mississippi Band of Choctaw Indians to raise awareness for MMIW by asking everyone to wear red on Friday, May 3, 2024, to make visible those indigenous women that have disappeared and/or been murdered."
+3. "The MMIP Regional Outreach Program prioritizes MMIP cases consistent with the Deputy Attorney General’s July 2022 directive to U.S. Attorneys’ offices promoting public safety in Indian country." 
+4. "Last July, the Justice Department announced the creation of the Missing or Murdered Indigenous Persons (MMIP) Regional Outreach Program, which permanently places 10 attorneys and coordinators in five designated regions across the United States to aid in the prevention and response to missing or murdered Indigenous people."</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>1. Consultations with community
-2. Tribal consultations
-3. Monitoring
-4. Data collection</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>The legislation refers to the crisis as "Missing or Murdered Indigenous Persons" (MMIP), which explicitly includes all genders rather than limiting the focus to women alone. This broadens the initiative's scope to address the needs and concerns of Indigenous communities as a whole. Additionally, throughout the text, language is used that encompasses various public safety challenges affecting Indigenous individuals regardless of gender, promoting a more inclusive approach.</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>1. "In recognition of MMIP Awareness Day, Attorney General Merrick B. Garland highlighted ongoing efforts to tackle the MMIP and human trafficking crises in American Indian and Alaska Native communities, and other pressing public safety challenges, like the fentanyl crisis, in Tribal communities."
-2. "The United States Attorney’s Office has joined forces with the Mississippi Band of Choctaw Indians to raise awareness for MMIW by asking everyone to wear red on Friday, May 3, 2024, to make visible those indigenous women that have disappeared and/or been murdered."
-3. "The Department of Justice has been working hard to strengthen law enforcement cooperation with the Mississippi Band of Choctaw Indians and other law enforcement partners in order to better address violent crime, the fentanyl crisis, and other public safety issues in Tribal communities." 
-4. "Last July, the Justice Department announced the creation of the Missing or Murdered Indigenous Persons (MMIP) Regional Outreach Program, which permanently places 10 attorneys and coordinators in five designated regions across the United States to aid in the prevention and response to missing or murdered Indigenous people."</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
         <is>
           <t>Somewhat</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>The legislation refers to the involvement of the Mississippi Band of Choctaw Indians, indicating a collaborative effort in addressing the MMIP crisis. However, it does not explicitly mention direct input or consultation from MMIP survivors or their relatives. Although the focus on awareness and community engagement suggests some level of support, there is no detailed description of processes for including individual survivor voices or experiences in shaping the initiative. Additionally, the mention of the Bureau of Indian Affairs' Missing and Murdered Unit implies organizational support, yet specific contributions from survivors or their families are not detailed</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>Somewhat</t>
-        </is>
-      </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>The legislation acknowledges the importance of partnerships between the Justice Department and Tribal communities, specifically citing collaboration with the Mississippi Band of Choctaw Indians in addressing the MMIP crisis. Although it does not provide detailed mechanisms for directly incorporating input from MMIP survivors or their relatives, the emphasis on awareness events, like the MMIP Awareness Day, suggests an effort to engage these communities. Indigenous politicians, such as Tribal Chief Cyrus Ben, are referenced in supportive roles, indicating a level of involvement but not specific individual contributions from survivors or their families.</t>
+          <t>The legislation emphasizes the importance of partnerships with Tribal communities and mentions the involvement of the Mississippi Band of Choctaw Indians, indicating some level of engagement with Indigenous communities. It also references the commitment to recognize National Missing or Murdered Indigenous Persons Awareness Day and discusses collaborative efforts, suggesting an attempt to include voices from these communities in awareness and prevention measures. However, specific testimony or input from MMIP survivors or their relatives is not detailed in the text, leading to a conclusion of "Somewhat" regarding direct input.</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>U.S. Attorney Todd Gee (R) - Southern District of Mississippi, FBI Director Christopher Wray - FBI, DEA Administrator Anne Milgram - DEA, Tribal Chief Cyrus Ben (Mississippi Band of Choctaw Indians) - Mississippi Band of Choctaw Indians, Choctaw Attorney General Dianne Maxwell - Mississippi Band of Choctaw Indians, M.B.C.I. Special Assistant United States Attorney Brian K. Burns - Mississippi Band of Choctaw Indians.</t>
+          <t>U.S. Attorney Todd Gee (R) - Southern District of Mississippi, FBI Director Christopher Wray - Federal Bureau of Investigation, DEA Administrator Anne Milgram - Drug Enforcement Administration, Mississippi Band of Choctaw Indians Tribal Chief Cyrus Ben (Mississippi Band of Choctaw Indians) - Tribal Government, Choctaw Attorney General Dianne Maxwell (Mississippi Band of Choctaw Indians) - Tribal Government, M.B.C.I. Special Assistant United States Attorney Brian K. Burns - United States Attorney's Office for the Southern District of Mississippi.</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>Biden Administration, 2020-2024</t>
+          <t>Biden Administration, 2020 - 2024</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -716,17 +716,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>National</t>
+          <t>NM</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Justice Department Strengthens Efforts to Address the Crisis of Missing or Murdered Indigenous Persons</t>
+          <t>Justice Department Launches Missing or Murdered Indigenous Persons Regional Outreach Program</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DOJ23-1013</t>
+          <t>DOJ23-138</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -746,53 +746,47 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>May 5, 2023 - For Immediate Release, U.S. Attorney's Office, District of Colorado</t>
+          <t>June 28, 2023 - Immediate release, U.S. Attorney's Office, District of New Mexico</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://www.justice.gov/usao-co/pr/justice-department-strengthens-efforts-address-crisis-missing-or-murdered-indigenous</t>
+          <t>https://www.justice.gov/usao-nm/pr/justice-department-launches-missing-or-murdered-indigenous-persons-regional-outreach</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>The Justice Department has intensified its efforts to address the crisis of Missing or Murdered Indigenous Persons (MMIP), recognizing May 5, 2023, as National Missing or Murdered Indigenous Persons Awareness Day. The initiative includes the establishment of the Not Invisible Act Commission, which aims to reduce violence against American Indian and Alaska Native communities. Attorney General Merrick B. Garland and other officials emphasize a comprehensive, collaborative approach involving federal, state, and tribal partnerships to confront this crisis. The department is committed to using its resources effectively to support tribes in developing response plans for missing persons cases and to improve public safety in Indian country. Additionally, ongoing collaborations and the implementation of updated guidelines demonstrate a focused effort to respond to the needs of affected individuals and communities.</t>
+          <t>The Justice Department has launched the Missing or Murdered Indigenous Persons (MMIP) Regional Outreach Program to address the crisis of missing or murdered Indigenous individuals across the United States. This initiative places ten dedicated attorneys and coordinators in five regions, providing specialized support to combat this issue in New Mexico, Colorado, Utah, Nevada, and Arizona. Attorney General Merrick B. Garland emphasized the program's focus on partnering with Tribal communities to enhance public safety and deliver justice for victims and their families. The MMIP program is part of the Department's broader strategy to improve criminal justice and public safety for Native Americans, as directed by Executive Order 14053. This initiative aims to facilitate collaboration among federal, state, and Tribal law enforcement agencies to effectively address and resolve MMIP cases.</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Establishes the Not Invisible Act Commission to directly address and reduce violence against American Indian and Alaska Native communities.  
-2. Recognizes May 5, 2023, as National Missing or Murdered Indigenous Persons Awareness Day, raising public awareness about the crisis.  
-3. Promotes a comprehensive and collaborative approach involving federal, state, and tribal partnerships to enhance public safety and support Indigenous communities.  
-4. Provides resources and guidance for tribes to develop tailored response plans for missing persons cases.  
-5. Expands the scope of funding under the Tribal Victim Services Set-Aside grant program, allowing tribal communities to generate awareness and support for individual missing persons cases.  
-6. Incorporates input from MMIP survivors and their families through the creation of a National Native American Outreach Services Liaison.  
-7. Acknowledges and addresses the unique challenges faced by Indigenous populations in relation to violence and abductions.  
-8. Supports data-driven decision-making regarding MMIP cases to improve future responses and strategies.  </t>
+          <t>1. Establishes a dedicated outreach program to address the crisis of missing or murdered Indigenous Persons, providing specialized legal support in key regions.
+2. Promotes collaboration among federal, state, and Tribal law enforcement agencies to enhance the effectiveness of investigations into MMIP cases.
+3. Utilizes resources from the Justice Department to combat the MMIP crisis, demonstrating a commitment to public safety for Indigenous communities.
+4. Engages with Tribal communities to improve public safety and deliver justice for victims and their families.
+5. Employs gender-neutral language that acknowledges the crisis affects all genders within Indigenous populations, promoting inclusivity in addressing the issue.</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The effectiveness of the initiatives may depend on the level of collaboration and commitment from multiple stakeholders, which can vary.  
-2. While the legislation promotes awareness, there may be challenges in implementing changes at the local level due to existing systemic issues and resource constraints.  
-3. The focus on grant funding may not guarantee sustained support or long-term solutions for all tribes, particularly smaller or less recognized communities.  
-4. The involvement of federal agencies could lead to concerns about sovereignty and self-determination among Indigenous communities regarding the handling of MMIP cases.  
-5. The legislation may lack explicit timelines or measurable outcomes, making it difficult to assess progress and accountability.  </t>
+          <t>1. No specific mechanisms for evaluation or monitoring are established, making it difficult to assess the effectiveness of the program over time.
+2. While the legislation acknowledges the importance of partnerships with Tribal communities, it lacks detailed input or consultation from MMIP survivors and their families.
+3. The lack of targeted support or resources for Indigenous organizations specifically focused on MMIP survivors may limit the program's impact.
+4. The initiative does not mention any concrete plans for data collection or analysis, which are essential for understanding the scope of the MMIP crisis.
+5. Although gender-inclusive language is used, the overall framework may not adequately address the unique needs of different groups within Indigenous populations affected by the crisis.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>1. "Since then, the department’s representatives on the commission—who are department leaders and subject matter experts—have participated in the Commission’s field hearings, which will continue through the summer."  
-2. "Later this year, the Commission will deliver recommendations for addressing the MMIP crisis to the Attorney General and the Secretary."  
-3. "This Guide is a resource for Tribes interested in developing a plan to respond to missing person cases that is tailored to the specific needs, resources, and culture of Tribal communities."  
-4. "These improvements will support data-driven decision-making regarding MMIP in New Mexico moving forward."</t>
+          <t>1. No specific mechanisms for evaluation are mentioned in the legislation.</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -802,7 +796,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>The legislation refers to the "Missing or Murdered Indigenous Persons" (MMIP) crisis, which inclusively addresses both men and women rather than focusing solely on women. This choice of language acknowledges that individuals of all genders are affected by violence and abductions within Indigenous communities. By using the term "persons," the legislation promotes a broader understanding of the issue and its impact on diverse Indigenous populations.</t>
+          <t>The legislation uses gender-neutral language by referring to "Missing or Murdered Indigenous Persons," which encompasses all genders rather than focusing solely on women. This approach recognizes that the crisis affects a broader demographic within Indigenous communities. Additionally, statements made by officials reinforce the importance of responding to all missing and murdered individuals, not just women.</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -812,21 +806,20 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. "The Justice Department joins its partners across the federal government, as well as people throughout American Indian and Alaska Native communities, in recognizing May 5, 2023 as National Missing or Murdered Indigenous Persons Awareness Day."  
-2. "The Justice Department is committed to using every resource at its disposal to combat the Missing or Murdered Indigenous Persons Crisis."  
-3. "We are providing grant funding and guidance to help Tribes develop response plans for missing-persons cases, partner effectively with local law enforcement, and provide resources for victims of crime."  
-4. "This Guide is a resource for Tribes interested in developing a plan to respond to missing person cases that is tailored to the specific needs, resources, and culture of Tribal communities."  
-5. "The department's Office for Victims of Crime (OVC) expanded the scope of allowable activities under its Tribal Victim Services Set-Aside (TVSSA) grant program to permit Tribal communities to pay for costs related to generating awareness of individual missing persons cases involving American Indians and Alaska Native persons."  </t>
+          <t>1. "This new program mobilizes the Justice Department’s resources to combat the crisis of Missing or Murdered Indigenous Persons, which has shattered the lives of victims, their families, and entire Tribal communities."
+2. "These new positions represent the Justice Department’s continuing commitment to addressing the MMIP crisis with urgency and all of the tools at our disposal."
+3. "MMIP prosecutors and coordinators will work with partners across jurisdictions and alongside the Tribal communities who have been most devastated by this epidemic."
+4. "This support includes assisting in the investigation of unresolved MMIP cases and related crimes, and promoting communication, coordination, and collaboration among federal, Tribal, local, and state law enforcement and non-governmental partners on MMIP issues."</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>The legislation explicitly mentions the creation of a National Native American Outreach Services Liaison, which aims to amplify the voices of crime victims in Indian country, including MMIP survivors and their families. Additionally, it discusses the department's commitment to developing response plans for missing-persons cases that incorporate input from Indigenous communities, suggesting a mechanism for engagement with affected individuals. The overall focus on collaboration with Tribal governments and the acknowledgment of the unique challenges faced by MMIP cases indicate a recognition of the importance of survivor and family input in addressing this crisis</t>
+          <t>No</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -836,30 +829,904 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>The legislation emphasizes a collaborative approach involving multiple stakeholders, including Indigenous communities, to address the MMIP crisis. It mentions ongoing participation from department leaders and subject matter experts in field hearings, which implies input from affected individuals and communities. Additionally, the creation of a National Native American Outreach Services Liaison suggests a structured effort to amplify the voices of MMIP survivors and their families.</t>
+          <t>The legislation emphasizes partnership with Tribal communities, indicating a recognition of the importance of their input in addressing the crisis of Missing or Murdered Indigenous Persons (MMIP). Statements from officials suggest a commitment to working alongside Indigenous politicians and communities to enhance public safety and justice for victims. However, while the involvement of Indigenous communities is acknowledged, the specific level and nature of direct input from MMIP survivors and their relatives is not detailed, leading to a conclusion of "somewhat."</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Deputy Attorney General Lisa Monaco - Department of Justice, Secretary of the Interior Deb Haaland (Laguna Pueblo) - 54th United States Secretary of the Interior, 2021–2025, Cole Finegan - U.S. Attorney (District of Colorado), Vanita Gupta - Associate Attorney General</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>Secretary of the Interior Deb Haaland (Laguna Pueblo) - 54th United States Secretary of the Interior, 2021–2025</t>
-        </is>
-      </c>
+          <t>Alexander M.M. Uballez - U.S. Attorney (District of New Mexico), Merrick B. Garland - Attorney General, Lisa O. Monaco - Deputy Attorney General, Heidi Todacheene - Senior Advisor to the Secretary, Elizabeth Hidalgo Reese - White House Senior Policy Advisor for Native Affairs</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr">
         <is>
+          <t>Biden Administration, 2020-2024</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>US Law Enforcement, Tribal Law Enforcement, Data Collection</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>2023-06-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>U.S. Attorney's Office Joins in Recognizing Missing and Murdered Indigenous Persons Awareness Day and Announces Appointment of Regional MMIP Coordinator</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>DOJ24-570</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Department of Justice</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>May 3, 2024 - Immediate release, U.S. Attorney's Office, District of Oregon</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>https://www.justice.gov/usao-or/pr/us-attorneys-office-joins-recognizing-missing-and-murdered-indigenous-persons-1</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>The U.S. Attorney's Office for the District of Oregon is recognizing May 5, 2024, as National Missing and Murdered Indigenous Persons (MMIP) Awareness Day and announced the appointment of Cedar Wilkie Gillette as the regional MMIP Coordinator for the Northwest Region. This initiative is part of the Justice Department's MMIP Regional Outreach Program, which aims to enhance collaboration among federal, tribal, and local law enforcement to address cases of missing and murdered indigenous individuals. The program, launched in July 2023, is focused on improving public safety in Indian Country and providing resources to tackle unresolved MMIP cases. The effort is reinforced by the commitment to prioritize resources as outlined in Executive Order 14053. The initiative also includes the establishment of an MMIP Working Group in Oregon, comprised of representatives from nine federally recognized tribes and various law enforcement agencies.</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Establishes a National Missing and Murdered Indigenous Persons (MMIP) Awareness Day to raise awareness of the issue.  
+2. Appoints a dedicated regional MMIP Coordinator to enhance the focus on addressing MMIP cases in the Northwest Region.  
+3. Enhances collaboration among federal, tribal, and local law enforcement agencies to tackle unresolved MMIP cases.  
+4. Launches the MMIP Regional Outreach Program, prioritizing public safety and resources for Indian Country.  
+5. Creates an MMIP Working Group that includes representatives from nine federally recognized tribes, promoting Indigenous community involvement.  
+6. Provides significant funding ($268 million) to improve Tribal justice systems and strengthen law enforcement responses.  
+7. Utilizes gender-inclusive language to address the crisis affecting individuals of all genders within Indigenous communities.  
+8. Implements mechanisms for evaluation, such as consultation with communities, monitoring, and data collection to assess the effectiveness of efforts.  </t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. The legislation does not explicitly detail input from MMIP survivors or their relatives, which may limit the incorporation of direct experiences in addressing the crisis.  
+2. While it establishes a working group, it does not specify mechanisms for ongoing consultation or engagement with Indigenous communities beyond initial representation.  
+3. The focus on police and law enforcement may raise concerns about prioritizing punitive measures over community-led healing and prevention strategies.  
+4. There is no mention of specific actions or timelines for assessing the effectiveness of the programs and initiatives outlined.  
+5. Certain Indigenous voices may still feel marginalized if the initiative does not adequately reflect the diverse perspectives within the tribes represented.  </t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>1. Consultation with community
+2. Tribal consultation
+3. Monitoring
+4. Data collection</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>The legislation uses gender inclusive language by referring to "Missing and Murdered Indigenous Persons" (MMIP) rather than exclusively focusing on women, thereby acknowledging that individuals of all genders can be affected by this crisis. By encompassing the broader term "persons," it reflects a more comprehensive understanding of the issue, rather than limiting it to a specific demographic. This approach promotes inclusivity and recognizes the experiences of all Indigenous individuals affected by violence and injustice.</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>1. "The office also announced today the appointment of an MMIP Regional Coordinator based in the District of Oregon."
+2. "This program is a critical next step in the department’s ongoing effort to address this crisis, which has affected tribes and communities across our region and country."
+3. "This support includes assisting in the investigation of unresolved MMIP cases and related crimes, and promoting communication, coordination, and collaboration among federal, tribal, local, and state law enforcement and non-governmental partners on MMIP issues."
+4. "The regional outreach program program prioritizes MMIP cases consistent with the Deputy Attorney General’s July 2022 directive to U.S. Attorney’s Offices promoting public safety in Indian Country." 
+5. "Over the past year, the Department awarded $268 million in grants to help enhance Tribal justice systems and strengthen law enforcement responses."</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Somewhat</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>The legislation indicates the establishment of an MMIP Working Group that includes representatives from each of the nine federally recognized tribes in Oregon, suggesting some level of inclusion of Indigenous communities in addressing the MMIP crisis. Furthermore, the appointment of Cedar Wilkie Gillette, who has direct ties to Indigenous nations, as the MMIP Coordinator signifies a recognition of Indigenous voices in the initiative. However, the specific input from MMIP survivors or their relatives is not explicitly detailed in the text, leading to a conclusion of "Somewhat" rather than "Yes."</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Cedar Wilkie Gillette (Mandan (Mandan, Hidatsa, Arikara Nation, Turtle Mountain Band of Chippewa) - MMIP Coordinator (Northwest Region), MMIP Coordinator (District of Oregon), Hidatsa, Arikara Nation) - MMIP Regional Coordinator, Natalie Wight - U.S. Attorney (District of Oregon), Merrick B. Garland - Attorney General</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>Cedar Wilkie Gillette (Mandan (Mandan, Hidatsa, Arikara Nation, Turtle Mountain Band of Chippewa) - MMIP Coordinator (Northwest Region), MMIP Coordinator (District of Oregon)</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
           <t>Biden Administration, 2020 - 2024</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
+      <c r="AA4" t="inlineStr">
         <is>
           <t>Taskforce, Day of Recognition, US Law Enforcement, Tribal Law Enforcement, Data Collection</t>
         </is>
       </c>
-      <c r="AB3" t="inlineStr">
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>2024-05-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>NM</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>U.S. Attorney Alexander M.M. Uballez Announces Selection of Missing or Murdered Indigenous Persons Assistant United States Attorney for the Southwest Region</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DOJ23-236</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Department of Justice</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>September 27, 2023 - Immediate release, U.S. Attorney's Office, District of New Mexico</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://www.justice.gov/usao-nm/pr/us-attorney-alexander-mm-uballez-announces-selection-missing-or-murdered-indigenous</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>U.S. Attorney Alexander M.M. Uballez announced the selection of Eliot Neal as the Missing or Murdered Indigenous Persons (MMIP) Assistant United States Attorney for the Southwest Region, which includes New Mexico, Colorado, Utah, Nevada, and Arizona. Neal will provide specialized support to address the crisis of missing or murdered Indigenous persons, focusing on unresolved cases and fostering collaboration among various law enforcement and community partners. He was previously the District’s Tribal Liaison to the Mescalero Apache Tribe, showcasing his commitment to building strong relationships with tribal communities. Through this initiative, Neal aims to promote justice and support for impacted families. The announcement highlights the Department of Justice's ongoing efforts to tackle issues affecting Indigenous populations.</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. The legislation aids in the selection of a dedicated Assistant United States Attorney focused on the crisis of missing or murdered Indigenous persons, promoting specialized support for affected communities.  
+2. It fosters collaboration among various law enforcement agencies and community partners, enhancing communication and resource sharing to address unresolved cases.  
+3. The use of gender-inclusive language demonstrates a commitment to recognizing and addressing the diverse impacts of violence on all genders within Indigenous populations.  
+4. Eliot Neal's previous experience as a Tribal Liaison to the Mescalero Apache Tribe strengthens relationships between federal law enforcement and tribal communities, potentially improving outreach and support.  
+5. The initiative highlights the Department of Justice's ongoing efforts to address serious issues affecting Indigenous populations, reinforcing its commitment to justice and advocacy for these communities.  </t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. The legislation lacks explicit mechanisms for evaluation or monitoring, which may hinder accountability and assessment of its effectiveness in addressing the MMIP crisis.  
+2. There are no identified prevention efforts included in the initiative, potentially limiting proactive measures to avoid future cases of missing or murdered Indigenous persons.  
+3. The absence of input from MMIP survivors, relatives, and Indigenous communities may undermine the initiative's relevance and effectiveness, as it does not center the voices most affected by the crisis.  
+4. The legislation does not specifically mention Indigenous organizations that support MMIP survivors, which could limit collaborative efforts and resources available for affected families.  
+5. While it addresses a critical issue, the focus on law enforcement could overshadow the need for comprehensive community-based approaches to support and empower Indigenous populations.  </t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>1. None</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>The legislation refers to the "Missing or Murdered Indigenous Persons (MMIP)" rather than specifically mentioning women, thereby encompassing all genders affected by this crisis. This inclusive terminology acknowledges that individuals of various genders can be victims of violence and disappearance in Indigenous communities. The use of "persons" instead of "women" demonstrates an effort to adopt gender-neutral language.</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>The legislation does not explicitly mention any input from MMIP survivors, relatives, Indigenous politicians, or Indigenous communities regarding the initiative. It primarily focuses on the announcement of the selection of Eliot Neal as the Assistant United States Attorney for Missing or Murdered Indigenous Persons, without detailing any collaborative processes or consultations. Therefore, the level and nature of input from these stakeholders are not addressed in the text.</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>Eliot Neal (Mescalero Apache Tribe) - Assistant United States Attorney, Alexander M.M. Uballez - U.S. Attorney, Department of Justice</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>Biden Administration, 2020-2024</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>US Law Enforcement, Tribal Law Enforcement, Data Collection</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>2023-09-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>National</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Justice Department Strengthens Efforts to Address the Crisis of Missing or Murdered Indigenous Persons</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>DOJ23-514</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Department of Justice</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>May 5, 2023 - For Immediate Release, U.S. Attorney's Office, District of Colorado</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>https://www.justice.gov/usao-co/pr/justice-department-strengthens-efforts-address-crisis-missing-or-murdered-indigenous</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>The Justice Department announced its strengthened efforts to address the crisis of Missing or Murdered Indigenous Persons (MMIP) on May 5, 2023, coinciding with National MMIP Awareness Day. This initiative includes collaboration between various federal agencies, including the Department of the Interior, to reduce violence against American Indian and Alaska Native communities. Key actions involve the Not Invisible Act Commission, which aims to develop comprehensive strategies and provide resources for support and prevention. The Department of Justice emphasizes its commitment to utilizing its resources to address this ongoing crisis, enhance public safety in Indian country, and support victims' families. Various programs and resources, including grants and guidance for tribal communities, have also been established to assist in this effort.</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Establishes a comprehensive framework to address the crisis of Missing or Murdered Indigenous Persons (MMIP) through collaboration among various federal agencies, enhancing public safety in Indian country.  
+2. Utilizes gender-inclusive language to acknowledge the experiences of all Indigenous individuals affected by violence, promoting inclusivity and broadening the scope of the initiative.  
+3. Incorporates mechanisms for evaluation and recommendations through the Not Invisible Act Commission and community engagement, ensuring that the voices of MMIP survivors and their families are heard.  
+4. Provides grant funding and resources to support Tribal communities in developing response plans, increasing awareness, and improving local law enforcement partnerships.  
+5. Expands efforts for data collection and analysis to better understand the prevalence of MMIP cases and inform future strategies.  </t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. While there is mention of collaboration with Tribal governments, the specifics on individual input from MMIP survivors and their families may not be detailed, potentially limiting the effectiveness of community engagement.  
+2. The broad language used to describe the initiative may lack focus on the unique challenges faced by specific subgroups within the Indigenous population, such as LGBTQ+ individuals, which could result in overlooked needs.  
+3. The effectiveness of the proposed measures and programs may be contingent on adequate funding and resources, with no guaranteed assurance that these will be consistently provided or managed.  
+4. The legislation outlines the establishment of a liaison but does not specify the timeline or mechanisms for ongoing evaluation of their effectiveness and the overall impact of the initiative on reducing violence against Indigenous persons.  </t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>1. "Later this year, the Commission will deliver recommendations for addressing the MMIP crisis to the Attorney General and the Secretary."
+2. "The Liaison will meet with survivors and family members of MMIP to learn more about the current challenges in MMIP cases and to make recommendations about the department’s continued response."
+3. "The Guide is a resource for Tribes interested in developing a plan to respond to missing person cases that is tailored to the specific needs, resources, and culture of Tribal communities."
+4. "The department’s National Institute of Justice (NIJ) funded a study that will provide vital information regarding the prevalence and context of cases of MMIP in New Mexico and, importantly, will inform long-term data collection, analysis, and reporting strategies on MMIP cases."</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>The legislation adopts gender-inclusive language by referring to the crisis as affecting "Missing or Murdered Indigenous Persons" rather than solely focusing on women. This broad terminology encompasses the experiences of all Indigenous individuals, including men and non-binary people, who may be victims of violence or going missing. By doing so, it acknowledges the wider scope of the issue and promotes inclusivity in addressing the crisis.</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>1. "Responding to the unacceptable levels of violence that have led to the crisis of Missing or Murdered Indigenous Persons (MMIP) is a priority of the Department of Justice every day."
+2. "Missing or Murdered Indigenous Persons Awareness Day calls on our nation to pause and honor the loved ones who have gone missing or who have been the victims of violent crime."
+3. "In addition to our core law-enforcement work, we are providing grant funding and guidance to help Tribes develop response plans for missing-persons cases, partner effectively with local law enforcement, and provide resources for victims of crime."
+4. "The department’s Office for Victims of Crime (OVC) expanded the scope of allowable activities under its Tribal Victim Services Set-Aside (TVSSA) grant program to permit Tribal communities to pay for costs related to generating awareness of individual missing persons cases involving American Indians and Alaska Native persons, supporting private search efforts for missing American Indians and Alaska Native persons in certain circumstances, and supporting efforts to coordinate the Tribal, state, and federal response to MMIP cases."</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>The legislation emphasizes the establishment of a National Native American Outreach Services Liaison, which is tasked with amplifying the voices of crime victims in Indian country, including survivors and their families of MMIP cases. Additionally, it notes that the Liaison will meet with survivors and family members to better understand their challenges and make recommendations for the department's continued response. This demonstrates a commitment to engaging with MMIP survivors and their relatives directly, indicating meaningful input from these communities in shaping the response to the crisis</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>Somewhat</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>The legislation emphasizes collaboration with Tribal governments and communities, indicating a partnership approach in addressing the MMIP crisis. Secretary Deb Haaland's involvement showcases representation from Indigenous leadership, highlighting the importance of community input in formulating responses to this issue. Additionally, the mention of developing a Tribal Community Response Plan suggests a framework for incorporating the voices of MMIP survivors and their families, though specifics on individual input may not be detailed in the text.</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>Deputy Attorney General Lisa Monaco - Department of Justice, Secretary Deb Haaland (Laguna Pueblo) - 54th United States Secretary of the Interior, 2021–2025, Cole Finegan - U.S. Attorney for the District of Colorado, Attorney General Merrick B. Garland - Department of Justice, Associate Attorney General Vanita Gupta - Department of Justice, Ute Mountain Ute Tribe - Tribal Government Partner, Southern Ute Tribe - Tribal Government Partner.</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>Secretary Deb Haaland (Laguna Pueblo) - 54th United States Secretary of the Interior, 2021–2025</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>Biden Administration, 2020 - 2024</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>Taskforce, Day of Recognition, US Law Enforcement, Tribal Law Enforcement, Data Collection, MMIP Relatives</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>2023-05-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AK</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Missing or Murdered Indigenous Persons</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Department of Justice</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>February 26, 2025 - Immediate release string, U.S. Attorney's Office</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://www.justice.gov/usao-ak/missing-or-murdered-indigenous-persons</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>The initiative addresses the ongoing violence faced by Native American families and communities, emphasizing the importance of tackling issues related to missing or murdered indigenous persons. The Department of Justice is committed to working alongside Tribal nations to prioritize this matter within its law enforcement efforts. The program includes guidelines for developing response plans for missing person cases, specifically in Alaska, under Savanna's Act. The U.S. Attorney's Office for the District of Alaska is a key entity involved in this initiative, spearheaded by coordinator E. Ingrid Goodyear. Updates and resources on the matter have been made available as of February 26, 2025.</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. The initiative addresses and prioritizes the ongoing violence against Native American families and communities related to missing or murdered indigenous persons.  
+2. It promotes collaboration with Tribal nations, ensuring that Indigenous perspectives are considered in law enforcement efforts.  
+3. The legislation includes guidelines for developing response plans for missing persons, specifically tailored to the context of Alaska.  
+4. It aims to improve the federal response to MMIP cases through ongoing work pursuant to Savanna’s Act.  
+5. The focus on all genders in the language used promotes inclusivity and recognizes the experiences of diverse Indigenous individuals.  </t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. The legislation does not provide specific details on direct input from MMIP survivors or their relatives, which may limit the initiative's responsiveness to their needs.  
+2. While it emphasizes collaboration with Tribal nations, the level of Indigenous input is categorized as "Somewhat," suggesting that more robust engagement could be achieved.  
+3. The legislation may lack comprehensive measures for follow-up and evaluation, potentially hindering its effectiveness in addressing the issues at hand.  
+4. There is no mention of specific Indigenous organizations that could provide additional support for MMIP survivors, which may limit the initiative's community connection.  
+5. The focus on broader categories without addressing specific local contexts for different Indigenous communities may overlook unique challenges faced by those groups.  </t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>1. Guide to Developing an Alaska Tribal Community Response Plan for Missing Person Cases  
+2. Consultation with Tribal nations  
+3. federal response to missing or murdered indigenous persons (MMIP)  
+4. Ongoing work pursuant to Savanna’s Act</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>The legislation addresses the broader issue of missing and murdered indigenous persons rather than focusing solely on women, indicating a recognition of the experiences of all genders within Indigenous communities. By utilizing terms like "Native American families and communities" and specifying "missing or murdered indigenous persons," it adopts a more inclusive language approach. This framing highlights the initiative's commitment to addressing violence against all Indigenous individuals, regardless of gender.</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. "The Department of Justice is committed to addressing the persistent violence endured by Native American families and communities across the country, including by working with Tribal nations to address the important issues of missing or murdered indigenous persons."  
+2. "The Department views this work as a priority for its law enforcement components."  
+3. "The Department is committed to its ongoing work pursuant to Savanna’s Act to improve the federal response to missing or murdered indigenous persons (MMIP)."  </t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>Somewhat</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>The legislation emphasizes collaboration with Tribal nations and acknowledges the importance of addressing issues faced by Indigenous communities, indicating some level of input from these stakeholders. The role of E. Ingrid Goodyear as the MMIP Coordinator suggests that Indigenous perspectives are being represented in the initiative. However, the text does not provide specific details on direct input from MMIP survivors or their relatives, leading to a determination of "Somewhat" in terms of overall input.</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>E. Ingrid Goodyear (Aleut, Tlingit) - MMIP Coordinator (Districts of Alaska &amp; Great Plains) (District of Alaska)</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>E. Ingrid Goodyear (Aleut, Tlingit) - MMIP Coordinator (Districts of Alaska &amp; Great Plains) (District of Alaska)</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>Biden Administration, 2020 - 2024</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>Taskforce, US Law Enforcement, Tribal Law Enforcement, Data Collection</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>2025-02-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>National</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Justice Department Strengthens Efforts to Address the Crisis of Missing or Murdered Indigenous Persons</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>DOJ23-1458</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Department of Justice</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>May 5, 2023 - Immediate release, U.S. Attorney's Office, District of Nevada</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>https://www.justice.gov/usao-nv/pr/justice-department-strengthens-efforts-address-crisis-missing-or-murdered-indigenous</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>The Justice Department has intensified its efforts to address the crisis of Missing or Murdered Indigenous Persons (MMIP), recognizing May 5, 2023, as National Missing or Murdered Indigenous Persons Awareness Day. The initiative aims to combat the violence affecting American Indian and Alaska Native communities through a coordinated approach involving federal partnerships and resources. Key actions include the establishment of the Not Invisible Act Commission to reduce violence against Indigenous peoples and the commitment to providing guidance and funding to Tribes for developing response plans for missing persons cases. The Department emphasizes collaboration with Tribal governments and law enforcement agencies to enhance public safety and support victims. This comprehensive effort seeks to address the disproportionately high rates of violence and missing persons among Indigenous populations in the U.S.</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Increases awareness of the crisis of Missing or Murdered Indigenous Persons (MMIP) through the recognition of National Missing or Murdered Indigenous Persons Awareness Day.  
+2. Establishes the Not Invisible Act Commission to reduce violence against Indigenous peoples, fostering collaboration among various stakeholders.  
+3. Provides guidance and funding to Tribes for developing response plans to address missing persons cases effectively.  
+4. Enhances public safety by promoting partnerships between the Department of Justice, Tribal governments, and law enforcement agencies.  
+5. Expands data collection and monitoring efforts to better understand the prevalence and context of MMIP cases.  
+6. Incorporates input from survivors and their families, giving them a voice in addressing the crisis.  
+7. Supports awareness initiatives through funding for Tribal communities to enhance their capacity to respond to missing persons cases.  
+8. Aims to address the disproportionately high rates of violence against Indigenous populations in the U.S. through coordinated federal efforts.  </t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>1. While the legislation refers to the involvement of Indigenous leaders, it lacks detailed specifics on how input from MMIP survivors and their families is integrated into decision-making processes.  
+2. The effectiveness of the initiatives and partnerships may depend on adequate funding and sustained political will, which may vary over time.  
+3. There may be challenges in coordinating efforts across different federal and Tribal agencies, potentially leading to inconsistencies in implementation.  
+4. The reliance on existing structures for data collection might limit the ability to capture the full scope of the MMIP crisis effectively.  
+5. Recognition of National Missing or Murdered Indigenous Persons Awareness Day, while symbolic, may not translate into concrete action without follow-up measures and accountability.  
+6. The focus on grant funding may inadvertently create competition among Tribes for limited resources instead of fostering collaboration.</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>1. "The Commission will deliver recommendations for addressing the MMIP crisis to the Attorney General and the Secretary."
+2. "published its Tribal Memorandum of Understanding (MOU)/Memorandum of Agreement (MOA) Sample Resource Library."
+3. "the department’s National Institute of Justice (NIJ) funded a study that will provide vital information regarding the prevalence and context of cases of MMIP in New Mexico and, importantly, will inform long-term data collection, analysis, and reporting strategies on MMIP cases."</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>The legislation uses gender inclusive language by referring to the crisis as the "Missing or Murdered Indigenous Persons (MMIP)" rather than focusing solely on women. This choice broadens the scope to acknowledge the experiences of all Indigenous individuals affected by violence and disappearance. Additionally, the emphasis on partnerships with Tribal governments indicates a commitment to addressing the needs of diverse community members.</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>1. "The Justice Department joins its partners across the federal government, as well as people throughout American Indian and Alaska Native communities, in recognizing May 5, 2023 as National Missing or Murdered Indigenous Persons Awareness Day."
+2. "The department is providing grant funding and guidance to help Tribes develop response plans for missing-persons cases, partner effectively with local law enforcement, and provide resources for victims of crime."
+3. "The department’s Office for Victims of Crime (OVC) expanded the scope of allowable activities under its Tribal Victim Services Set-Aside (TVSSA) grant program to permit Tribal communities to pay for costs related to generating awareness of individual missing persons cases involving American Indians and Alaska Native persons."</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>The legislation establishes the Not Invisible Act Commission, which is dedicated to addressing violence against American Indians and Alaska Natives and involves various stakeholders, including Indigenous leaders and community members. It also highlights the creation of a National Native American Outreach Services Liaison, whose role is to amplify the voices of crime victims in Indian country and their families as they navigate the federal criminal justice system. These initiatives suggest a commitment to incorporating input from MMIP survivors and their relatives; thus, this indicates that their perspectives and needs are acknowledged within the legislation</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Somewhat</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>The legislation mentions the establishment of the Not Invisible Act Commission, which involves various stakeholders, including Indigenous leaders, to address violence against American Indian and Alaska Native communities. It also emphasizes the ongoing participation of the Department of Justice in consultations with community members and Tribal governments, indicating a degree of input from survivors and their families. However, while there is recognition of these groups, the specifics of survivor input are not detailed, leading to the conclusion of "Somewhat" regarding the overall level of inclusion.</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>Deputy Attorney General Lisa O. Monaco - Department of Justice, Secretary Deb Haaland (Laguna Pueblo) - 54th United States Secretary of the Interior, 2021–2025, Attorney General Merrick B. Garland - Department of Justice, United States Attorney Jason M. Frierson - District of Nevada, Associate Attorney General Vanita Gupta - Department of Justice.</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>Secretary Deb Haaland (Laguna Pueblo) - 54th United States Secretary of the Interior, 2021–2025</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>Biden Administration, 2020-2024</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>Taskforce, Day of Recognition, US Law Enforcement, Tribal Law Enforcement, Data Collection, MMIP Relatives</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>2023-05-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>National</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Justice Department Strengthens Efforts to Address the Crisis of Missing or Murdered Indigenous Persons</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DOJ24-570</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Department of Justice, Department of the Interior</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>May 5, 2023 - For Immediate Release, U.S. Attorney's Office, Eastern District of Oklahoma</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://www.justice.gov/usao-edok/pr/justice-department-strengthens-efforts-address-crisis-missing-or-murdered-indigenous</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>The Justice Department has announced enhanced efforts to address the crisis of Missing or Murdered Indigenous Persons (MMIP), recognizing May 5, 2023, as National MMIP Awareness Day. This initiative is supported by multiple stakeholders, including the Not Invisible Act Commission led by Deputy Attorney General Lisa Monaco and Secretary of the Interior Deb Haaland, aimed at reducing violence against American Indians and Alaska Natives. The department emphasizes a whole-of-government approach, collaborating with Tribal and law enforcement agencies to mitigate violence and support victims. A series of measures, such as updated guidelines for victim assistance and the establishment of new liaison positions, are being implemented to improve responses to MMIP cases. The initiative also highlights the importance of cultural competence and community engagement in addressing the crisis effectively.</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Enhanced efforts to address the crisis of Missing or Murdered Indigenous Persons (MMIP) through initiatives like National MMIP Awareness Day, increasing public recognition and engagement on the issue.  
+2. Inclusion of a diverse range of stakeholders, such as the Not Invisible Act Commission and tribal governments, promoting a collaborative approach to violence reduction and victim support.  
+3. Utilization of gender-inclusive language and recognition of all genders affected by violence, ensuring that the initiative addresses the needs of the entire Indigenous community.  
+4. Implementation of mechanisms for evaluation and response, including guidelines for victim assistance and a Tribal Community Response Plan, which will provide structured support for affected communities.  
+5. Establishment of roles such as the National Native American Outreach Services Liaison, aimed at amplifying the voices of MMIP survivors and their families, ensuring their perspectives are considered in decision-making processes.  
+6. Commitment to data collection and analysis on the prevalence of MMIP cases, leading to informed strategies and improved public safety initiatives in Indian Country.  </t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. While there is recognition of the crisis, the effectiveness of implementation and actual results in reducing violence against Missing or Murdered Indigenous Persons (MMIP) remains to be seen and may be slow to materialize.  
+2. The focus on developing guidelines and resources may lead to bureaucratic delays, potentially hindering immediate action needed to support victims and prevent future incidents.  
+3. Involvement of multiple stakeholders may complicate collaboration and coordination efforts, leading to fragmented responses rather than a unified approach to addressing the MMIP crisis.  
+4. While there are efforts to amplify Indigenous voices, the extent and effectiveness of community engagement and input in decision-making processes are not fully guaranteed or defined.  
+5. The legislation's reliance on grant funding may create uncertainty in resource availability for ongoing support and initiatives aimed at addressing MMIP cases.  </t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>1. "Later this year, the Commission will deliver recommendations for addressing the MMIP crisis to the Attorney General and the Secretary."
+2. "the department published a Guide to Developing a Tribal Community Response Plan for Missing Persons Cases."
+3. "the department’s National Institute of Justice (NIJ) funded a study that will provide vital information regarding the prevalence and context of cases of MMIP in New Mexico and, importantly, will inform long-term data collection, analysis, and reporting strategies on MMIP cases."</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>The legislation addresses the crisis as "Missing or Murdered Indigenous Persons" (MMIP), which explicitly includes individuals of all genders rather than focusing solely on women. This terminology reflects an understanding of the broader impact of violence affecting Indigenous communities, recognizing that both men and women can be victims of such crimes. Additionally, the use of gender-neutral language throughout demonstrates an effort to be inclusive and comprehensive in addressing the needs of all Indigenous individuals.</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>1. "Responding to the unacceptable levels of violence that have led to the crisis of Missing or Murdered Indigenous Persons (MMIP) is a priority of the Department of Justice every day."
+2. "The department is committed to using every resource at its disposal to combat the Missing or Murdered Indigenous Persons Crisis."
+3. "In addition to our core law-enforcement work, we are providing grant funding and guidance to help Tribes develop response plans for missing-persons cases, partner effectively with local law enforcement, and provide resources for victims of crime."
+4. "These sessions reinforced the need for federal, state, local and tribal law enforcement agencies to work cooperatively to confront violent crime within Indian Country."</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>The legislation includes the establishment of the Not Invisible Act Commission, which is specifically designed to involve community members, including MMIP survivors and their families, in addressing the crisis surrounding missing and murdered Indigenous persons. Additionally, it mentions the role of a National Native American Outreach Services Liaison, whose purpose is to amplify the voices of crime victims in Indian country, indicating a structured approach to incorporating feedback from affected individuals. Furthermore, the legislation's commitment to funding and guiding Tribal communities in developing response plans highlights an active effort to consider the perspectives and needs of MMIP survivors and their relatives</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Somewhat</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>The legislation highlights the involvement of Indigenous communities through the Not Invisible Act Commission, which was launched to address violence against American Indians and Alaska Natives, indicating a focus on community input. Additionally, the statement by Deputy Attorney General Lisa O. Monaco emphasizes the importance of working as partners with Tribal governments, suggesting a collaborative approach that includes Indigenous voices. The presence of Secretary Deb Haaland, an Indigenous politician, further underscores the commitment to representation and engagement of Indigenous communities in the process.</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>Deputy Attorney General Lisa Monaco - Department of Justice, Secretary Deb Haaland (Laguna Pueblo) - 54th United States Secretary of the Interior, 2021–2025, Attorney General Merrick B. Garland - Department of Justice, Associate Attorney General Vanita Gupta - Department of Justice, United States Attorney Christopher J. Wilson - Eastern District of Oklahoma</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>Secretary Deb Haaland (Laguna Pueblo) - 54th United States Secretary of the Interior, 2021–2025</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>Biden Administration, 2020 - 2024</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>Taskforce, Day of Recognition, US Law Enforcement, Tribal Law Enforcement, Data Collection, MMIP Relatives</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
         <is>
           <t>2023-05-05</t>
         </is>

</xml_diff>